<commit_message>
Graphics done, they really look this way and I don't understand why
</commit_message>
<xml_diff>
--- a/DecompositionLU/docs/statistics.xlsx
+++ b/DecompositionLU/docs/statistics.xlsx
@@ -8,24 +8,31 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Maxim\source\repos\practice\SECOND_COURSE\FOR_ITLAB\ArchBenchs\DecompositionLU\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41A68739-CF7C-43FF-A221-C9063AB72525}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BF38F48-B947-4425-AE12-16D6FDB9CE80}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-114" yWindow="-114" windowWidth="27602" windowHeight="15027" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Лист1" sheetId="1" r:id="rId1"/>
+    <sheet name="Таблица" sheetId="1" r:id="rId1"/>
+    <sheet name="Графики" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="82">
   <si>
     <t>Я не уверен, будет ли это использоваться в готовой презентации и так ли это надо делать, если да, так что пока считаем, что файл для личного пользования.</t>
   </si>
@@ -251,9 +258,6 @@
     <t>~1162</t>
   </si>
   <si>
-    <t>чет очень скромное ускорение</t>
-  </si>
-  <si>
     <t>~673</t>
   </si>
   <si>
@@ -327,13 +331,28 @@
   </si>
   <si>
     <t>~82</t>
+  </si>
+  <si>
+    <t>Кол-во потоков</t>
+  </si>
+  <si>
+    <t>Время вычисления</t>
+  </si>
+  <si>
+    <t>n = 5000</t>
+  </si>
+  <si>
+    <t>n = 3000</t>
+  </si>
+  <si>
+    <t>Я искренне не понимаю этих результатов</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -398,6 +417,43 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="GOST Common"/>
+      <family val="2"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <name val="GOST Common"/>
+      <family val="2"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="14"/>
+      <color rgb="FF0070C0"/>
+      <name val="GOST Common"/>
+      <family val="2"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="14"/>
+      <name val="GOST Common"/>
+      <family val="2"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="GOST Common"/>
+      <family val="2"/>
+      <charset val="204"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -419,7 +475,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -488,11 +544,48 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
@@ -520,6 +613,16 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -528,9 +631,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -541,8 +641,60 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -559,6 +711,1704 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="ru-RU"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="104"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="4"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="GOST Common" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>n = 5000</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="GOST Common" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="ru-RU"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Графики!$C$4:$C$19</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="16"/>
+                <c:pt idx="0">
+                  <c:v>40525</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>40933</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>35748</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>34657</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>36335</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>38071</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>36151</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>37594</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>36727</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>36931</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>38323</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>40896</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>38132</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>38962</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>38825</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>39364</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-DFDA-4FBA-8E35-21ED64A1AC56}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:marker val="1"/>
+        <c:smooth val="0"/>
+        <c:axId val="2034815519"/>
+        <c:axId val="1972086687"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="2034815519"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="GOST Common" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="ru-RU"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1972086687"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1972086687"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:min val="34000"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="GOST Common" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="ru-RU"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="2034815519"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr>
+          <a:latin typeface="GOST Common" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+        </a:defRPr>
+      </a:pPr>
+      <a:endParaRPr lang="ru-RU"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="ru-RU"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="108"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="8"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="GOST Common" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>n = 3000</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="GOST Common" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="ru-RU"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent6"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent6"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent6"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Графики!$D$4:$D$19</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="16"/>
+                <c:pt idx="0">
+                  <c:v>8737</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>8116</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>8005</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>7387</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>6863</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>7472</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>6861</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>7389</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>7908</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>8155</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>7985</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>8411</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>8314</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>8287</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>8452</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>7844</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-8747-4A5E-85F4-772AAE4EC689}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:marker val="1"/>
+        <c:smooth val="0"/>
+        <c:axId val="52875439"/>
+        <c:axId val="1972084607"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="52875439"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="GOST Common" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="ru-RU"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1972084607"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1972084607"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:min val="6500"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="GOST Common" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="ru-RU"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="52875439"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr>
+          <a:latin typeface="GOST Common" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+        </a:defRPr>
+      </a:pPr>
+      <a:endParaRPr lang="ru-RU"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="withinLinear" id="15">
+  <a:schemeClr val="accent2"/>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="withinLinear" id="19">
+  <a:schemeClr val="accent6"/>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="332">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="332">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -728,6 +2578,83 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>9052</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>13579</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>525100</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>40739</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="5" name="Диаграмма 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D9C1BB01-F75F-4D40-BA20-D7288523072B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>9052</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>13579</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>525100</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>176542</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="7" name="Диаграмма 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{63E3D050-E508-4926-853F-B56EA689B234}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -994,15 +2921,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:T42"/>
+  <dimension ref="A1:W42"/>
   <sheetFormatPr defaultRowHeight="17.850000000000001" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="71.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="65.7109375" style="1" customWidth="1"/>
     <col min="2" max="5" width="26.7109375" style="1" customWidth="1"/>
-    <col min="6" max="16384" width="9.140625" style="1"/>
+    <col min="6" max="6" width="9.140625" style="1"/>
+    <col min="7" max="7" width="23.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="24.85546875" style="1" customWidth="1"/>
+    <col min="10" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>1</v>
       </c>
@@ -1026,7 +2956,7 @@
       <c r="S1" s="2"/>
       <c r="T1" s="2"/>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -1050,7 +2980,7 @@
       <c r="S2" s="2"/>
       <c r="T2" s="2"/>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>2</v>
       </c>
@@ -1068,39 +2998,43 @@
       <c r="M3" s="6"/>
       <c r="N3" s="6"/>
     </row>
-    <row r="5" spans="1:20" ht="17.850000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="13" t="s">
+    <row r="5" spans="1:23" ht="17.850000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="13"/>
-      <c r="C5" s="13"/>
-      <c r="D5" s="13"/>
-      <c r="E5" s="13"/>
-      <c r="G5" s="16" t="s">
+      <c r="B5" s="38"/>
+      <c r="C5" s="38"/>
+      <c r="D5" s="38"/>
+      <c r="E5" s="39"/>
+      <c r="G5" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="H5" s="16"/>
-      <c r="I5" s="16"/>
-      <c r="J5" s="16"/>
-      <c r="K5" s="16"/>
-    </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="H5" s="15"/>
+      <c r="S5" s="5"/>
+      <c r="T5" s="14"/>
+      <c r="U5" s="14"/>
+      <c r="V5" s="14"/>
+      <c r="W5" s="14"/>
+    </row>
+    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="14" t="s">
+      <c r="B6" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="14"/>
-      <c r="D6" s="14"/>
-      <c r="E6" s="14"/>
-      <c r="G6" s="16"/>
-      <c r="H6" s="16"/>
-      <c r="I6" s="16"/>
-      <c r="J6" s="16"/>
-      <c r="K6" s="16"/>
-    </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="C6" s="18"/>
+      <c r="D6" s="18"/>
+      <c r="E6" s="18"/>
+      <c r="G6" s="15"/>
+      <c r="H6" s="15"/>
+      <c r="S6" s="14"/>
+      <c r="T6" s="14"/>
+      <c r="U6" s="14"/>
+      <c r="V6" s="14"/>
+      <c r="W6" s="14"/>
+    </row>
+    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>6</v>
       </c>
@@ -1116,27 +3050,31 @@
       <c r="E7" s="8">
         <v>10000</v>
       </c>
-      <c r="G7" s="16"/>
-      <c r="H7" s="16"/>
-      <c r="I7" s="16"/>
-      <c r="J7" s="16"/>
-      <c r="K7" s="16"/>
-    </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A8" s="15" t="s">
+      <c r="G7" s="15"/>
+      <c r="H7" s="15"/>
+      <c r="S7" s="14"/>
+      <c r="T7" s="14"/>
+      <c r="U7" s="14"/>
+      <c r="V7" s="14"/>
+      <c r="W7" s="14"/>
+    </row>
+    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A8" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="15"/>
-      <c r="C8" s="15"/>
-      <c r="D8" s="15"/>
-      <c r="E8" s="15"/>
-      <c r="G8" s="16"/>
-      <c r="H8" s="16"/>
-      <c r="I8" s="16"/>
-      <c r="J8" s="16"/>
-      <c r="K8" s="16"/>
-    </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="B8" s="19"/>
+      <c r="C8" s="19"/>
+      <c r="D8" s="19"/>
+      <c r="E8" s="19"/>
+      <c r="G8" s="15"/>
+      <c r="H8" s="15"/>
+      <c r="S8" s="14"/>
+      <c r="T8" s="14"/>
+      <c r="U8" s="14"/>
+      <c r="V8" s="14"/>
+      <c r="W8" s="14"/>
+    </row>
+    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>7</v>
       </c>
@@ -1152,13 +3090,13 @@
       <c r="E9" s="10">
         <v>1746</v>
       </c>
-      <c r="G9" s="16"/>
-      <c r="H9" s="16"/>
-      <c r="I9" s="16"/>
-      <c r="J9" s="16"/>
-      <c r="K9" s="16"/>
-    </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="S9" s="14"/>
+      <c r="T9" s="14"/>
+      <c r="U9" s="14"/>
+      <c r="V9" s="14"/>
+      <c r="W9" s="14"/>
+    </row>
+    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>8</v>
       </c>
@@ -1174,8 +3112,13 @@
       <c r="E10" s="10" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="S10" s="5"/>
+      <c r="T10" s="5"/>
+      <c r="U10" s="5"/>
+      <c r="V10" s="5"/>
+      <c r="W10" s="5"/>
+    </row>
+    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>9</v>
       </c>
@@ -1193,19 +3136,23 @@
       </c>
       <c r="F11" s="5"/>
       <c r="G11" s="5"/>
-    </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A12" s="15" t="s">
+      <c r="S11" s="5"/>
+      <c r="T11" s="5"/>
+      <c r="U11" s="5"/>
+      <c r="V11" s="5"/>
+      <c r="W11" s="5"/>
+    </row>
+    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A12" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="B12" s="15"/>
-      <c r="C12" s="15"/>
-      <c r="D12" s="15"/>
-      <c r="E12" s="15"/>
+      <c r="B12" s="19"/>
+      <c r="C12" s="19"/>
+      <c r="D12" s="19"/>
+      <c r="E12" s="19"/>
       <c r="F12" s="5"/>
-      <c r="G12" s="5"/>
-    </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
+    </row>
+    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>7</v>
       </c>
@@ -1215,16 +3162,15 @@
       <c r="C13" s="10">
         <v>232</v>
       </c>
-      <c r="D13" s="17" t="s">
+      <c r="D13" s="20" t="s">
         <v>21</v>
       </c>
       <c r="E13" s="10">
         <v>1811</v>
       </c>
       <c r="F13" s="5"/>
-      <c r="G13" s="5"/>
-    </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
+    </row>
+    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>8</v>
       </c>
@@ -1234,7 +3180,7 @@
       <c r="C14" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="D14" s="18"/>
+      <c r="D14" s="21"/>
       <c r="E14" s="10" t="s">
         <v>10</v>
       </c>
@@ -1242,7 +3188,7 @@
       <c r="G14" s="5"/>
       <c r="H14" s="5"/>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>9</v>
       </c>
@@ -1252,32 +3198,32 @@
       <c r="C15" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="D15" s="19"/>
+      <c r="D15" s="22"/>
       <c r="E15" s="10" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="13" t="s">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="B18" s="13"/>
-      <c r="C18" s="13"/>
-      <c r="D18" s="13"/>
-      <c r="E18" s="13"/>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B18" s="17"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="17"/>
+      <c r="E18" s="17"/>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B19" s="14" t="s">
+      <c r="B19" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="C19" s="14"/>
-      <c r="D19" s="14"/>
-      <c r="E19" s="14"/>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C19" s="18"/>
+      <c r="D19" s="18"/>
+      <c r="E19" s="18"/>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>6</v>
       </c>
@@ -1294,16 +3240,16 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" s="15" t="s">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="B21" s="15"/>
-      <c r="C21" s="15"/>
-      <c r="D21" s="15"/>
-      <c r="E21" s="15"/>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B21" s="19"/>
+      <c r="C21" s="19"/>
+      <c r="D21" s="19"/>
+      <c r="E21" s="19"/>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>7</v>
       </c>
@@ -1320,7 +3266,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
         <v>8</v>
       </c>
@@ -1337,7 +3283,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
         <v>9</v>
       </c>
@@ -1353,17 +3299,23 @@
       <c r="E24" s="10" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" s="15" t="s">
+      <c r="G24" s="29"/>
+      <c r="H24" s="30"/>
+      <c r="I24" s="30"/>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A25" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="B25" s="15"/>
-      <c r="C25" s="15"/>
-      <c r="D25" s="15"/>
-      <c r="E25" s="15"/>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B25" s="19"/>
+      <c r="C25" s="19"/>
+      <c r="D25" s="19"/>
+      <c r="E25" s="19"/>
+      <c r="G25" s="31"/>
+      <c r="H25" s="26"/>
+      <c r="I25" s="26"/>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
         <v>7</v>
       </c>
@@ -1379,8 +3331,11 @@
       <c r="E26" s="10" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="G26" s="32"/>
+      <c r="H26" s="33"/>
+      <c r="I26" s="34"/>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
         <v>8</v>
       </c>
@@ -1396,8 +3351,11 @@
       <c r="E27" s="10" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="G27" s="32"/>
+      <c r="H27" s="33"/>
+      <c r="I27" s="29"/>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
         <v>9</v>
       </c>
@@ -1413,8 +3371,11 @@
       <c r="E28" s="10" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="G28" s="35"/>
+      <c r="H28" s="29"/>
+      <c r="I28" s="29"/>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="C29" s="1" t="s">
         <v>40</v>
       </c>
@@ -1424,28 +3385,42 @@
       <c r="E29" s="1" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31" s="13" t="s">
-        <v>71</v>
-      </c>
-      <c r="B31" s="13"/>
-      <c r="C31" s="13"/>
-      <c r="D31" s="13"/>
-      <c r="E31" s="13"/>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="G29" s="32"/>
+      <c r="H29" s="33"/>
+      <c r="I29" s="29"/>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="G30" s="35"/>
+      <c r="H30" s="29"/>
+      <c r="I30" s="29"/>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A31" s="17" t="s">
+        <v>70</v>
+      </c>
+      <c r="B31" s="17"/>
+      <c r="C31" s="17"/>
+      <c r="D31" s="17"/>
+      <c r="E31" s="17"/>
+      <c r="G31" s="32"/>
+      <c r="H31" s="33"/>
+      <c r="I31" s="29"/>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B32" s="14" t="s">
+      <c r="B32" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="C32" s="14"/>
-      <c r="D32" s="14"/>
-      <c r="E32" s="14"/>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C32" s="18"/>
+      <c r="D32" s="18"/>
+      <c r="E32" s="18"/>
+      <c r="G32" s="35"/>
+      <c r="H32" s="29"/>
+      <c r="I32" s="29"/>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
         <v>6</v>
       </c>
@@ -1461,146 +3436,171 @@
       <c r="E33" s="8">
         <v>10000</v>
       </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A34" s="15" t="s">
+      <c r="G33" s="32"/>
+      <c r="H33" s="33"/>
+      <c r="I33" s="29"/>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A34" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="B34" s="15"/>
-      <c r="C34" s="15"/>
-      <c r="D34" s="15"/>
-      <c r="E34" s="15"/>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B34" s="19"/>
+      <c r="C34" s="19"/>
+      <c r="D34" s="19"/>
+      <c r="E34" s="19"/>
+      <c r="G34" s="35"/>
+      <c r="H34" s="29"/>
+      <c r="I34" s="29"/>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C35" s="10" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D35" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E35" s="10" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G35" s="35"/>
+      <c r="H35" s="29"/>
+      <c r="I35" s="29"/>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
         <v>8</v>
       </c>
       <c r="B36" s="9" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C36" s="10" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D36" s="10" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E36" s="10" t="s">
-        <v>54</v>
-      </c>
-      <c r="F36" s="1" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+        <v>53</v>
+      </c>
+      <c r="G36" s="35"/>
+      <c r="H36" s="29"/>
+      <c r="I36" s="29"/>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
         <v>9</v>
       </c>
       <c r="B37" s="9" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C37" s="10" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D37" s="10" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E37" s="10" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A38" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="G37" s="32"/>
+      <c r="H37" s="33"/>
+      <c r="I37" s="29"/>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A38" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="B38" s="15"/>
-      <c r="C38" s="15"/>
-      <c r="D38" s="15"/>
-      <c r="E38" s="15"/>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B38" s="19"/>
+      <c r="C38" s="19"/>
+      <c r="D38" s="19"/>
+      <c r="E38" s="19"/>
+      <c r="G38" s="35"/>
+      <c r="H38" s="29"/>
+      <c r="I38" s="29"/>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C39" s="10" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D39" s="10" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E39" s="10" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+        <v>63</v>
+      </c>
+      <c r="G39" s="35"/>
+      <c r="H39" s="29"/>
+      <c r="I39" s="29"/>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
         <v>8</v>
       </c>
       <c r="B40" s="9" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C40" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D40" s="10" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E40" s="10" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+        <v>64</v>
+      </c>
+      <c r="G40" s="35"/>
+      <c r="H40" s="29"/>
+      <c r="I40" s="29"/>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
         <v>9</v>
       </c>
       <c r="B41" s="9" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C41" s="10" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D41" s="10" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E41" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="G41" s="32"/>
+      <c r="H41" s="33"/>
+      <c r="I41" s="29"/>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B42" s="16" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B42" s="20" t="s">
-        <v>67</v>
-      </c>
-      <c r="C42" s="20"/>
-      <c r="D42" s="20"/>
-      <c r="E42" s="20"/>
+      <c r="C42" s="16"/>
+      <c r="D42" s="16"/>
+      <c r="E42" s="16"/>
     </row>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="16">
+    <mergeCell ref="H24:I24"/>
+    <mergeCell ref="G5:H8"/>
     <mergeCell ref="B42:E42"/>
     <mergeCell ref="A31:E31"/>
     <mergeCell ref="B32:E32"/>
     <mergeCell ref="A34:E34"/>
     <mergeCell ref="A38:E38"/>
-    <mergeCell ref="G5:K9"/>
     <mergeCell ref="B6:E6"/>
     <mergeCell ref="A12:E12"/>
     <mergeCell ref="A8:E8"/>
@@ -1616,4 +3616,232 @@
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09C7CB48-3C9F-48A0-8672-FA001DBD72EC}">
+  <dimension ref="B2:E24"/>
+  <sheetFormatPr defaultRowHeight="13.55" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="9.140625" style="42"/>
+    <col min="2" max="2" width="23.140625" style="42" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="21.28515625" style="42" customWidth="1"/>
+    <col min="5" max="16384" width="9.140625" style="42"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:5" ht="17.850000000000001" x14ac:dyDescent="0.25">
+      <c r="B2" s="25"/>
+      <c r="C2" s="27" t="s">
+        <v>78</v>
+      </c>
+      <c r="D2" s="27"/>
+    </row>
+    <row r="3" spans="2:5" ht="17.850000000000001" x14ac:dyDescent="0.25">
+      <c r="B3" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="C3" s="41" t="s">
+        <v>79</v>
+      </c>
+      <c r="D3" s="41" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="4" spans="2:5" ht="17.850000000000001" x14ac:dyDescent="0.25">
+      <c r="B4" s="23">
+        <v>1</v>
+      </c>
+      <c r="C4" s="36">
+        <v>40525</v>
+      </c>
+      <c r="D4" s="28">
+        <v>8737</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5" ht="17.850000000000001" x14ac:dyDescent="0.25">
+      <c r="B5" s="23">
+        <v>2</v>
+      </c>
+      <c r="C5" s="36">
+        <v>40933</v>
+      </c>
+      <c r="D5" s="28">
+        <v>8116</v>
+      </c>
+    </row>
+    <row r="6" spans="2:5" ht="17.850000000000001" x14ac:dyDescent="0.25">
+      <c r="B6" s="24">
+        <v>3</v>
+      </c>
+      <c r="C6" s="24">
+        <v>35748</v>
+      </c>
+      <c r="D6" s="24">
+        <v>8005</v>
+      </c>
+    </row>
+    <row r="7" spans="2:5" ht="17.850000000000001" x14ac:dyDescent="0.25">
+      <c r="B7" s="23">
+        <v>4</v>
+      </c>
+      <c r="C7" s="36">
+        <v>34657</v>
+      </c>
+      <c r="D7" s="28">
+        <v>7387</v>
+      </c>
+    </row>
+    <row r="8" spans="2:5" ht="17.850000000000001" x14ac:dyDescent="0.25">
+      <c r="B8" s="24">
+        <v>5</v>
+      </c>
+      <c r="C8" s="24">
+        <v>36335</v>
+      </c>
+      <c r="D8" s="24">
+        <v>6863</v>
+      </c>
+    </row>
+    <row r="9" spans="2:5" ht="17.850000000000001" x14ac:dyDescent="0.25">
+      <c r="B9" s="23">
+        <v>6</v>
+      </c>
+      <c r="C9" s="36">
+        <v>38071</v>
+      </c>
+      <c r="D9" s="28">
+        <v>7472</v>
+      </c>
+    </row>
+    <row r="10" spans="2:5" ht="17.850000000000001" x14ac:dyDescent="0.25">
+      <c r="B10" s="24">
+        <v>7</v>
+      </c>
+      <c r="C10" s="24">
+        <v>36151</v>
+      </c>
+      <c r="D10" s="24">
+        <v>6861</v>
+      </c>
+    </row>
+    <row r="11" spans="2:5" ht="17.850000000000001" x14ac:dyDescent="0.25">
+      <c r="B11" s="23">
+        <v>8</v>
+      </c>
+      <c r="C11" s="36">
+        <v>37594</v>
+      </c>
+      <c r="D11" s="28">
+        <v>7389</v>
+      </c>
+    </row>
+    <row r="12" spans="2:5" ht="17.850000000000001" x14ac:dyDescent="0.25">
+      <c r="B12" s="24">
+        <v>9</v>
+      </c>
+      <c r="C12" s="24">
+        <v>36727</v>
+      </c>
+      <c r="D12" s="24">
+        <v>7908</v>
+      </c>
+      <c r="E12" s="43"/>
+    </row>
+    <row r="13" spans="2:5" ht="17.850000000000001" x14ac:dyDescent="0.25">
+      <c r="B13" s="24">
+        <v>10</v>
+      </c>
+      <c r="C13" s="24">
+        <v>36931</v>
+      </c>
+      <c r="D13" s="24">
+        <v>8155</v>
+      </c>
+    </row>
+    <row r="14" spans="2:5" ht="17.850000000000001" x14ac:dyDescent="0.25">
+      <c r="B14" s="24">
+        <v>11</v>
+      </c>
+      <c r="C14" s="24">
+        <v>38323</v>
+      </c>
+      <c r="D14" s="24">
+        <v>7985</v>
+      </c>
+    </row>
+    <row r="15" spans="2:5" ht="17.850000000000001" x14ac:dyDescent="0.25">
+      <c r="B15" s="23">
+        <v>12</v>
+      </c>
+      <c r="C15" s="36">
+        <v>40896</v>
+      </c>
+      <c r="D15" s="28">
+        <v>8411</v>
+      </c>
+    </row>
+    <row r="16" spans="2:5" ht="17.850000000000001" x14ac:dyDescent="0.25">
+      <c r="B16" s="24">
+        <v>13</v>
+      </c>
+      <c r="C16" s="24">
+        <v>38132</v>
+      </c>
+      <c r="D16" s="24">
+        <v>8314</v>
+      </c>
+    </row>
+    <row r="17" spans="2:4" ht="17.850000000000001" x14ac:dyDescent="0.25">
+      <c r="B17" s="24">
+        <v>14</v>
+      </c>
+      <c r="C17" s="24">
+        <v>38962</v>
+      </c>
+      <c r="D17" s="24">
+        <v>8287</v>
+      </c>
+    </row>
+    <row r="18" spans="2:4" ht="17.850000000000001" x14ac:dyDescent="0.25">
+      <c r="B18" s="24">
+        <v>15</v>
+      </c>
+      <c r="C18" s="24">
+        <v>38825</v>
+      </c>
+      <c r="D18" s="24">
+        <v>8452</v>
+      </c>
+    </row>
+    <row r="19" spans="2:4" ht="17.850000000000001" x14ac:dyDescent="0.25">
+      <c r="B19" s="23">
+        <v>16</v>
+      </c>
+      <c r="C19" s="36">
+        <v>39364</v>
+      </c>
+      <c r="D19" s="28">
+        <v>7844</v>
+      </c>
+    </row>
+    <row r="20" spans="2:4" ht="17.850000000000001" x14ac:dyDescent="0.2">
+      <c r="C20" s="40">
+        <v>4</v>
+      </c>
+      <c r="D20" s="40">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="24" spans="2:4" ht="17.850000000000001" x14ac:dyDescent="0.25">
+      <c r="B24" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="C2:D2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Now I have a plan of work
</commit_message>
<xml_diff>
--- a/DecompositionLU/docs/statistics.xlsx
+++ b/DecompositionLU/docs/statistics.xlsx
@@ -1,24 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="22527"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="6" rupBuild="4505"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Maxim\source\repos\practice\SECOND_COURSE\FOR_ITLAB\ArchBenchs\DecompositionLU\docs\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BF38F48-B947-4425-AE12-16D6FDB9CE80}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-114" yWindow="-114" windowWidth="27602" windowHeight="15027" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="27600" windowHeight="15030" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Таблица" sheetId="1" r:id="rId1"/>
     <sheet name="Графики" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+  <calcPr calcId="124519"/>
+  <extLst xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -32,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="82">
   <si>
     <t>Я не уверен, будет ли это использоваться в готовой презентации и так ли это надо делать, если да, так что пока считаем, что файл для личного пользования.</t>
   </si>
@@ -351,8 +345,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="14" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -617,30 +611,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -651,16 +621,10 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -678,15 +642,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -695,6 +650,45 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -714,18 +708,9 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
-  <c:date1904 val="0"/>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:lang val="ru-RU"/>
-  <c:roundedCorners val="0"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
-      <c14:style val="104"/>
-    </mc:Choice>
-    <mc:Fallback>
-      <c:style val="4"/>
-    </mc:Fallback>
-  </mc:AlternateContent>
+  <c:style val="4"/>
   <c:chart>
     <c:title>
       <c:tx>
@@ -753,7 +738,7 @@
           </a:p>
         </c:rich>
       </c:tx>
-      <c:overlay val="0"/>
+      <c:layout/>
       <c:spPr>
         <a:noFill/>
         <a:ln>
@@ -761,33 +746,11 @@
         </a:ln>
         <a:effectLst/>
       </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="GOST Common" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="ru-RU"/>
-        </a:p>
-      </c:txPr>
     </c:title>
-    <c:autoTitleDeleted val="0"/>
     <c:plotArea>
       <c:layout/>
       <c:lineChart>
         <c:grouping val="standard"/>
-        <c:varyColors val="0"/>
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
@@ -872,35 +835,24 @@
               </c:numCache>
             </c:numRef>
           </c:val>
-          <c:smooth val="0"/>
-          <c:extLst>
+          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000000-DFDA-4FBA-8E35-21ED64A1AC56}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
-        <c:dLbls>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-        </c:dLbls>
+        <c:dLbls/>
         <c:marker val="1"/>
-        <c:smooth val="0"/>
-        <c:axId val="2034815519"/>
-        <c:axId val="1972086687"/>
+        <c:axId val="153173376"/>
+        <c:axId val="153175168"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="2034815519"/>
+        <c:axId val="153173376"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
-        <c:delete val="0"/>
         <c:axPos val="b"/>
         <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
           <a:noFill/>
@@ -935,20 +887,18 @@
             <a:endParaRPr lang="ru-RU"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1972086687"/>
+        <c:crossAx val="153175168"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
-        <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1972086687"/>
+        <c:axId val="153175168"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="34000"/>
         </c:scaling>
-        <c:delete val="0"/>
         <c:axPos val="l"/>
         <c:majorGridlines>
           <c:spPr>
@@ -966,7 +916,6 @@
         </c:majorGridlines>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
           <a:noFill/>
@@ -995,7 +944,7 @@
             <a:endParaRPr lang="ru-RU"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2034815519"/>
+        <c:crossAx val="153173376"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1009,14 +958,13 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:extLst>
+    <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
           <c16r3:dispNaAsBlank val="1"/>
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1047,25 +995,16 @@
   </c:txPr>
   <c:printSettings>
     <c:headerFooter/>
-    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageMargins b="0.75000000000000011" l="0.70000000000000007" r="0.70000000000000007" t="0.75000000000000011" header="0.30000000000000004" footer="0.30000000000000004"/>
     <c:pageSetup/>
   </c:printSettings>
 </c:chartSpace>
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
-  <c:date1904 val="0"/>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:lang val="ru-RU"/>
-  <c:roundedCorners val="0"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
-      <c14:style val="108"/>
-    </mc:Choice>
-    <mc:Fallback>
-      <c:style val="8"/>
-    </mc:Fallback>
-  </mc:AlternateContent>
+  <c:style val="8"/>
   <c:chart>
     <c:title>
       <c:tx>
@@ -1093,7 +1032,7 @@
           </a:p>
         </c:rich>
       </c:tx>
-      <c:overlay val="0"/>
+      <c:layout/>
       <c:spPr>
         <a:noFill/>
         <a:ln>
@@ -1101,33 +1040,11 @@
         </a:ln>
         <a:effectLst/>
       </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="GOST Common" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="ru-RU"/>
-        </a:p>
-      </c:txPr>
     </c:title>
-    <c:autoTitleDeleted val="0"/>
     <c:plotArea>
       <c:layout/>
       <c:lineChart>
         <c:grouping val="standard"/>
-        <c:varyColors val="0"/>
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
@@ -1212,35 +1129,24 @@
               </c:numCache>
             </c:numRef>
           </c:val>
-          <c:smooth val="0"/>
-          <c:extLst>
+          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000000-8747-4A5E-85F4-772AAE4EC689}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
-        <c:dLbls>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-        </c:dLbls>
+        <c:dLbls/>
         <c:marker val="1"/>
-        <c:smooth val="0"/>
-        <c:axId val="52875439"/>
-        <c:axId val="1972084607"/>
+        <c:axId val="153621248"/>
+        <c:axId val="153622784"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="52875439"/>
+        <c:axId val="153621248"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
-        <c:delete val="0"/>
         <c:axPos val="b"/>
         <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
           <a:noFill/>
@@ -1275,20 +1181,18 @@
             <a:endParaRPr lang="ru-RU"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1972084607"/>
+        <c:crossAx val="153622784"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
-        <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1972084607"/>
+        <c:axId val="153622784"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="6500"/>
         </c:scaling>
-        <c:delete val="0"/>
         <c:axPos val="l"/>
         <c:majorGridlines>
           <c:spPr>
@@ -1306,7 +1210,6 @@
         </c:majorGridlines>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
           <a:noFill/>
@@ -1335,7 +1238,7 @@
             <a:endParaRPr lang="ru-RU"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="52875439"/>
+        <c:crossAx val="153621248"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1349,14 +1252,13 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:extLst>
+    <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
           <c16r3:dispNaAsBlank val="1"/>
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1387,1028 +1289,118 @@
   </c:txPr>
   <c:printSettings>
     <c:headerFooter/>
-    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageMargins b="0.75000000000000011" l="0.70000000000000007" r="0.70000000000000007" t="0.75000000000000011" header="0.30000000000000004" footer="0.30000000000000004"/>
     <c:pageSetup/>
   </c:printSettings>
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="withinLinear" id="15">
-  <a:schemeClr val="accent2"/>
-</cs:colorStyle>
-</file>
-
-<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="withinLinear" id="19">
-  <a:schemeClr val="accent6"/>
-</cs:colorStyle>
-</file>
-
-<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="332">
-  <cs:axisTitle>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:axisTitle>
-  <cs:categoryAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:categoryAxis>
-  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="bg1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:chartArea>
-  <cs:dataLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="75000"/>
-        <a:lumOff val="25000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataLabel>
-  <cs:dataLabelCallout>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
-      <a:spAutoFit/>
-    </cs:bodyPr>
-  </cs:dataLabelCallout>
-  <cs:dataPoint>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:dataPoint>
-  <cs:dataPoint3D>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:dataPoint3D>
-  <cs:dataPointLine>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="28575" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointLine>
-  <cs:dataPointMarker>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointMarker>
-  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
-  <cs:dataPointWireframe>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointWireframe>
-  <cs:dataTable>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataTable>
-  <cs:downBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="dk1">
-          <a:lumMod val="65000"/>
-          <a:lumOff val="35000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:downBar>
-  <cs:dropLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dropLine>
-  <cs:errorBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:errorBar>
-  <cs:floor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
-  </cs:floor>
-  <cs:gridlineMajor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMajor>
-  <cs:gridlineMinor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="5000"/>
-            <a:lumOff val="95000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMinor>
-  <cs:hiLoLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="75000"/>
-            <a:lumOff val="25000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:hiLoLine>
-  <cs:leaderLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:leaderLine>
-  <cs:legend>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:legend>
-  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea>
-  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea3D>
-  <cs:seriesAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:seriesAxis>
-  <cs:seriesLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:seriesLine>
-  <cs:title>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
-  </cs:title>
-  <cs:trendline>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="19050" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:prstDash val="sysDot"/>
-      </a:ln>
-    </cs:spPr>
-  </cs:trendline>
-  <cs:trendlineLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:trendlineLabel>
-  <cs:upBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:upBar>
-  <cs:valueAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:valueAxis>
-  <cs:wall>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
-  </cs:wall>
-</cs:chartStyle>
-</file>
-
-<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="332">
-  <cs:axisTitle>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:axisTitle>
-  <cs:categoryAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:categoryAxis>
-  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="bg1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:chartArea>
-  <cs:dataLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="75000"/>
-        <a:lumOff val="25000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataLabel>
-  <cs:dataLabelCallout>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
-      <a:spAutoFit/>
-    </cs:bodyPr>
-  </cs:dataLabelCallout>
-  <cs:dataPoint>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:dataPoint>
-  <cs:dataPoint3D>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:dataPoint3D>
-  <cs:dataPointLine>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="28575" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointLine>
-  <cs:dataPointMarker>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointMarker>
-  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
-  <cs:dataPointWireframe>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointWireframe>
-  <cs:dataTable>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataTable>
-  <cs:downBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="dk1">
-          <a:lumMod val="65000"/>
-          <a:lumOff val="35000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:downBar>
-  <cs:dropLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dropLine>
-  <cs:errorBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:errorBar>
-  <cs:floor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
-  </cs:floor>
-  <cs:gridlineMajor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMajor>
-  <cs:gridlineMinor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="5000"/>
-            <a:lumOff val="95000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMinor>
-  <cs:hiLoLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="75000"/>
-            <a:lumOff val="25000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:hiLoLine>
-  <cs:leaderLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:leaderLine>
-  <cs:legend>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:legend>
-  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea>
-  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea3D>
-  <cs:seriesAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:seriesAxis>
-  <cs:seriesLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:seriesLine>
-  <cs:title>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
-  </cs:title>
-  <cs:trendline>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="19050" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:prstDash val="sysDot"/>
-      </a:ln>
-    </cs:spPr>
-  </cs:trendline>
-  <cs:trendlineLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:trendlineLabel>
-  <cs:upBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:upBar>
-  <cs:valueAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:valueAxis>
-  <cs:wall>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
-  </cs:wall>
-</cs:chartStyle>
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="ru-RU"/>
+  <c:chart>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln w="19050">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Графики!$O$4:$O$8</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Графики!$Q$4:$Q$8</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>4557</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3948</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4020</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3448</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>3996</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+        </c:ser>
+        <c:axId val="54167424"/>
+        <c:axId val="54165888"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="54167424"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="54165888"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="54165888"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="l"/>
+        <c:majorGridlines/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="54167424"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:layout/>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2426,7 +1418,7 @@
         <xdr:cNvPr id="2" name="TextBox 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{77301E52-0432-4D04-B3B3-00D890F3A041}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{77301E52-0432-4D04-B3B3-00D890F3A041}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2481,7 +1473,7 @@
         <xdr:cNvPr id="3" name="TextBox 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A60DEF0B-7AC5-4BE9-B97A-367940A351A6}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{A60DEF0B-7AC5-4BE9-B97A-367940A351A6}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2536,7 +1528,7 @@
         <xdr:cNvPr id="4" name="TextBox 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{35C2101E-3BC3-486A-87D7-AB0DA6ED7DA8}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{35C2101E-3BC3-486A-87D7-AB0DA6ED7DA8}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2601,7 +1593,7 @@
         <xdr:cNvPr id="5" name="Диаграмма 4">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D9C1BB01-F75F-4D40-BA20-D7288523072B}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{D9C1BB01-F75F-4D40-BA20-D7288523072B}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2637,7 +1629,7 @@
         <xdr:cNvPr id="7" name="Диаграмма 6">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{63E3D050-E508-4926-853F-B56EA689B234}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{63E3D050-E508-4926-853F-B56EA689B234}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2650,6 +1642,36 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>257175</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>561975</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="8" name="Диаграмма 7"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2701,7 +1723,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Calibri Light"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="Yu Gothic Light"/>
@@ -2736,7 +1758,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="Yu Gothic"/>
@@ -2913,16 +1935,16 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:W42"/>
-  <sheetFormatPr defaultRowHeight="17.850000000000001" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="65.7109375" style="1" customWidth="1"/>
     <col min="2" max="5" width="26.7109375" style="1" customWidth="1"/>
@@ -2932,7 +1954,7 @@
     <col min="10" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:23">
       <c r="A1" s="2" t="s">
         <v>1</v>
       </c>
@@ -2956,7 +1978,7 @@
       <c r="S1" s="2"/>
       <c r="T1" s="2"/>
     </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:23">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -2980,7 +2002,7 @@
       <c r="S2" s="2"/>
       <c r="T2" s="2"/>
     </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:23">
       <c r="A3" s="6" t="s">
         <v>2</v>
       </c>
@@ -2998,7 +2020,7 @@
       <c r="M3" s="6"/>
       <c r="N3" s="6"/>
     </row>
-    <row r="5" spans="1:23" ht="17.850000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:23" ht="17.850000000000001" customHeight="1">
       <c r="A5" s="37" t="s">
         <v>22</v>
       </c>
@@ -3006,35 +2028,35 @@
       <c r="C5" s="38"/>
       <c r="D5" s="38"/>
       <c r="E5" s="39"/>
-      <c r="G5" s="15" t="s">
+      <c r="G5" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="H5" s="15"/>
+      <c r="H5" s="32"/>
       <c r="S5" s="5"/>
       <c r="T5" s="14"/>
       <c r="U5" s="14"/>
       <c r="V5" s="14"/>
       <c r="W5" s="14"/>
     </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:23" ht="18.75">
       <c r="A6" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="18" t="s">
+      <c r="B6" s="35" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="18"/>
-      <c r="D6" s="18"/>
-      <c r="E6" s="18"/>
-      <c r="G6" s="15"/>
-      <c r="H6" s="15"/>
+      <c r="C6" s="35"/>
+      <c r="D6" s="35"/>
+      <c r="E6" s="35"/>
+      <c r="G6" s="32"/>
+      <c r="H6" s="32"/>
       <c r="S6" s="14"/>
       <c r="T6" s="14"/>
       <c r="U6" s="14"/>
       <c r="V6" s="14"/>
       <c r="W6" s="14"/>
     </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:23" ht="18.75">
       <c r="A7" s="3" t="s">
         <v>6</v>
       </c>
@@ -3050,31 +2072,31 @@
       <c r="E7" s="8">
         <v>10000</v>
       </c>
-      <c r="G7" s="15"/>
-      <c r="H7" s="15"/>
+      <c r="G7" s="32"/>
+      <c r="H7" s="32"/>
       <c r="S7" s="14"/>
       <c r="T7" s="14"/>
       <c r="U7" s="14"/>
       <c r="V7" s="14"/>
       <c r="W7" s="14"/>
     </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A8" s="19" t="s">
+    <row r="8" spans="1:23" ht="18.75">
+      <c r="A8" s="36" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="19"/>
-      <c r="C8" s="19"/>
-      <c r="D8" s="19"/>
-      <c r="E8" s="19"/>
-      <c r="G8" s="15"/>
-      <c r="H8" s="15"/>
+      <c r="B8" s="36"/>
+      <c r="C8" s="36"/>
+      <c r="D8" s="36"/>
+      <c r="E8" s="36"/>
+      <c r="G8" s="32"/>
+      <c r="H8" s="32"/>
       <c r="S8" s="14"/>
       <c r="T8" s="14"/>
       <c r="U8" s="14"/>
       <c r="V8" s="14"/>
       <c r="W8" s="14"/>
     </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:23" ht="18.75">
       <c r="A9" s="3" t="s">
         <v>7</v>
       </c>
@@ -3096,7 +2118,7 @@
       <c r="V9" s="14"/>
       <c r="W9" s="14"/>
     </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:23">
       <c r="A10" s="3" t="s">
         <v>8</v>
       </c>
@@ -3118,7 +2140,7 @@
       <c r="V10" s="5"/>
       <c r="W10" s="5"/>
     </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:23">
       <c r="A11" s="3" t="s">
         <v>9</v>
       </c>
@@ -3142,17 +2164,17 @@
       <c r="V11" s="5"/>
       <c r="W11" s="5"/>
     </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A12" s="19" t="s">
+    <row r="12" spans="1:23">
+      <c r="A12" s="36" t="s">
         <v>12</v>
       </c>
-      <c r="B12" s="19"/>
-      <c r="C12" s="19"/>
-      <c r="D12" s="19"/>
-      <c r="E12" s="19"/>
+      <c r="B12" s="36"/>
+      <c r="C12" s="36"/>
+      <c r="D12" s="36"/>
+      <c r="E12" s="36"/>
       <c r="F12" s="5"/>
     </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:23">
       <c r="A13" s="3" t="s">
         <v>7</v>
       </c>
@@ -3162,7 +2184,7 @@
       <c r="C13" s="10">
         <v>232</v>
       </c>
-      <c r="D13" s="20" t="s">
+      <c r="D13" s="40" t="s">
         <v>21</v>
       </c>
       <c r="E13" s="10">
@@ -3170,7 +2192,7 @@
       </c>
       <c r="F13" s="5"/>
     </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:23">
       <c r="A14" s="3" t="s">
         <v>8</v>
       </c>
@@ -3180,7 +2202,7 @@
       <c r="C14" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="D14" s="21"/>
+      <c r="D14" s="41"/>
       <c r="E14" s="10" t="s">
         <v>10</v>
       </c>
@@ -3188,7 +2210,7 @@
       <c r="G14" s="5"/>
       <c r="H14" s="5"/>
     </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:23">
       <c r="A15" s="3" t="s">
         <v>9</v>
       </c>
@@ -3198,32 +2220,32 @@
       <c r="C15" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="D15" s="22"/>
+      <c r="D15" s="42"/>
       <c r="E15" s="10" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A18" s="17" t="s">
+    <row r="18" spans="1:9">
+      <c r="A18" s="34" t="s">
         <v>32</v>
       </c>
-      <c r="B18" s="17"/>
-      <c r="C18" s="17"/>
-      <c r="D18" s="17"/>
-      <c r="E18" s="17"/>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B18" s="34"/>
+      <c r="C18" s="34"/>
+      <c r="D18" s="34"/>
+      <c r="E18" s="34"/>
+    </row>
+    <row r="19" spans="1:9">
       <c r="A19" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B19" s="18" t="s">
+      <c r="B19" s="35" t="s">
         <v>5</v>
       </c>
-      <c r="C19" s="18"/>
-      <c r="D19" s="18"/>
-      <c r="E19" s="18"/>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C19" s="35"/>
+      <c r="D19" s="35"/>
+      <c r="E19" s="35"/>
+    </row>
+    <row r="20" spans="1:9">
       <c r="A20" s="3" t="s">
         <v>6</v>
       </c>
@@ -3240,16 +2262,16 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A21" s="19" t="s">
+    <row r="21" spans="1:9">
+      <c r="A21" s="36" t="s">
         <v>11</v>
       </c>
-      <c r="B21" s="19"/>
-      <c r="C21" s="19"/>
-      <c r="D21" s="19"/>
-      <c r="E21" s="19"/>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B21" s="36"/>
+      <c r="C21" s="36"/>
+      <c r="D21" s="36"/>
+      <c r="E21" s="36"/>
+    </row>
+    <row r="22" spans="1:9">
       <c r="A22" s="3" t="s">
         <v>7</v>
       </c>
@@ -3266,7 +2288,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9">
       <c r="A23" s="3" t="s">
         <v>8</v>
       </c>
@@ -3283,7 +2305,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9">
       <c r="A24" s="3" t="s">
         <v>9</v>
       </c>
@@ -3299,23 +2321,23 @@
       <c r="E24" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="G24" s="29"/>
-      <c r="H24" s="30"/>
-      <c r="I24" s="30"/>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" s="19" t="s">
+      <c r="G24" s="20"/>
+      <c r="H24" s="31"/>
+      <c r="I24" s="31"/>
+    </row>
+    <row r="25" spans="1:9">
+      <c r="A25" s="36" t="s">
         <v>12</v>
       </c>
-      <c r="B25" s="19"/>
-      <c r="C25" s="19"/>
-      <c r="D25" s="19"/>
-      <c r="E25" s="19"/>
-      <c r="G25" s="31"/>
-      <c r="H25" s="26"/>
-      <c r="I25" s="26"/>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B25" s="36"/>
+      <c r="C25" s="36"/>
+      <c r="D25" s="36"/>
+      <c r="E25" s="36"/>
+      <c r="G25" s="21"/>
+      <c r="H25" s="18"/>
+      <c r="I25" s="18"/>
+    </row>
+    <row r="26" spans="1:9" ht="18.75">
       <c r="A26" s="3" t="s">
         <v>7</v>
       </c>
@@ -3331,11 +2353,11 @@
       <c r="E26" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="G26" s="32"/>
-      <c r="H26" s="33"/>
-      <c r="I26" s="34"/>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="G26" s="22"/>
+      <c r="H26" s="23"/>
+      <c r="I26" s="24"/>
+    </row>
+    <row r="27" spans="1:9" ht="18.75">
       <c r="A27" s="3" t="s">
         <v>8</v>
       </c>
@@ -3351,11 +2373,11 @@
       <c r="E27" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="G27" s="32"/>
-      <c r="H27" s="33"/>
-      <c r="I27" s="29"/>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="G27" s="22"/>
+      <c r="H27" s="23"/>
+      <c r="I27" s="20"/>
+    </row>
+    <row r="28" spans="1:9" ht="18.75">
       <c r="A28" s="3" t="s">
         <v>9</v>
       </c>
@@ -3371,11 +2393,11 @@
       <c r="E28" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="G28" s="35"/>
-      <c r="H28" s="29"/>
-      <c r="I28" s="29"/>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="G28" s="25"/>
+      <c r="H28" s="20"/>
+      <c r="I28" s="20"/>
+    </row>
+    <row r="29" spans="1:9" ht="18.75">
       <c r="C29" s="1" t="s">
         <v>40</v>
       </c>
@@ -3385,42 +2407,42 @@
       <c r="E29" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="G29" s="32"/>
-      <c r="H29" s="33"/>
-      <c r="I29" s="29"/>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="G30" s="35"/>
-      <c r="H30" s="29"/>
-      <c r="I30" s="29"/>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A31" s="17" t="s">
+      <c r="G29" s="22"/>
+      <c r="H29" s="23"/>
+      <c r="I29" s="20"/>
+    </row>
+    <row r="30" spans="1:9" ht="18.75">
+      <c r="G30" s="25"/>
+      <c r="H30" s="20"/>
+      <c r="I30" s="20"/>
+    </row>
+    <row r="31" spans="1:9" ht="18.75">
+      <c r="A31" s="34" t="s">
         <v>70</v>
       </c>
-      <c r="B31" s="17"/>
-      <c r="C31" s="17"/>
-      <c r="D31" s="17"/>
-      <c r="E31" s="17"/>
-      <c r="G31" s="32"/>
-      <c r="H31" s="33"/>
-      <c r="I31" s="29"/>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B31" s="34"/>
+      <c r="C31" s="34"/>
+      <c r="D31" s="34"/>
+      <c r="E31" s="34"/>
+      <c r="G31" s="22"/>
+      <c r="H31" s="23"/>
+      <c r="I31" s="20"/>
+    </row>
+    <row r="32" spans="1:9" ht="18.75">
       <c r="A32" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B32" s="18" t="s">
+      <c r="B32" s="35" t="s">
         <v>5</v>
       </c>
-      <c r="C32" s="18"/>
-      <c r="D32" s="18"/>
-      <c r="E32" s="18"/>
-      <c r="G32" s="35"/>
-      <c r="H32" s="29"/>
-      <c r="I32" s="29"/>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C32" s="35"/>
+      <c r="D32" s="35"/>
+      <c r="E32" s="35"/>
+      <c r="G32" s="25"/>
+      <c r="H32" s="20"/>
+      <c r="I32" s="20"/>
+    </row>
+    <row r="33" spans="1:9" ht="18.75">
       <c r="A33" s="3" t="s">
         <v>6</v>
       </c>
@@ -3436,23 +2458,23 @@
       <c r="E33" s="8">
         <v>10000</v>
       </c>
-      <c r="G33" s="32"/>
-      <c r="H33" s="33"/>
-      <c r="I33" s="29"/>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A34" s="19" t="s">
+      <c r="G33" s="22"/>
+      <c r="H33" s="23"/>
+      <c r="I33" s="20"/>
+    </row>
+    <row r="34" spans="1:9" ht="18.75">
+      <c r="A34" s="36" t="s">
         <v>11</v>
       </c>
-      <c r="B34" s="19"/>
-      <c r="C34" s="19"/>
-      <c r="D34" s="19"/>
-      <c r="E34" s="19"/>
-      <c r="G34" s="35"/>
-      <c r="H34" s="29"/>
-      <c r="I34" s="29"/>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B34" s="36"/>
+      <c r="C34" s="36"/>
+      <c r="D34" s="36"/>
+      <c r="E34" s="36"/>
+      <c r="G34" s="25"/>
+      <c r="H34" s="20"/>
+      <c r="I34" s="20"/>
+    </row>
+    <row r="35" spans="1:9" ht="18.75">
       <c r="A35" s="3" t="s">
         <v>7</v>
       </c>
@@ -3468,11 +2490,11 @@
       <c r="E35" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="G35" s="35"/>
-      <c r="H35" s="29"/>
-      <c r="I35" s="29"/>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="G35" s="25"/>
+      <c r="H35" s="20"/>
+      <c r="I35" s="20"/>
+    </row>
+    <row r="36" spans="1:9" ht="18.75">
       <c r="A36" s="3" t="s">
         <v>8</v>
       </c>
@@ -3488,11 +2510,11 @@
       <c r="E36" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="G36" s="35"/>
-      <c r="H36" s="29"/>
-      <c r="I36" s="29"/>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="G36" s="25"/>
+      <c r="H36" s="20"/>
+      <c r="I36" s="20"/>
+    </row>
+    <row r="37" spans="1:9" ht="18.75">
       <c r="A37" s="3" t="s">
         <v>9</v>
       </c>
@@ -3508,23 +2530,23 @@
       <c r="E37" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="G37" s="32"/>
-      <c r="H37" s="33"/>
-      <c r="I37" s="29"/>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A38" s="19" t="s">
+      <c r="G37" s="22"/>
+      <c r="H37" s="23"/>
+      <c r="I37" s="20"/>
+    </row>
+    <row r="38" spans="1:9" ht="18.75">
+      <c r="A38" s="36" t="s">
         <v>12</v>
       </c>
-      <c r="B38" s="19"/>
-      <c r="C38" s="19"/>
-      <c r="D38" s="19"/>
-      <c r="E38" s="19"/>
-      <c r="G38" s="35"/>
-      <c r="H38" s="29"/>
-      <c r="I38" s="29"/>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B38" s="36"/>
+      <c r="C38" s="36"/>
+      <c r="D38" s="36"/>
+      <c r="E38" s="36"/>
+      <c r="G38" s="25"/>
+      <c r="H38" s="20"/>
+      <c r="I38" s="20"/>
+    </row>
+    <row r="39" spans="1:9" ht="18.75">
       <c r="A39" s="3" t="s">
         <v>7</v>
       </c>
@@ -3540,11 +2562,11 @@
       <c r="E39" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="G39" s="35"/>
-      <c r="H39" s="29"/>
-      <c r="I39" s="29"/>
-    </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="G39" s="25"/>
+      <c r="H39" s="20"/>
+      <c r="I39" s="20"/>
+    </row>
+    <row r="40" spans="1:9" ht="18.75">
       <c r="A40" s="3" t="s">
         <v>8</v>
       </c>
@@ -3560,11 +2582,11 @@
       <c r="E40" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="G40" s="35"/>
-      <c r="H40" s="29"/>
-      <c r="I40" s="29"/>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="G40" s="25"/>
+      <c r="H40" s="20"/>
+      <c r="I40" s="20"/>
+    </row>
+    <row r="41" spans="1:9" ht="18.75">
       <c r="A41" s="3" t="s">
         <v>9</v>
       </c>
@@ -3580,17 +2602,17 @@
       <c r="E41" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="G41" s="32"/>
-      <c r="H41" s="33"/>
-      <c r="I41" s="29"/>
-    </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B42" s="16" t="s">
+      <c r="G41" s="22"/>
+      <c r="H41" s="23"/>
+      <c r="I41" s="20"/>
+    </row>
+    <row r="42" spans="1:9">
+      <c r="B42" s="33" t="s">
         <v>66</v>
       </c>
-      <c r="C42" s="16"/>
-      <c r="D42" s="16"/>
-      <c r="E42" s="16"/>
+      <c r="C42" s="33"/>
+      <c r="D42" s="33"/>
+      <c r="E42" s="33"/>
     </row>
   </sheetData>
   <mergeCells count="16">
@@ -3619,227 +2641,330 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09C7CB48-3C9F-48A0-8672-FA001DBD72EC}">
-  <dimension ref="B2:E24"/>
-  <sheetFormatPr defaultRowHeight="13.55" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="B2:Q24"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="9.140625" style="42"/>
-    <col min="2" max="2" width="23.140625" style="42" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="21.28515625" style="42" customWidth="1"/>
-    <col min="5" max="16384" width="9.140625" style="42"/>
+    <col min="1" max="1" width="9.140625" style="29"/>
+    <col min="2" max="2" width="23.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="21.28515625" style="29" customWidth="1"/>
+    <col min="5" max="14" width="9.140625" style="29"/>
+    <col min="15" max="15" width="23" style="29" bestFit="1" customWidth="1"/>
+    <col min="16" max="17" width="15.28515625" style="29" customWidth="1"/>
+    <col min="18" max="16384" width="9.140625" style="29"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:5" ht="17.850000000000001" x14ac:dyDescent="0.25">
-      <c r="B2" s="25"/>
-      <c r="C2" s="27" t="s">
+    <row r="2" spans="2:17" ht="18">
+      <c r="B2" s="17"/>
+      <c r="C2" s="43" t="s">
         <v>78</v>
       </c>
-      <c r="D2" s="27"/>
-    </row>
-    <row r="3" spans="2:5" ht="17.850000000000001" x14ac:dyDescent="0.25">
+      <c r="D2" s="43"/>
+      <c r="O2" s="17"/>
+      <c r="P2" s="43" t="s">
+        <v>78</v>
+      </c>
+      <c r="Q2" s="43"/>
+    </row>
+    <row r="3" spans="2:17" ht="18">
       <c r="B3" s="13" t="s">
         <v>77</v>
       </c>
-      <c r="C3" s="41" t="s">
+      <c r="C3" s="28" t="s">
         <v>79</v>
       </c>
-      <c r="D3" s="41" t="s">
+      <c r="D3" s="28" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="4" spans="2:5" ht="17.850000000000001" x14ac:dyDescent="0.25">
-      <c r="B4" s="23">
+      <c r="O3" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="P3" s="28" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q3" s="28" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="4" spans="2:17" ht="18.75">
+      <c r="B4" s="15">
         <v>1</v>
       </c>
-      <c r="C4" s="36">
+      <c r="C4" s="26">
         <v>40525</v>
       </c>
-      <c r="D4" s="28">
+      <c r="D4" s="19">
         <v>8737</v>
       </c>
-    </row>
-    <row r="5" spans="2:5" ht="17.850000000000001" x14ac:dyDescent="0.25">
-      <c r="B5" s="23">
+      <c r="O4" s="15">
+        <v>1</v>
+      </c>
+      <c r="Q4" s="19">
+        <v>4557</v>
+      </c>
+    </row>
+    <row r="5" spans="2:17" ht="18.75">
+      <c r="B5" s="15">
         <v>2</v>
       </c>
-      <c r="C5" s="36">
+      <c r="C5" s="26">
         <v>40933</v>
       </c>
-      <c r="D5" s="28">
+      <c r="D5" s="19">
         <v>8116</v>
       </c>
-    </row>
-    <row r="6" spans="2:5" ht="17.850000000000001" x14ac:dyDescent="0.25">
-      <c r="B6" s="24">
+      <c r="O5" s="15">
+        <v>2</v>
+      </c>
+      <c r="Q5" s="19">
+        <v>3948</v>
+      </c>
+    </row>
+    <row r="6" spans="2:17" ht="18.75">
+      <c r="B6" s="16">
         <v>3</v>
       </c>
-      <c r="C6" s="24">
+      <c r="C6" s="16">
         <v>35748</v>
       </c>
-      <c r="D6" s="24">
+      <c r="D6" s="16">
         <v>8005</v>
       </c>
-    </row>
-    <row r="7" spans="2:5" ht="17.850000000000001" x14ac:dyDescent="0.25">
-      <c r="B7" s="23">
+      <c r="O6" s="16">
+        <v>3</v>
+      </c>
+      <c r="Q6" s="16">
+        <v>4020</v>
+      </c>
+    </row>
+    <row r="7" spans="2:17" ht="18.75">
+      <c r="B7" s="15">
         <v>4</v>
       </c>
-      <c r="C7" s="36">
+      <c r="C7" s="26">
         <v>34657</v>
       </c>
-      <c r="D7" s="28">
+      <c r="D7" s="19">
         <v>7387</v>
       </c>
-    </row>
-    <row r="8" spans="2:5" ht="17.850000000000001" x14ac:dyDescent="0.25">
-      <c r="B8" s="24">
+      <c r="O7" s="15">
+        <v>4</v>
+      </c>
+      <c r="Q7" s="19">
+        <v>3448</v>
+      </c>
+    </row>
+    <row r="8" spans="2:17" ht="18.75">
+      <c r="B8" s="16">
         <v>5</v>
       </c>
-      <c r="C8" s="24">
+      <c r="C8" s="16">
         <v>36335</v>
       </c>
-      <c r="D8" s="24">
+      <c r="D8" s="16">
         <v>6863</v>
       </c>
-    </row>
-    <row r="9" spans="2:5" ht="17.850000000000001" x14ac:dyDescent="0.25">
-      <c r="B9" s="23">
+      <c r="O8" s="16">
+        <v>5</v>
+      </c>
+      <c r="Q8" s="16">
+        <v>3996</v>
+      </c>
+    </row>
+    <row r="9" spans="2:17" ht="18.75">
+      <c r="B9" s="15">
         <v>6</v>
       </c>
-      <c r="C9" s="36">
+      <c r="C9" s="26">
         <v>38071</v>
       </c>
-      <c r="D9" s="28">
+      <c r="D9" s="19">
         <v>7472</v>
       </c>
-    </row>
-    <row r="10" spans="2:5" ht="17.850000000000001" x14ac:dyDescent="0.25">
-      <c r="B10" s="24">
+      <c r="O9" s="15">
+        <v>6</v>
+      </c>
+      <c r="P9" s="26"/>
+      <c r="Q9" s="19"/>
+    </row>
+    <row r="10" spans="2:17" ht="18.75">
+      <c r="B10" s="16">
         <v>7</v>
       </c>
-      <c r="C10" s="24">
+      <c r="C10" s="16">
         <v>36151</v>
       </c>
-      <c r="D10" s="24">
+      <c r="D10" s="16">
         <v>6861</v>
       </c>
-    </row>
-    <row r="11" spans="2:5" ht="17.850000000000001" x14ac:dyDescent="0.25">
-      <c r="B11" s="23">
+      <c r="O10" s="16">
+        <v>7</v>
+      </c>
+      <c r="P10" s="16"/>
+      <c r="Q10" s="16"/>
+    </row>
+    <row r="11" spans="2:17" ht="18.75">
+      <c r="B11" s="15">
         <v>8</v>
       </c>
-      <c r="C11" s="36">
+      <c r="C11" s="26">
         <v>37594</v>
       </c>
-      <c r="D11" s="28">
+      <c r="D11" s="19">
         <v>7389</v>
       </c>
-    </row>
-    <row r="12" spans="2:5" ht="17.850000000000001" x14ac:dyDescent="0.25">
-      <c r="B12" s="24">
+      <c r="O11" s="15">
+        <v>8</v>
+      </c>
+      <c r="P11" s="26"/>
+      <c r="Q11" s="19"/>
+    </row>
+    <row r="12" spans="2:17" ht="18.75">
+      <c r="B12" s="16">
         <v>9</v>
       </c>
-      <c r="C12" s="24">
+      <c r="C12" s="16">
         <v>36727</v>
       </c>
-      <c r="D12" s="24">
+      <c r="D12" s="16">
         <v>7908</v>
       </c>
-      <c r="E12" s="43"/>
-    </row>
-    <row r="13" spans="2:5" ht="17.850000000000001" x14ac:dyDescent="0.25">
-      <c r="B13" s="24">
+      <c r="E12" s="30"/>
+      <c r="O12" s="16">
+        <v>9</v>
+      </c>
+      <c r="P12" s="16"/>
+      <c r="Q12" s="16"/>
+    </row>
+    <row r="13" spans="2:17" ht="18.75">
+      <c r="B13" s="16">
         <v>10</v>
       </c>
-      <c r="C13" s="24">
+      <c r="C13" s="16">
         <v>36931</v>
       </c>
-      <c r="D13" s="24">
+      <c r="D13" s="16">
         <v>8155</v>
       </c>
-    </row>
-    <row r="14" spans="2:5" ht="17.850000000000001" x14ac:dyDescent="0.25">
-      <c r="B14" s="24">
+      <c r="O13" s="16">
+        <v>10</v>
+      </c>
+      <c r="P13" s="16"/>
+      <c r="Q13" s="16"/>
+    </row>
+    <row r="14" spans="2:17" ht="18.75">
+      <c r="B14" s="16">
         <v>11</v>
       </c>
-      <c r="C14" s="24">
+      <c r="C14" s="16">
         <v>38323</v>
       </c>
-      <c r="D14" s="24">
+      <c r="D14" s="16">
         <v>7985</v>
       </c>
-    </row>
-    <row r="15" spans="2:5" ht="17.850000000000001" x14ac:dyDescent="0.25">
-      <c r="B15" s="23">
+      <c r="O14" s="16">
+        <v>11</v>
+      </c>
+      <c r="P14" s="16"/>
+      <c r="Q14" s="16"/>
+    </row>
+    <row r="15" spans="2:17" ht="18.75">
+      <c r="B15" s="15">
         <v>12</v>
       </c>
-      <c r="C15" s="36">
+      <c r="C15" s="26">
         <v>40896</v>
       </c>
-      <c r="D15" s="28">
+      <c r="D15" s="19">
         <v>8411</v>
       </c>
-    </row>
-    <row r="16" spans="2:5" ht="17.850000000000001" x14ac:dyDescent="0.25">
-      <c r="B16" s="24">
+      <c r="O15" s="15">
+        <v>12</v>
+      </c>
+      <c r="P15" s="26"/>
+      <c r="Q15" s="19"/>
+    </row>
+    <row r="16" spans="2:17" ht="18.75">
+      <c r="B16" s="16">
         <v>13</v>
       </c>
-      <c r="C16" s="24">
+      <c r="C16" s="16">
         <v>38132</v>
       </c>
-      <c r="D16" s="24">
+      <c r="D16" s="16">
         <v>8314</v>
       </c>
-    </row>
-    <row r="17" spans="2:4" ht="17.850000000000001" x14ac:dyDescent="0.25">
-      <c r="B17" s="24">
+      <c r="O16" s="16">
+        <v>13</v>
+      </c>
+      <c r="P16" s="16"/>
+      <c r="Q16" s="16"/>
+    </row>
+    <row r="17" spans="2:17" ht="18.75">
+      <c r="B17" s="16">
         <v>14</v>
       </c>
-      <c r="C17" s="24">
+      <c r="C17" s="16">
         <v>38962</v>
       </c>
-      <c r="D17" s="24">
+      <c r="D17" s="16">
         <v>8287</v>
       </c>
-    </row>
-    <row r="18" spans="2:4" ht="17.850000000000001" x14ac:dyDescent="0.25">
-      <c r="B18" s="24">
+      <c r="O17" s="16">
+        <v>14</v>
+      </c>
+      <c r="P17" s="16"/>
+      <c r="Q17" s="16"/>
+    </row>
+    <row r="18" spans="2:17" ht="18.75">
+      <c r="B18" s="16">
         <v>15</v>
       </c>
-      <c r="C18" s="24">
+      <c r="C18" s="16">
         <v>38825</v>
       </c>
-      <c r="D18" s="24">
+      <c r="D18" s="16">
         <v>8452</v>
       </c>
-    </row>
-    <row r="19" spans="2:4" ht="17.850000000000001" x14ac:dyDescent="0.25">
-      <c r="B19" s="23">
+      <c r="O18" s="16">
+        <v>15</v>
+      </c>
+      <c r="P18" s="16"/>
+      <c r="Q18" s="16"/>
+    </row>
+    <row r="19" spans="2:17" ht="18.75">
+      <c r="B19" s="15">
         <v>16</v>
       </c>
-      <c r="C19" s="36">
+      <c r="C19" s="26">
         <v>39364</v>
       </c>
-      <c r="D19" s="28">
+      <c r="D19" s="19">
         <v>7844</v>
       </c>
-    </row>
-    <row r="20" spans="2:4" ht="17.850000000000001" x14ac:dyDescent="0.2">
-      <c r="C20" s="40">
+      <c r="O19" s="15">
+        <v>16</v>
+      </c>
+      <c r="P19" s="26"/>
+      <c r="Q19" s="19"/>
+    </row>
+    <row r="20" spans="2:17" ht="18">
+      <c r="C20" s="27">
         <v>4</v>
       </c>
-      <c r="D20" s="40">
+      <c r="D20" s="27">
         <v>7</v>
       </c>
     </row>
-    <row r="24" spans="2:4" ht="17.850000000000001" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:17" ht="18">
       <c r="B24" s="1" t="s">
         <v>81</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="C2:D2"/>
+    <mergeCell ref="P2:Q2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Added statistics for block version.
</commit_message>
<xml_diff>
--- a/DecompositionLU/docs/statistics.xlsx
+++ b/DecompositionLU/docs/statistics.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Maxim\source\repos\practice\SECOND_COURSE\FOR_ITLAB\ArchBenchs\DecompositionLU\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F28F07AA-7477-46AC-9E9D-97388D1E91EE}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F99DBD33-6294-41FD-B06B-01AC3F0208A9}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-114" yWindow="-114" windowWidth="27602" windowHeight="15027" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-114" yWindow="-114" windowWidth="27602" windowHeight="15027" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Таблица" sheetId="1" r:id="rId1"/>
     <sheet name="Графики" sheetId="2" r:id="rId2"/>
+    <sheet name="Про процессор" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="124519"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="94">
   <si>
     <t>Я не уверен, будет ли это использоваться в готовой презентации и так ли это надо делать, если да, так что пока считаем, что файл для личного пользования.</t>
   </si>
@@ -342,14 +343,47 @@
     <t>Я искренне не понимаю этих результатов</t>
   </si>
   <si>
-    <t>Тесты были на машине с числом физ ядер - 6 и лог ядер - 12</t>
+    <t>Версия 3.0 (блочная версия алгоритма)</t>
+  </si>
+  <si>
+    <t>Хотя бы здесь логично</t>
+  </si>
+  <si>
+    <t>Замеры версии 2.0</t>
+  </si>
+  <si>
+    <t>Замеры на ноутбуке, данные процессора на вкладке "про процессор"</t>
+  </si>
+  <si>
+    <t>Комментарии:</t>
+  </si>
+  <si>
+    <t>Замеры на учебном компьютере, число физ ядер - 6 и лог ядер - 12</t>
+  </si>
+  <si>
+    <t>Функция плохо распараллеливается больше чем на 4 потока</t>
+  </si>
+  <si>
+    <t>Замеры версии 3.0</t>
+  </si>
+  <si>
+    <t>Соотв. таблица</t>
+  </si>
+  <si>
+    <t>Соотв. графики</t>
+  </si>
+  <si>
+    <t>Соотв. Графики</t>
+  </si>
+  <si>
+    <t>Мне нравится</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -451,8 +485,16 @@
       <family val="2"/>
       <charset val="204"/>
     </font>
+    <font>
+      <i/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="GOST Common"/>
+      <family val="2"/>
+      <charset val="204"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -471,8 +513,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="9">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -578,11 +632,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
@@ -617,14 +680,8 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
@@ -644,17 +701,17 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -692,6 +749,44 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -793,12 +888,45 @@
               <a:effectLst/>
             </c:spPr>
           </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>Графики!$B$4:$B$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>16</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Графики!$C$4:$C$19</c:f>
+              <c:f>Графики!$C$4:$C$11</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="16"/>
+                <c:ptCount val="8"/>
                 <c:pt idx="0">
                   <c:v>40525</c:v>
                 </c:pt>
@@ -806,45 +934,21 @@
                   <c:v>40933</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>35748</c:v>
+                  <c:v>34657</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>34657</c:v>
+                  <c:v>38071</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>36335</c:v>
+                  <c:v>37594</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>38071</c:v>
+                  <c:v>36931</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>36151</c:v>
+                  <c:v>40896</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>37594</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>36727</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>36931</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>38323</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>40896</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>38132</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>38962</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>38825</c:v>
-                </c:pt>
-                <c:pt idx="15">
                   <c:v>39364</c:v>
                 </c:pt>
               </c:numCache>
@@ -853,7 +957,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-DFDA-4FBA-8E35-21ED64A1AC56}"/>
+              <c16:uniqueId val="{00000000-2BAF-4570-BC3E-1CD3E98D98FB}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -877,6 +981,7 @@
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1038,6 +1143,407 @@
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0"/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1400" b="0"/>
+              <a:t>n = 3000</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="FF0000"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>Графики!$B$15:$B$21</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>12</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Графики!$D$15:$D$21</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>4557</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3948</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3448</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3554</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>3538</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>3696</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>4272</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-BEB4-4AD3-9B18-79E032C5B9F9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:marker val="1"/>
+        <c:smooth val="0"/>
+        <c:axId val="128556416"/>
+        <c:axId val="142235520"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="128556416"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="142235520"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="142235520"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:min val="3250"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="128556416"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+        <c:majorUnit val="250"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr>
+          <a:latin typeface="GOST Common" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+        </a:defRPr>
+      </a:pPr>
+      <a:endParaRPr lang="ru-RU"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75000000000000011" l="0.70000000000000007" r="0.70000000000000007" t="0.75000000000000011" header="0.30000000000000004" footer="0.30000000000000004"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="ru-RU"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0"/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1400" b="0"/>
+              <a:t>n = 5000</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="FF0000"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>Графики!$B$15:$B$21</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>12</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Графики!$C$15:$C$21</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>21978</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>18990</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>18915</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>19263</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>19123</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>19536</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>20535</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-E356-49E0-978B-AE57A6813BB1}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:marker val="1"/>
+        <c:smooth val="0"/>
+        <c:axId val="130061824"/>
+        <c:axId val="130781568"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="130061824"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="130781568"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="130781568"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:min val="18500"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="130061824"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr>
+          <a:latin typeface="GOST Common" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+        </a:defRPr>
+      </a:pPr>
+      <a:endParaRPr lang="ru-RU"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75000000000000033" l="0.70000000000000029" r="0.70000000000000029" t="0.75000000000000033" header="0.30000000000000016" footer="0.30000000000000016"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="ru-RU"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
       <c14:style val="108"/>
     </mc:Choice>
     <mc:Fallback>
@@ -1113,12 +1619,45 @@
               <a:effectLst/>
             </c:spPr>
           </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>Графики!$B$4:$B$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>16</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Графики!$D$4:$D$19</c:f>
+              <c:f>Графики!$D$4:$D$11</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="16"/>
+                <c:ptCount val="8"/>
                 <c:pt idx="0">
                   <c:v>8737</c:v>
                 </c:pt>
@@ -1126,45 +1665,21 @@
                   <c:v>8116</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>8005</c:v>
+                  <c:v>7387</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>7387</c:v>
+                  <c:v>7472</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>6863</c:v>
+                  <c:v>7389</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>7472</c:v>
+                  <c:v>8155</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>6861</c:v>
+                  <c:v>8411</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>7389</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>7908</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>8155</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>7985</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>8411</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>8314</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>8287</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>8452</c:v>
-                </c:pt>
-                <c:pt idx="15">
                   <c:v>7844</c:v>
                 </c:pt>
               </c:numCache>
@@ -1173,7 +1688,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-8747-4A5E-85F4-772AAE4EC689}"/>
+              <c16:uniqueId val="{00000000-6156-4052-AC80-4496F909B3BD}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1197,6 +1712,7 @@
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1244,7 +1760,648 @@
         <c:axId val="141687040"/>
         <c:scaling>
           <c:orientation val="minMax"/>
-          <c:min val="6500"/>
+          <c:min val="7250"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="GOST Common" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="ru-RU"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="141685504"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+        <c:majorUnit val="250"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr>
+          <a:latin typeface="GOST Common" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+        </a:defRPr>
+      </a:pPr>
+      <a:endParaRPr lang="ru-RU"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75000000000000022" l="0.70000000000000018" r="0.70000000000000018" t="0.75000000000000022" header="0.3000000000000001" footer="0.3000000000000001"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="ru-RU"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="104"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="4"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="GOST Common" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>n = 5000</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>Графики!$B$4:$B$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>16</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Графики!$C$27:$C$34</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>84305</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>42965</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>23077</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>18001</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>14258</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>12636</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>11424</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>9939</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-DA14-44C0-8EE4-78CA089A0DB1}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:marker val="1"/>
+        <c:smooth val="0"/>
+        <c:axId val="141630848"/>
+        <c:axId val="141640832"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="141630848"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="GOST Common" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="ru-RU"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="141640832"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="141640832"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="GOST Common" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="ru-RU"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="141630848"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr>
+          <a:latin typeface="GOST Common" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+        </a:defRPr>
+      </a:pPr>
+      <a:endParaRPr lang="ru-RU"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75000000000000022" l="0.70000000000000018" r="0.70000000000000018" t="0.75000000000000022" header="0.3000000000000001" footer="0.3000000000000001"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="ru-RU"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="108"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="8"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="GOST Common" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>n = 3000</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent6"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent6"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>Графики!$B$4:$B$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>16</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Графики!$D$27:$D$34</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>17805</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>9403</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4920</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4044</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>3317</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2987</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2738</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>2487</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-4C4E-49A3-9476-E67D282226BE}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:marker val="1"/>
+        <c:smooth val="0"/>
+        <c:axId val="141685504"/>
+        <c:axId val="141687040"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="141685504"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="GOST Common" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="ru-RU"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="141687040"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="141687040"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
@@ -1346,344 +2503,6 @@
   <c:printSettings>
     <c:headerFooter/>
     <c:pageMargins b="0.75000000000000022" l="0.70000000000000018" r="0.70000000000000018" t="0.75000000000000022" header="0.3000000000000001" footer="0.3000000000000001"/>
-    <c:pageSetup/>
-  </c:printSettings>
-</c:chartSpace>
-</file>
-
-<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
-  <c:date1904 val="0"/>
-  <c:lang val="ru-RU"/>
-  <c:roundedCorners val="0"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
-      <c14:style val="102"/>
-    </mc:Choice>
-    <mc:Fallback>
-      <c:style val="2"/>
-    </mc:Fallback>
-  </mc:AlternateContent>
-  <c:chart>
-    <c:autoTitleDeleted val="0"/>
-    <c:plotArea>
-      <c:layout/>
-      <c:lineChart>
-        <c:grouping val="standard"/>
-        <c:varyColors val="0"/>
-        <c:ser>
-          <c:idx val="0"/>
-          <c:order val="0"/>
-          <c:spPr>
-            <a:ln>
-              <a:solidFill>
-                <a:srgbClr val="FF0000"/>
-              </a:solidFill>
-            </a:ln>
-          </c:spPr>
-          <c:marker>
-            <c:spPr>
-              <a:solidFill>
-                <a:srgbClr val="FF0000"/>
-              </a:solidFill>
-              <a:ln>
-                <a:solidFill>
-                  <a:srgbClr val="FF0000"/>
-                </a:solidFill>
-              </a:ln>
-            </c:spPr>
-          </c:marker>
-          <c:cat>
-            <c:numRef>
-              <c:f>Графики!$O$4:$O$10</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="7"/>
-                <c:pt idx="0">
-                  <c:v>1</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>2</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>4</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>6</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>8</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>10</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>12</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>Графики!$Q$4:$Q$10</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="7"/>
-                <c:pt idx="0">
-                  <c:v>4557</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>3948</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>3448</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>3554</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>3538</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>3696</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>4272</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-6F6D-4B42-88DB-CFE117E40602}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:dLbls>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-        </c:dLbls>
-        <c:marker val="1"/>
-        <c:smooth val="0"/>
-        <c:axId val="128556416"/>
-        <c:axId val="142235520"/>
-      </c:lineChart>
-      <c:catAx>
-        <c:axId val="128556416"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="b"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="out"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="142235520"/>
-        <c:crosses val="autoZero"/>
-        <c:auto val="1"/>
-        <c:lblAlgn val="ctr"/>
-        <c:lblOffset val="100"/>
-        <c:noMultiLvlLbl val="0"/>
-      </c:catAx>
-      <c:valAx>
-        <c:axId val="142235520"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:majorGridlines/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="out"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="128556416"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="between"/>
-      </c:valAx>
-    </c:plotArea>
-    <c:plotVisOnly val="1"/>
-    <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
-  </c:chart>
-  <c:printSettings>
-    <c:headerFooter/>
-    <c:pageMargins b="0.75000000000000011" l="0.70000000000000007" r="0.70000000000000007" t="0.75000000000000011" header="0.30000000000000004" footer="0.30000000000000004"/>
-    <c:pageSetup/>
-  </c:printSettings>
-</c:chartSpace>
-</file>
-
-<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
-  <c:date1904 val="0"/>
-  <c:lang val="ru-RU"/>
-  <c:roundedCorners val="0"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
-      <c14:style val="102"/>
-    </mc:Choice>
-    <mc:Fallback>
-      <c:style val="2"/>
-    </mc:Fallback>
-  </mc:AlternateContent>
-  <c:chart>
-    <c:autoTitleDeleted val="0"/>
-    <c:plotArea>
-      <c:layout/>
-      <c:lineChart>
-        <c:grouping val="standard"/>
-        <c:varyColors val="0"/>
-        <c:ser>
-          <c:idx val="0"/>
-          <c:order val="0"/>
-          <c:spPr>
-            <a:ln>
-              <a:solidFill>
-                <a:srgbClr val="FF0000"/>
-              </a:solidFill>
-            </a:ln>
-          </c:spPr>
-          <c:marker>
-            <c:spPr>
-              <a:solidFill>
-                <a:srgbClr val="FF0000"/>
-              </a:solidFill>
-              <a:ln>
-                <a:solidFill>
-                  <a:srgbClr val="FF0000"/>
-                </a:solidFill>
-              </a:ln>
-            </c:spPr>
-          </c:marker>
-          <c:cat>
-            <c:numRef>
-              <c:f>Графики!$O$4:$O$10</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="7"/>
-                <c:pt idx="0">
-                  <c:v>1</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>2</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>4</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>6</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>8</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>10</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>12</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>Графики!$P$4:$P$10</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="7"/>
-                <c:pt idx="0">
-                  <c:v>21978</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>18990</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>18915</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>19263</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>19123</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>19536</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>20535</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-052C-4765-B247-6AC6F5FF1439}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:dLbls>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-        </c:dLbls>
-        <c:marker val="1"/>
-        <c:smooth val="0"/>
-        <c:axId val="130061824"/>
-        <c:axId val="130781568"/>
-      </c:lineChart>
-      <c:catAx>
-        <c:axId val="130061824"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="b"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="out"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="130781568"/>
-        <c:crosses val="autoZero"/>
-        <c:auto val="1"/>
-        <c:lblAlgn val="ctr"/>
-        <c:lblOffset val="100"/>
-        <c:noMultiLvlLbl val="0"/>
-      </c:catAx>
-      <c:valAx>
-        <c:axId val="130781568"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:majorGridlines/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="out"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="130061824"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="between"/>
-      </c:valAx>
-    </c:plotArea>
-    <c:plotVisOnly val="1"/>
-    <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
-  </c:chart>
-  <c:printSettings>
-    <c:headerFooter/>
-    <c:pageMargins b="0.75000000000000033" l="0.70000000000000029" r="0.70000000000000029" t="0.75000000000000033" header="0.30000000000000016" footer="0.30000000000000016"/>
     <c:pageSetup/>
   </c:printSettings>
 </c:chartSpace>
@@ -1856,25 +2675,318 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:oneCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
+  <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>9</xdr:row>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>9054</xdr:colOff>
+      <xdr:row>51</xdr:row>
+      <xdr:rowOff>113168</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="65" cy="172227"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="7" name="TextBox 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{99E00BDC-B281-41DE-A145-891E1532423F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9252642" y="8713960"/>
+          <a:ext cx="65" cy="172227"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="t">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:endParaRPr lang="ru-RU" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>1</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>474897</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>66375</xdr:rowOff>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>887241</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>253497</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="11" name="Диаграмма 10">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E443F810-5600-4C30-9DCC-5AD5631F4F58}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>869133</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="12" name="Диаграмма 11">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CF924618-0EBE-45C7-9FEC-B38948D0143F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>860080</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>235390</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="14" name="Диаграмма 13">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C244D70C-7C69-4FEE-AC69-87AAB93ABCB6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>887239</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>244519</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="15" name="Диаграмма 14">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{62D131ED-68EE-4A0F-9CBC-7D599203312A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>887241</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>253497</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="16" name="Диаграмма 15">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9834E67B-593D-4CC3-84B5-CB678D7E053C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>887239</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>244519</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="17" name="Диаграмма 16">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B83444C0-C37D-421E-91A4-54A85174FBA9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>9053</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>465843</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>156910</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="Рисунок 4">
+        <xdr:cNvPr id="2" name="Рисунок 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BCB4897C-D529-49E0-9F69-9210738BDAF8}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{77F3D0DE-7688-4F41-B6B2-A8862A31AAEF}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1890,7 +3002,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="11516008" y="2037030"/>
+          <a:off x="9053" y="0"/>
           <a:ext cx="6251008" cy="1424395"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1902,23 +3014,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>6</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>36214</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>446456</xdr:colOff>
-      <xdr:row>38</xdr:row>
-      <xdr:rowOff>182892</xdr:rowOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>428349</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>128571</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="6" name="Рисунок 5">
+        <xdr:cNvPr id="3" name="Рисунок 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BC18F56D-86EB-4BFF-98EC-5332254432C5}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8AF8B7F6-D74A-4CDC-B0AF-980BCBE244CF}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1934,7 +3046,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="11516008" y="3621386"/>
+          <a:off x="0" y="1484768"/>
           <a:ext cx="5643145" cy="5162298"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1942,155 +3054,6 @@
         </a:prstGeom>
       </xdr:spPr>
     </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>9052</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>13579</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>525100</xdr:colOff>
-      <xdr:row>13</xdr:row>
-      <xdr:rowOff>40739</xdr:rowOff>
-    </xdr:to>
-    <xdr:graphicFrame macro="">
-      <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="5" name="Диаграмма 4">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000005000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvGraphicFramePr/>
-      </xdr:nvGraphicFramePr>
-      <xdr:xfrm>
-        <a:off x="0" y="0"/>
-        <a:ext cx="0" cy="0"/>
-      </xdr:xfrm>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </xdr:graphicFrame>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>9052</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>13579</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>525100</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>176542</xdr:rowOff>
-    </xdr:to>
-    <xdr:graphicFrame macro="">
-      <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="7" name="Диаграмма 6">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000007000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvGraphicFramePr/>
-      </xdr:nvGraphicFramePr>
-      <xdr:xfrm>
-        <a:off x="0" y="0"/>
-        <a:ext cx="0" cy="0"/>
-      </xdr:xfrm>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
-        </a:graphicData>
-      </a:graphic>
-    </xdr:graphicFrame>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>247650</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>133350</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>25</xdr:col>
-      <xdr:colOff>552450</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>28575</xdr:rowOff>
-    </xdr:to>
-    <xdr:graphicFrame macro="">
-      <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="8" name="Диаграмма 7">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000008000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvGraphicFramePr/>
-      </xdr:nvGraphicFramePr>
-      <xdr:xfrm>
-        <a:off x="0" y="0"/>
-        <a:ext cx="0" cy="0"/>
-      </xdr:xfrm>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
-        </a:graphicData>
-      </a:graphic>
-    </xdr:graphicFrame>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>257175</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>142875</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>38100</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>152400</xdr:rowOff>
-    </xdr:to>
-    <xdr:graphicFrame macro="">
-      <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="6" name="Диаграмма 5">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000006000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvGraphicFramePr/>
-      </xdr:nvGraphicFramePr>
-      <xdr:xfrm>
-        <a:off x="0" y="0"/>
-        <a:ext cx="0" cy="0"/>
-      </xdr:xfrm>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
-        </a:graphicData>
-      </a:graphic>
-    </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -2359,7 +3322,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:W42"/>
+  <dimension ref="A1:W55"/>
   <sheetFormatPr defaultRowHeight="17.850000000000001" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="65.7109375" style="1" customWidth="1"/>
@@ -2437,17 +3400,17 @@
       <c r="N3" s="6"/>
     </row>
     <row r="5" spans="1:23" ht="17.850000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="38" t="s">
+      <c r="A5" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="39"/>
-      <c r="C5" s="39"/>
-      <c r="D5" s="39"/>
-      <c r="E5" s="40"/>
-      <c r="G5" s="33" t="s">
+      <c r="B5" s="37"/>
+      <c r="C5" s="37"/>
+      <c r="D5" s="37"/>
+      <c r="E5" s="38"/>
+      <c r="G5" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="H5" s="33"/>
+      <c r="H5" s="31"/>
       <c r="S5" s="5"/>
       <c r="T5" s="14"/>
       <c r="U5" s="14"/>
@@ -2458,14 +3421,14 @@
       <c r="A6" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="36" t="s">
+      <c r="B6" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="36"/>
-      <c r="D6" s="36"/>
-      <c r="E6" s="36"/>
-      <c r="G6" s="33"/>
-      <c r="H6" s="33"/>
+      <c r="C6" s="34"/>
+      <c r="D6" s="34"/>
+      <c r="E6" s="34"/>
+      <c r="G6" s="31"/>
+      <c r="H6" s="31"/>
       <c r="S6" s="14"/>
       <c r="T6" s="14"/>
       <c r="U6" s="14"/>
@@ -2488,8 +3451,8 @@
       <c r="E7" s="8">
         <v>10000</v>
       </c>
-      <c r="G7" s="33"/>
-      <c r="H7" s="33"/>
+      <c r="G7" s="31"/>
+      <c r="H7" s="31"/>
       <c r="S7" s="14"/>
       <c r="T7" s="14"/>
       <c r="U7" s="14"/>
@@ -2497,15 +3460,15 @@
       <c r="W7" s="14"/>
     </row>
     <row r="8" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A8" s="37" t="s">
+      <c r="A8" s="35" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="37"/>
-      <c r="C8" s="37"/>
-      <c r="D8" s="37"/>
-      <c r="E8" s="37"/>
-      <c r="G8" s="33"/>
-      <c r="H8" s="33"/>
+      <c r="B8" s="35"/>
+      <c r="C8" s="35"/>
+      <c r="D8" s="35"/>
+      <c r="E8" s="35"/>
+      <c r="G8" s="31"/>
+      <c r="H8" s="31"/>
       <c r="S8" s="14"/>
       <c r="T8" s="14"/>
       <c r="U8" s="14"/>
@@ -2581,13 +3544,13 @@
       <c r="W11" s="5"/>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A12" s="37" t="s">
+      <c r="A12" s="35" t="s">
         <v>12</v>
       </c>
-      <c r="B12" s="37"/>
-      <c r="C12" s="37"/>
-      <c r="D12" s="37"/>
-      <c r="E12" s="37"/>
+      <c r="B12" s="35"/>
+      <c r="C12" s="35"/>
+      <c r="D12" s="35"/>
+      <c r="E12" s="35"/>
       <c r="F12" s="5"/>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.25">
@@ -2600,7 +3563,7 @@
       <c r="C13" s="10">
         <v>232</v>
       </c>
-      <c r="D13" s="41" t="s">
+      <c r="D13" s="39" t="s">
         <v>21</v>
       </c>
       <c r="E13" s="10">
@@ -2618,7 +3581,7 @@
       <c r="C14" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="D14" s="42"/>
+      <c r="D14" s="40"/>
       <c r="E14" s="10" t="s">
         <v>10</v>
       </c>
@@ -2636,30 +3599,30 @@
       <c r="C15" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="D15" s="43"/>
+      <c r="D15" s="41"/>
       <c r="E15" s="10" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A18" s="35" t="s">
+      <c r="A18" s="33" t="s">
         <v>32</v>
       </c>
-      <c r="B18" s="35"/>
-      <c r="C18" s="35"/>
-      <c r="D18" s="35"/>
-      <c r="E18" s="35"/>
+      <c r="B18" s="33"/>
+      <c r="C18" s="33"/>
+      <c r="D18" s="33"/>
+      <c r="E18" s="33"/>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B19" s="36" t="s">
+      <c r="B19" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="C19" s="36"/>
-      <c r="D19" s="36"/>
-      <c r="E19" s="36"/>
+      <c r="C19" s="34"/>
+      <c r="D19" s="34"/>
+      <c r="E19" s="34"/>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
@@ -2679,13 +3642,13 @@
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A21" s="37" t="s">
+      <c r="A21" s="35" t="s">
         <v>11</v>
       </c>
-      <c r="B21" s="37"/>
-      <c r="C21" s="37"/>
-      <c r="D21" s="37"/>
-      <c r="E21" s="37"/>
+      <c r="B21" s="35"/>
+      <c r="C21" s="35"/>
+      <c r="D21" s="35"/>
+      <c r="E21" s="35"/>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
@@ -2737,21 +3700,21 @@
       <c r="E24" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="G24" s="20"/>
-      <c r="H24" s="32"/>
-      <c r="I24" s="32"/>
+      <c r="G24" s="18"/>
+      <c r="H24" s="30"/>
+      <c r="I24" s="30"/>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" s="37" t="s">
+      <c r="A25" s="35" t="s">
         <v>12</v>
       </c>
-      <c r="B25" s="37"/>
-      <c r="C25" s="37"/>
-      <c r="D25" s="37"/>
-      <c r="E25" s="37"/>
-      <c r="G25" s="21"/>
-      <c r="H25" s="18"/>
-      <c r="I25" s="18"/>
+      <c r="B25" s="35"/>
+      <c r="C25" s="35"/>
+      <c r="D25" s="35"/>
+      <c r="E25" s="35"/>
+      <c r="G25" s="19"/>
+      <c r="H25" s="17"/>
+      <c r="I25" s="17"/>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
@@ -2769,9 +3732,9 @@
       <c r="E26" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="G26" s="22"/>
-      <c r="H26" s="23"/>
-      <c r="I26" s="24"/>
+      <c r="G26" s="20"/>
+      <c r="H26" s="21"/>
+      <c r="I26" s="22"/>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
@@ -2789,9 +3752,9 @@
       <c r="E27" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="G27" s="22"/>
-      <c r="H27" s="23"/>
-      <c r="I27" s="20"/>
+      <c r="G27" s="20"/>
+      <c r="H27" s="21"/>
+      <c r="I27" s="18"/>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
@@ -2809,9 +3772,9 @@
       <c r="E28" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="G28" s="25"/>
-      <c r="H28" s="20"/>
-      <c r="I28" s="20"/>
+      <c r="G28" s="23"/>
+      <c r="H28" s="18"/>
+      <c r="I28" s="18"/>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="C29" s="1" t="s">
@@ -2823,40 +3786,44 @@
       <c r="E29" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="G29" s="22"/>
-      <c r="H29" s="23"/>
-      <c r="I29" s="20"/>
+      <c r="G29" s="20"/>
+      <c r="H29" s="21"/>
+      <c r="I29" s="18"/>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="G30" s="25"/>
-      <c r="H30" s="20"/>
-      <c r="I30" s="20"/>
+      <c r="G30" s="23"/>
+      <c r="H30" s="18"/>
+      <c r="I30" s="18"/>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A31" s="35" t="s">
+      <c r="A31" s="36" t="s">
         <v>70</v>
       </c>
-      <c r="B31" s="35"/>
-      <c r="C31" s="35"/>
-      <c r="D31" s="35"/>
-      <c r="E31" s="35"/>
-      <c r="G31" s="22"/>
-      <c r="H31" s="23"/>
-      <c r="I31" s="20"/>
+      <c r="B31" s="37"/>
+      <c r="C31" s="38"/>
+      <c r="D31" s="59" t="s">
+        <v>91</v>
+      </c>
+      <c r="E31" s="59" t="s">
+        <v>91</v>
+      </c>
+      <c r="G31" s="20"/>
+      <c r="H31" s="21"/>
+      <c r="I31" s="18"/>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B32" s="36" t="s">
+      <c r="B32" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="C32" s="36"/>
-      <c r="D32" s="36"/>
-      <c r="E32" s="36"/>
-      <c r="G32" s="25"/>
-      <c r="H32" s="20"/>
-      <c r="I32" s="20"/>
+      <c r="C32" s="34"/>
+      <c r="D32" s="34"/>
+      <c r="E32" s="34"/>
+      <c r="G32" s="23"/>
+      <c r="H32" s="18"/>
+      <c r="I32" s="18"/>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
@@ -2874,21 +3841,21 @@
       <c r="E33" s="8">
         <v>10000</v>
       </c>
-      <c r="G33" s="22"/>
-      <c r="H33" s="23"/>
-      <c r="I33" s="20"/>
+      <c r="G33" s="20"/>
+      <c r="H33" s="21"/>
+      <c r="I33" s="18"/>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A34" s="37" t="s">
+      <c r="A34" s="35" t="s">
         <v>11</v>
       </c>
-      <c r="B34" s="37"/>
-      <c r="C34" s="37"/>
-      <c r="D34" s="37"/>
-      <c r="E34" s="37"/>
-      <c r="G34" s="25"/>
-      <c r="H34" s="20"/>
-      <c r="I34" s="20"/>
+      <c r="B34" s="35"/>
+      <c r="C34" s="35"/>
+      <c r="D34" s="35"/>
+      <c r="E34" s="35"/>
+      <c r="G34" s="23"/>
+      <c r="H34" s="18"/>
+      <c r="I34" s="18"/>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
@@ -2906,9 +3873,9 @@
       <c r="E35" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="G35" s="25"/>
-      <c r="H35" s="20"/>
-      <c r="I35" s="20"/>
+      <c r="G35" s="23"/>
+      <c r="H35" s="18"/>
+      <c r="I35" s="18"/>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
@@ -2926,9 +3893,9 @@
       <c r="E36" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="G36" s="25"/>
-      <c r="H36" s="20"/>
-      <c r="I36" s="20"/>
+      <c r="G36" s="23"/>
+      <c r="H36" s="18"/>
+      <c r="I36" s="18"/>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
@@ -2946,21 +3913,21 @@
       <c r="E37" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="G37" s="22"/>
-      <c r="H37" s="23"/>
-      <c r="I37" s="20"/>
+      <c r="G37" s="20"/>
+      <c r="H37" s="21"/>
+      <c r="I37" s="18"/>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A38" s="37" t="s">
+      <c r="A38" s="35" t="s">
         <v>12</v>
       </c>
-      <c r="B38" s="37"/>
-      <c r="C38" s="37"/>
-      <c r="D38" s="37"/>
-      <c r="E38" s="37"/>
-      <c r="G38" s="25"/>
-      <c r="H38" s="20"/>
-      <c r="I38" s="20"/>
+      <c r="B38" s="35"/>
+      <c r="C38" s="35"/>
+      <c r="D38" s="35"/>
+      <c r="E38" s="35"/>
+      <c r="G38" s="23"/>
+      <c r="H38" s="18"/>
+      <c r="I38" s="18"/>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
@@ -2978,9 +3945,9 @@
       <c r="E39" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="G39" s="25"/>
-      <c r="H39" s="20"/>
-      <c r="I39" s="20"/>
+      <c r="G39" s="23"/>
+      <c r="H39" s="18"/>
+      <c r="I39" s="18"/>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
@@ -2998,9 +3965,9 @@
       <c r="E40" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="G40" s="25"/>
-      <c r="H40" s="20"/>
-      <c r="I40" s="20"/>
+      <c r="G40" s="23"/>
+      <c r="H40" s="18"/>
+      <c r="I40" s="18"/>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
@@ -3018,24 +3985,196 @@
       <c r="E41" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="G41" s="22"/>
-      <c r="H41" s="23"/>
-      <c r="I41" s="20"/>
+      <c r="G41" s="20"/>
+      <c r="H41" s="21"/>
+      <c r="I41" s="18"/>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B42" s="34" t="s">
+      <c r="B42" s="32" t="s">
         <v>66</v>
       </c>
-      <c r="C42" s="34"/>
-      <c r="D42" s="34"/>
-      <c r="E42" s="34"/>
+      <c r="C42" s="32"/>
+      <c r="D42" s="32"/>
+      <c r="E42" s="32"/>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A44" s="36" t="s">
+        <v>82</v>
+      </c>
+      <c r="B44" s="37"/>
+      <c r="C44" s="38"/>
+      <c r="D44" s="59" t="s">
+        <v>92</v>
+      </c>
+      <c r="E44" s="59" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A45" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B45" s="34" t="s">
+        <v>5</v>
+      </c>
+      <c r="C45" s="34"/>
+      <c r="D45" s="34"/>
+      <c r="E45" s="34"/>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A46" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B46" s="28">
+        <v>1000</v>
+      </c>
+      <c r="C46" s="28">
+        <v>3000</v>
+      </c>
+      <c r="D46" s="8">
+        <v>7000</v>
+      </c>
+      <c r="E46" s="8">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A47" s="35" t="s">
+        <v>11</v>
+      </c>
+      <c r="B47" s="35"/>
+      <c r="C47" s="35"/>
+      <c r="D47" s="35"/>
+      <c r="E47" s="35"/>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A48" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B48" s="9">
+        <v>16</v>
+      </c>
+      <c r="C48" s="10">
+        <v>123</v>
+      </c>
+      <c r="D48" s="10">
+        <v>378</v>
+      </c>
+      <c r="E48" s="10">
+        <v>1131</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A49" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B49" s="9">
+        <v>122</v>
+      </c>
+      <c r="C49" s="10">
+        <v>2103</v>
+      </c>
+      <c r="D49" s="10">
+        <v>26833</v>
+      </c>
+      <c r="E49" s="10">
+        <v>73485</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A50" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B50" s="9">
+        <v>139</v>
+      </c>
+      <c r="C50" s="10">
+        <v>2226</v>
+      </c>
+      <c r="D50" s="10">
+        <v>27211</v>
+      </c>
+      <c r="E50" s="10">
+        <v>74635</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A51" s="35" t="s">
+        <v>12</v>
+      </c>
+      <c r="B51" s="35"/>
+      <c r="C51" s="35"/>
+      <c r="D51" s="35"/>
+      <c r="E51" s="35"/>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A52" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B52" s="9">
+        <v>8</v>
+      </c>
+      <c r="C52" s="10">
+        <v>114</v>
+      </c>
+      <c r="D52" s="10">
+        <v>627</v>
+      </c>
+      <c r="E52" s="10">
+        <v>1285</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A53" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B53" s="9">
+        <v>145</v>
+      </c>
+      <c r="C53" s="10">
+        <v>6258</v>
+      </c>
+      <c r="D53" s="10">
+        <v>77559</v>
+      </c>
+      <c r="E53" s="10">
+        <v>224458</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A54" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B54" s="9">
+        <v>155</v>
+      </c>
+      <c r="C54" s="10">
+        <v>6373</v>
+      </c>
+      <c r="D54" s="10">
+        <v>78186</v>
+      </c>
+      <c r="E54" s="10">
+        <v>225744</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C55" s="1" t="s">
+        <v>83</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="16">
+  <mergeCells count="22">
+    <mergeCell ref="B45:E45"/>
+    <mergeCell ref="A47:E47"/>
+    <mergeCell ref="A51:E51"/>
+    <mergeCell ref="D44:E44"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="A44:C44"/>
+    <mergeCell ref="A31:C31"/>
     <mergeCell ref="H24:I24"/>
     <mergeCell ref="G5:H8"/>
     <mergeCell ref="B42:E42"/>
-    <mergeCell ref="A31:E31"/>
     <mergeCell ref="B32:E32"/>
     <mergeCell ref="A34:E34"/>
     <mergeCell ref="A38:E38"/>
@@ -3050,6 +4189,10 @@
     <mergeCell ref="A25:E25"/>
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="E31" location="Графики!A1" display="Соотв. графики" xr:uid="{B555E463-05C4-4E05-8D89-54A4D9AA7A6E}"/>
+    <hyperlink ref="E44" location="Графики!A24" display="Соотв. графики" xr:uid="{E92A20FD-A4FF-4EDF-8463-75004668F010}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
@@ -3058,337 +4201,920 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="B2:S24"/>
+  <dimension ref="A1:Z50"/>
   <sheetFormatPr defaultRowHeight="13.55" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="9.140625" style="29"/>
-    <col min="2" max="2" width="23.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="21.28515625" style="29" customWidth="1"/>
-    <col min="5" max="14" width="9.140625" style="29"/>
-    <col min="15" max="15" width="23" style="29" bestFit="1" customWidth="1"/>
-    <col min="16" max="17" width="15.28515625" style="29" customWidth="1"/>
-    <col min="18" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" width="15.28515625" style="26" customWidth="1"/>
+    <col min="2" max="2" width="28" style="26" customWidth="1"/>
+    <col min="3" max="3" width="23.5703125" style="26" customWidth="1"/>
+    <col min="4" max="4" width="21.42578125" style="26" customWidth="1"/>
+    <col min="5" max="17" width="14.28515625" style="26" customWidth="1"/>
+    <col min="18" max="16384" width="9.140625" style="26"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:19" ht="17.850000000000001" x14ac:dyDescent="0.25">
-      <c r="B2" s="17"/>
-      <c r="C2" s="44" t="s">
+    <row r="1" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="33" t="s">
+        <v>84</v>
+      </c>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+      <c r="G1" s="33"/>
+      <c r="H1" s="33"/>
+      <c r="I1" s="33"/>
+      <c r="J1" s="33"/>
+      <c r="K1" s="33"/>
+      <c r="L1" s="33"/>
+      <c r="M1" s="59" t="s">
+        <v>90</v>
+      </c>
+      <c r="N1" s="59"/>
+      <c r="O1" s="55"/>
+      <c r="P1" s="52"/>
+      <c r="Q1" s="52"/>
+      <c r="R1" s="52"/>
+      <c r="S1" s="52"/>
+      <c r="T1" s="52"/>
+      <c r="U1" s="52"/>
+      <c r="V1" s="52"/>
+      <c r="W1" s="52"/>
+      <c r="X1" s="52"/>
+      <c r="Y1" s="52"/>
+      <c r="Z1" s="52"/>
+    </row>
+    <row r="2" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="46" t="s">
+        <v>85</v>
+      </c>
+      <c r="B2" s="16"/>
+      <c r="C2" s="42" t="s">
         <v>78</v>
       </c>
-      <c r="D2" s="44"/>
-      <c r="O2" s="17"/>
-      <c r="P2" s="44" t="s">
-        <v>78</v>
-      </c>
-      <c r="Q2" s="44"/>
-      <c r="S2" s="29" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="3" spans="2:19" ht="17.850000000000001" x14ac:dyDescent="0.25">
-      <c r="B3" s="13" t="s">
+      <c r="D2" s="42"/>
+      <c r="E2" s="44"/>
+      <c r="F2" s="44"/>
+      <c r="G2" s="44"/>
+      <c r="H2" s="44"/>
+      <c r="I2" s="44"/>
+      <c r="J2" s="44"/>
+      <c r="K2" s="44"/>
+      <c r="L2" s="44"/>
+      <c r="M2" s="44"/>
+      <c r="N2" s="51"/>
+      <c r="O2" s="56"/>
+      <c r="P2" s="43"/>
+      <c r="Q2" s="43"/>
+      <c r="R2" s="43"/>
+      <c r="S2" s="43"/>
+      <c r="T2" s="43"/>
+      <c r="U2" s="43"/>
+      <c r="V2" s="43"/>
+      <c r="W2" s="43"/>
+      <c r="X2" s="43"/>
+      <c r="Y2" s="43"/>
+      <c r="Z2" s="43"/>
+    </row>
+    <row r="3" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="46"/>
+      <c r="B3" s="29" t="s">
         <v>77</v>
       </c>
-      <c r="C3" s="28" t="s">
+      <c r="C3" s="25" t="s">
         <v>79</v>
       </c>
-      <c r="D3" s="28" t="s">
+      <c r="D3" s="25" t="s">
         <v>80</v>
       </c>
-      <c r="O3" s="13" t="s">
-        <v>77</v>
-      </c>
-      <c r="P3" s="28" t="s">
-        <v>79</v>
-      </c>
-      <c r="Q3" s="28" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="4" spans="2:19" ht="17.850000000000001" x14ac:dyDescent="0.25">
+      <c r="E3" s="44"/>
+      <c r="F3" s="44"/>
+      <c r="G3" s="44"/>
+      <c r="H3" s="44"/>
+      <c r="I3" s="44"/>
+      <c r="J3" s="44"/>
+      <c r="K3" s="44"/>
+      <c r="L3" s="44"/>
+      <c r="M3" s="44"/>
+      <c r="N3" s="51"/>
+      <c r="O3" s="56"/>
+      <c r="P3" s="43"/>
+      <c r="Q3" s="43"/>
+      <c r="R3" s="43"/>
+      <c r="S3" s="43"/>
+      <c r="T3" s="43"/>
+      <c r="U3" s="43"/>
+      <c r="V3" s="43"/>
+      <c r="W3" s="43"/>
+      <c r="X3" s="43"/>
+      <c r="Y3" s="43"/>
+      <c r="Z3" s="43"/>
+    </row>
+    <row r="4" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="46"/>
       <c r="B4" s="15">
         <v>1</v>
       </c>
-      <c r="C4" s="26">
+      <c r="C4" s="24">
         <v>40525</v>
       </c>
-      <c r="D4" s="19">
+      <c r="D4" s="60">
         <v>8737</v>
       </c>
-      <c r="O4" s="15">
-        <v>1</v>
-      </c>
-      <c r="P4" s="19">
-        <v>21978</v>
-      </c>
-      <c r="Q4" s="19">
-        <v>4557</v>
-      </c>
-    </row>
-    <row r="5" spans="2:19" ht="17.850000000000001" x14ac:dyDescent="0.25">
+      <c r="E4" s="44"/>
+      <c r="F4" s="44"/>
+      <c r="G4" s="44"/>
+      <c r="H4" s="44"/>
+      <c r="I4" s="44"/>
+      <c r="J4" s="44"/>
+      <c r="K4" s="44"/>
+      <c r="L4" s="44"/>
+      <c r="M4" s="44"/>
+      <c r="N4" s="51"/>
+      <c r="O4" s="56"/>
+      <c r="P4" s="43"/>
+      <c r="Q4" s="43"/>
+      <c r="R4" s="43"/>
+      <c r="S4" s="43"/>
+      <c r="T4" s="43"/>
+      <c r="U4" s="43"/>
+      <c r="V4" s="43"/>
+      <c r="W4" s="43"/>
+      <c r="X4" s="43"/>
+      <c r="Y4" s="43"/>
+      <c r="Z4" s="43"/>
+    </row>
+    <row r="5" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="46"/>
       <c r="B5" s="15">
         <v>2</v>
       </c>
-      <c r="C5" s="26">
+      <c r="C5" s="24">
         <v>40933</v>
       </c>
-      <c r="D5" s="19">
+      <c r="D5" s="60">
         <v>8116</v>
       </c>
-      <c r="O5" s="15">
+      <c r="E5" s="44"/>
+      <c r="F5" s="44"/>
+      <c r="G5" s="44"/>
+      <c r="H5" s="44"/>
+      <c r="I5" s="44"/>
+      <c r="J5" s="44"/>
+      <c r="K5" s="44"/>
+      <c r="L5" s="44"/>
+      <c r="M5" s="44"/>
+      <c r="N5" s="51"/>
+      <c r="O5" s="56"/>
+      <c r="P5" s="43"/>
+      <c r="Q5" s="43"/>
+      <c r="R5" s="43"/>
+      <c r="S5" s="43"/>
+      <c r="T5" s="43"/>
+      <c r="U5" s="43"/>
+      <c r="V5" s="43"/>
+      <c r="W5" s="43"/>
+      <c r="X5" s="43"/>
+      <c r="Y5" s="43"/>
+      <c r="Z5" s="43"/>
+    </row>
+    <row r="6" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="46"/>
+      <c r="B6" s="15">
+        <v>4</v>
+      </c>
+      <c r="C6" s="24">
+        <v>34657</v>
+      </c>
+      <c r="D6" s="60">
+        <v>7387</v>
+      </c>
+      <c r="E6" s="44"/>
+      <c r="F6" s="44"/>
+      <c r="G6" s="44"/>
+      <c r="H6" s="44"/>
+      <c r="I6" s="44"/>
+      <c r="J6" s="44"/>
+      <c r="K6" s="44"/>
+      <c r="L6" s="44"/>
+      <c r="M6" s="44"/>
+      <c r="N6" s="51"/>
+      <c r="O6" s="57"/>
+    </row>
+    <row r="7" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="46"/>
+      <c r="B7" s="15">
+        <v>6</v>
+      </c>
+      <c r="C7" s="24">
+        <v>38071</v>
+      </c>
+      <c r="D7" s="60">
+        <v>7472</v>
+      </c>
+      <c r="E7" s="44"/>
+      <c r="F7" s="44"/>
+      <c r="G7" s="44"/>
+      <c r="H7" s="44"/>
+      <c r="I7" s="44"/>
+      <c r="J7" s="44"/>
+      <c r="K7" s="44"/>
+      <c r="L7" s="44"/>
+      <c r="M7" s="44"/>
+      <c r="N7" s="51"/>
+      <c r="O7" s="57"/>
+    </row>
+    <row r="8" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="46"/>
+      <c r="B8" s="15">
+        <v>8</v>
+      </c>
+      <c r="C8" s="24">
+        <v>37594</v>
+      </c>
+      <c r="D8" s="60">
+        <v>7389</v>
+      </c>
+      <c r="E8" s="44"/>
+      <c r="F8" s="44"/>
+      <c r="G8" s="44"/>
+      <c r="H8" s="44"/>
+      <c r="I8" s="44"/>
+      <c r="J8" s="44"/>
+      <c r="K8" s="44"/>
+      <c r="L8" s="44"/>
+      <c r="M8" s="44"/>
+      <c r="N8" s="51"/>
+      <c r="O8" s="57"/>
+    </row>
+    <row r="9" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="46"/>
+      <c r="B9" s="15">
+        <v>10</v>
+      </c>
+      <c r="C9" s="24">
+        <v>36931</v>
+      </c>
+      <c r="D9" s="60">
+        <v>8155</v>
+      </c>
+      <c r="E9" s="44"/>
+      <c r="F9" s="44"/>
+      <c r="G9" s="44"/>
+      <c r="H9" s="44"/>
+      <c r="I9" s="44"/>
+      <c r="J9" s="44"/>
+      <c r="K9" s="44"/>
+      <c r="L9" s="44"/>
+      <c r="M9" s="44"/>
+      <c r="N9" s="51"/>
+      <c r="O9" s="57"/>
+    </row>
+    <row r="10" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="46"/>
+      <c r="B10" s="15">
+        <v>12</v>
+      </c>
+      <c r="C10" s="24">
+        <v>40896</v>
+      </c>
+      <c r="D10" s="60">
+        <v>8411</v>
+      </c>
+      <c r="E10" s="44"/>
+      <c r="F10" s="44"/>
+      <c r="G10" s="44"/>
+      <c r="H10" s="44"/>
+      <c r="I10" s="44"/>
+      <c r="J10" s="44"/>
+      <c r="K10" s="44"/>
+      <c r="L10" s="44"/>
+      <c r="M10" s="44"/>
+      <c r="N10" s="51"/>
+      <c r="O10" s="57"/>
+    </row>
+    <row r="11" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="46"/>
+      <c r="B11" s="15">
+        <v>16</v>
+      </c>
+      <c r="C11" s="24">
+        <v>39364</v>
+      </c>
+      <c r="D11" s="60">
+        <v>7844</v>
+      </c>
+      <c r="E11" s="44"/>
+      <c r="F11" s="44"/>
+      <c r="G11" s="44"/>
+      <c r="H11" s="44"/>
+      <c r="I11" s="44"/>
+      <c r="J11" s="44"/>
+      <c r="K11" s="44"/>
+      <c r="L11" s="44"/>
+      <c r="M11" s="44"/>
+      <c r="N11" s="51"/>
+      <c r="O11" s="57"/>
+      <c r="P11" s="27"/>
+      <c r="Q11" s="27"/>
+    </row>
+    <row r="12" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="46"/>
+      <c r="B12" s="47" t="s">
+        <v>86</v>
+      </c>
+      <c r="C12" s="48" t="s">
+        <v>81</v>
+      </c>
+      <c r="D12" s="48"/>
+      <c r="E12" s="48"/>
+      <c r="F12" s="48"/>
+      <c r="G12" s="48"/>
+      <c r="H12" s="48"/>
+      <c r="I12" s="48"/>
+      <c r="J12" s="48"/>
+      <c r="K12" s="48"/>
+      <c r="L12" s="48"/>
+      <c r="M12" s="48"/>
+      <c r="N12" s="53"/>
+      <c r="O12" s="58"/>
+      <c r="P12" s="23"/>
+      <c r="Q12" s="23"/>
+    </row>
+    <row r="13" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="46" t="s">
+        <v>87</v>
+      </c>
+      <c r="B13" s="16"/>
+      <c r="C13" s="42" t="s">
+        <v>78</v>
+      </c>
+      <c r="D13" s="42"/>
+      <c r="E13" s="45"/>
+      <c r="F13" s="44"/>
+      <c r="G13" s="44"/>
+      <c r="H13" s="44"/>
+      <c r="I13" s="44"/>
+      <c r="J13" s="44"/>
+      <c r="K13" s="44"/>
+      <c r="L13" s="44"/>
+      <c r="M13" s="44"/>
+      <c r="N13" s="51"/>
+      <c r="O13" s="58"/>
+      <c r="P13" s="23"/>
+      <c r="Q13" s="23"/>
+    </row>
+    <row r="14" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="46"/>
+      <c r="B14" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="C14" s="25" t="s">
+        <v>79</v>
+      </c>
+      <c r="D14" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="E14" s="45"/>
+      <c r="F14" s="44"/>
+      <c r="G14" s="44"/>
+      <c r="H14" s="44"/>
+      <c r="I14" s="44"/>
+      <c r="J14" s="44"/>
+      <c r="K14" s="44"/>
+      <c r="L14" s="44"/>
+      <c r="M14" s="44"/>
+      <c r="N14" s="51"/>
+      <c r="O14" s="58"/>
+      <c r="P14" s="23"/>
+      <c r="Q14" s="23"/>
+    </row>
+    <row r="15" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="46"/>
+      <c r="B15" s="15">
+        <v>1</v>
+      </c>
+      <c r="C15" s="60">
+        <v>21978</v>
+      </c>
+      <c r="D15" s="60">
+        <v>4557</v>
+      </c>
+      <c r="E15" s="44"/>
+      <c r="F15" s="44"/>
+      <c r="G15" s="44"/>
+      <c r="H15" s="44"/>
+      <c r="I15" s="44"/>
+      <c r="J15" s="44"/>
+      <c r="K15" s="44"/>
+      <c r="L15" s="44"/>
+      <c r="M15" s="44"/>
+      <c r="N15" s="51"/>
+      <c r="O15" s="57"/>
+      <c r="P15" s="27"/>
+      <c r="Q15" s="27"/>
+    </row>
+    <row r="16" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="46"/>
+      <c r="B16" s="15">
         <v>2</v>
       </c>
-      <c r="P5" s="19">
+      <c r="C16" s="60">
         <v>18990</v>
       </c>
-      <c r="Q5" s="19">
+      <c r="D16" s="60">
         <v>3948</v>
       </c>
-    </row>
-    <row r="6" spans="2:19" ht="17.850000000000001" x14ac:dyDescent="0.25">
-      <c r="B6" s="16">
-        <v>3</v>
-      </c>
-      <c r="C6" s="16">
-        <v>35748</v>
-      </c>
-      <c r="D6" s="16">
-        <v>8005</v>
-      </c>
-      <c r="O6" s="15">
+      <c r="E16" s="44"/>
+      <c r="F16" s="44"/>
+      <c r="G16" s="44"/>
+      <c r="H16" s="44"/>
+      <c r="I16" s="44"/>
+      <c r="J16" s="44"/>
+      <c r="K16" s="44"/>
+      <c r="L16" s="44"/>
+      <c r="M16" s="44"/>
+      <c r="N16" s="51"/>
+      <c r="O16" s="58"/>
+      <c r="P16" s="23"/>
+      <c r="Q16" s="23"/>
+    </row>
+    <row r="17" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="46"/>
+      <c r="B17" s="15">
         <v>4</v>
       </c>
-      <c r="P6" s="19">
+      <c r="C17" s="60">
         <v>18915</v>
       </c>
-      <c r="Q6" s="19">
+      <c r="D17" s="60">
         <v>3448</v>
       </c>
-    </row>
-    <row r="7" spans="2:19" ht="17.850000000000001" x14ac:dyDescent="0.25">
-      <c r="B7" s="15">
+      <c r="E17" s="44"/>
+      <c r="F17" s="44"/>
+      <c r="G17" s="44"/>
+      <c r="H17" s="44"/>
+      <c r="I17" s="44"/>
+      <c r="J17" s="44"/>
+      <c r="K17" s="44"/>
+      <c r="L17" s="44"/>
+      <c r="M17" s="44"/>
+      <c r="N17" s="51"/>
+      <c r="O17" s="58"/>
+      <c r="P17" s="23"/>
+      <c r="Q17" s="23"/>
+    </row>
+    <row r="18" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="46"/>
+      <c r="B18" s="15">
+        <v>6</v>
+      </c>
+      <c r="C18" s="60">
+        <v>19263</v>
+      </c>
+      <c r="D18" s="60">
+        <v>3554</v>
+      </c>
+      <c r="E18" s="44"/>
+      <c r="F18" s="44"/>
+      <c r="G18" s="44"/>
+      <c r="H18" s="44"/>
+      <c r="I18" s="44"/>
+      <c r="J18" s="44"/>
+      <c r="K18" s="44"/>
+      <c r="L18" s="44"/>
+      <c r="M18" s="44"/>
+      <c r="N18" s="51"/>
+      <c r="O18" s="58"/>
+      <c r="P18" s="23"/>
+      <c r="Q18" s="23"/>
+    </row>
+    <row r="19" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="46"/>
+      <c r="B19" s="15">
+        <v>8</v>
+      </c>
+      <c r="C19" s="24">
+        <v>19123</v>
+      </c>
+      <c r="D19" s="60">
+        <v>3538</v>
+      </c>
+      <c r="E19" s="44"/>
+      <c r="F19" s="44"/>
+      <c r="G19" s="44"/>
+      <c r="H19" s="44"/>
+      <c r="I19" s="44"/>
+      <c r="J19" s="44"/>
+      <c r="K19" s="44"/>
+      <c r="L19" s="44"/>
+      <c r="M19" s="44"/>
+      <c r="N19" s="51"/>
+      <c r="O19" s="57"/>
+    </row>
+    <row r="20" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="46"/>
+      <c r="B20" s="15">
+        <v>10</v>
+      </c>
+      <c r="C20" s="24">
+        <v>19536</v>
+      </c>
+      <c r="D20" s="60">
+        <v>3696</v>
+      </c>
+      <c r="E20" s="44"/>
+      <c r="F20" s="44"/>
+      <c r="G20" s="44"/>
+      <c r="H20" s="44"/>
+      <c r="I20" s="44"/>
+      <c r="J20" s="44"/>
+      <c r="K20" s="44"/>
+      <c r="L20" s="44"/>
+      <c r="M20" s="44"/>
+      <c r="N20" s="51"/>
+      <c r="O20" s="57"/>
+    </row>
+    <row r="21" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="46"/>
+      <c r="B21" s="15">
+        <v>12</v>
+      </c>
+      <c r="C21" s="24">
+        <v>20535</v>
+      </c>
+      <c r="D21" s="60">
+        <v>4272</v>
+      </c>
+      <c r="E21" s="44"/>
+      <c r="F21" s="44"/>
+      <c r="G21" s="44"/>
+      <c r="H21" s="44"/>
+      <c r="I21" s="44"/>
+      <c r="J21" s="44"/>
+      <c r="K21" s="44"/>
+      <c r="L21" s="44"/>
+      <c r="M21" s="44"/>
+      <c r="N21" s="51"/>
+      <c r="O21" s="57"/>
+    </row>
+    <row r="22" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="46"/>
+      <c r="B22" s="49" t="s">
+        <v>86</v>
+      </c>
+      <c r="C22" s="50" t="s">
+        <v>88</v>
+      </c>
+      <c r="D22" s="50"/>
+      <c r="E22" s="50"/>
+      <c r="F22" s="50"/>
+      <c r="G22" s="50"/>
+      <c r="H22" s="50"/>
+      <c r="I22" s="50"/>
+      <c r="J22" s="50"/>
+      <c r="K22" s="50"/>
+      <c r="L22" s="50"/>
+      <c r="M22" s="50"/>
+      <c r="N22" s="54"/>
+      <c r="O22" s="57"/>
+    </row>
+    <row r="23" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="46"/>
+      <c r="B23" s="49"/>
+      <c r="C23" s="50"/>
+      <c r="D23" s="50"/>
+      <c r="E23" s="50"/>
+      <c r="F23" s="50"/>
+      <c r="G23" s="50"/>
+      <c r="H23" s="50"/>
+      <c r="I23" s="50"/>
+      <c r="J23" s="50"/>
+      <c r="K23" s="50"/>
+      <c r="L23" s="50"/>
+      <c r="M23" s="50"/>
+      <c r="N23" s="54"/>
+      <c r="O23" s="57"/>
+    </row>
+    <row r="24" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="33" t="s">
+        <v>89</v>
+      </c>
+      <c r="B24" s="33"/>
+      <c r="C24" s="33"/>
+      <c r="D24" s="33"/>
+      <c r="E24" s="33"/>
+      <c r="F24" s="33"/>
+      <c r="G24" s="33"/>
+      <c r="H24" s="33"/>
+      <c r="I24" s="33"/>
+      <c r="J24" s="33"/>
+      <c r="K24" s="33"/>
+      <c r="L24" s="33"/>
+      <c r="M24" s="59" t="s">
+        <v>90</v>
+      </c>
+      <c r="N24" s="59"/>
+      <c r="O24" s="57"/>
+    </row>
+    <row r="25" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="46" t="s">
+        <v>85</v>
+      </c>
+      <c r="B25" s="16"/>
+      <c r="C25" s="42" t="s">
+        <v>78</v>
+      </c>
+      <c r="D25" s="42"/>
+      <c r="E25" s="44"/>
+      <c r="F25" s="44"/>
+      <c r="G25" s="44"/>
+      <c r="H25" s="44"/>
+      <c r="I25" s="44"/>
+      <c r="J25" s="44"/>
+      <c r="K25" s="44"/>
+      <c r="L25" s="44"/>
+      <c r="M25" s="44"/>
+      <c r="N25" s="51"/>
+      <c r="O25" s="57"/>
+    </row>
+    <row r="26" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="46"/>
+      <c r="B26" s="29" t="s">
+        <v>77</v>
+      </c>
+      <c r="C26" s="25" t="s">
+        <v>79</v>
+      </c>
+      <c r="D26" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="E26" s="44"/>
+      <c r="F26" s="44"/>
+      <c r="G26" s="44"/>
+      <c r="H26" s="44"/>
+      <c r="I26" s="44"/>
+      <c r="J26" s="44"/>
+      <c r="K26" s="44"/>
+      <c r="L26" s="44"/>
+      <c r="M26" s="44"/>
+      <c r="N26" s="51"/>
+      <c r="O26" s="57"/>
+    </row>
+    <row r="27" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="46"/>
+      <c r="B27" s="15">
+        <v>1</v>
+      </c>
+      <c r="C27" s="24">
+        <v>84305</v>
+      </c>
+      <c r="D27" s="60">
+        <v>17805</v>
+      </c>
+      <c r="E27" s="44"/>
+      <c r="F27" s="44"/>
+      <c r="G27" s="44"/>
+      <c r="H27" s="44"/>
+      <c r="I27" s="44"/>
+      <c r="J27" s="44"/>
+      <c r="K27" s="44"/>
+      <c r="L27" s="44"/>
+      <c r="M27" s="44"/>
+      <c r="N27" s="51"/>
+      <c r="O27" s="57"/>
+    </row>
+    <row r="28" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="46"/>
+      <c r="B28" s="15">
+        <v>2</v>
+      </c>
+      <c r="C28" s="24">
+        <v>42965</v>
+      </c>
+      <c r="D28" s="60">
+        <v>9403</v>
+      </c>
+      <c r="E28" s="44"/>
+      <c r="F28" s="44"/>
+      <c r="G28" s="44"/>
+      <c r="H28" s="44"/>
+      <c r="I28" s="44"/>
+      <c r="J28" s="44"/>
+      <c r="K28" s="44"/>
+      <c r="L28" s="44"/>
+      <c r="M28" s="44"/>
+      <c r="N28" s="51"/>
+      <c r="O28" s="57"/>
+    </row>
+    <row r="29" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="46"/>
+      <c r="B29" s="15">
         <v>4</v>
       </c>
-      <c r="C7" s="26">
-        <v>34657</v>
-      </c>
-      <c r="D7" s="19">
-        <v>7387</v>
-      </c>
-      <c r="O7" s="15">
+      <c r="C29" s="24">
+        <v>23077</v>
+      </c>
+      <c r="D29" s="60">
+        <v>4920</v>
+      </c>
+      <c r="E29" s="44"/>
+      <c r="F29" s="44"/>
+      <c r="G29" s="44"/>
+      <c r="H29" s="44"/>
+      <c r="I29" s="44"/>
+      <c r="J29" s="44"/>
+      <c r="K29" s="44"/>
+      <c r="L29" s="44"/>
+      <c r="M29" s="44"/>
+      <c r="N29" s="51"/>
+      <c r="O29" s="57"/>
+    </row>
+    <row r="30" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="46"/>
+      <c r="B30" s="15">
         <v>6</v>
       </c>
-      <c r="P7" s="19">
-        <v>19263</v>
-      </c>
-      <c r="Q7" s="19">
-        <v>3554</v>
-      </c>
-    </row>
-    <row r="8" spans="2:19" ht="17.850000000000001" x14ac:dyDescent="0.25">
-      <c r="B8" s="16">
-        <v>5</v>
-      </c>
-      <c r="C8" s="16">
-        <v>36335</v>
-      </c>
-      <c r="D8" s="16">
-        <v>6863</v>
-      </c>
-      <c r="O8" s="15">
+      <c r="C30" s="24">
+        <v>18001</v>
+      </c>
+      <c r="D30" s="60">
+        <v>4044</v>
+      </c>
+      <c r="E30" s="44"/>
+      <c r="F30" s="44"/>
+      <c r="G30" s="44"/>
+      <c r="H30" s="44"/>
+      <c r="I30" s="44"/>
+      <c r="J30" s="44"/>
+      <c r="K30" s="44"/>
+      <c r="L30" s="44"/>
+      <c r="M30" s="44"/>
+      <c r="N30" s="51"/>
+      <c r="O30" s="57"/>
+    </row>
+    <row r="31" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="46"/>
+      <c r="B31" s="15">
         <v>8</v>
       </c>
-      <c r="P8" s="26">
-        <v>19123</v>
-      </c>
-      <c r="Q8" s="19">
-        <v>3538</v>
-      </c>
-    </row>
-    <row r="9" spans="2:19" ht="17.850000000000001" x14ac:dyDescent="0.25">
-      <c r="B9" s="15">
-        <v>6</v>
-      </c>
-      <c r="C9" s="26">
-        <v>38071</v>
-      </c>
-      <c r="D9" s="19">
-        <v>7472</v>
-      </c>
-      <c r="O9" s="15">
+      <c r="C31" s="24">
+        <v>14258</v>
+      </c>
+      <c r="D31" s="60">
+        <v>3317</v>
+      </c>
+      <c r="E31" s="44"/>
+      <c r="F31" s="44"/>
+      <c r="G31" s="44"/>
+      <c r="H31" s="44"/>
+      <c r="I31" s="44"/>
+      <c r="J31" s="44"/>
+      <c r="K31" s="44"/>
+      <c r="L31" s="44"/>
+      <c r="M31" s="44"/>
+      <c r="N31" s="51"/>
+      <c r="O31" s="57"/>
+    </row>
+    <row r="32" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="46"/>
+      <c r="B32" s="15">
         <v>10</v>
       </c>
-      <c r="P9" s="26">
-        <v>19536</v>
-      </c>
-      <c r="Q9" s="19">
-        <v>3696</v>
-      </c>
-    </row>
-    <row r="10" spans="2:19" ht="17.850000000000001" x14ac:dyDescent="0.25">
-      <c r="B10" s="16">
-        <v>7</v>
-      </c>
-      <c r="C10" s="16">
-        <v>36151</v>
-      </c>
-      <c r="D10" s="16">
-        <v>6861</v>
-      </c>
-      <c r="O10" s="15">
+      <c r="C32" s="24">
+        <v>12636</v>
+      </c>
+      <c r="D32" s="60">
+        <v>2987</v>
+      </c>
+      <c r="E32" s="44"/>
+      <c r="F32" s="44"/>
+      <c r="G32" s="44"/>
+      <c r="H32" s="44"/>
+      <c r="I32" s="44"/>
+      <c r="J32" s="44"/>
+      <c r="K32" s="44"/>
+      <c r="L32" s="44"/>
+      <c r="M32" s="44"/>
+      <c r="N32" s="51"/>
+      <c r="O32" s="57"/>
+    </row>
+    <row r="33" spans="1:15" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="46"/>
+      <c r="B33" s="15">
         <v>12</v>
       </c>
-      <c r="P10" s="26">
-        <v>20535</v>
-      </c>
-      <c r="Q10" s="19">
-        <v>4272</v>
-      </c>
-    </row>
-    <row r="11" spans="2:19" ht="17.850000000000001" x14ac:dyDescent="0.25">
-      <c r="B11" s="15">
-        <v>8</v>
-      </c>
-      <c r="C11" s="26">
-        <v>37594</v>
-      </c>
-      <c r="D11" s="19">
-        <v>7389</v>
-      </c>
-      <c r="O11" s="31"/>
-      <c r="P11" s="31"/>
-      <c r="Q11" s="31"/>
-    </row>
-    <row r="12" spans="2:19" ht="17.850000000000001" x14ac:dyDescent="0.25">
-      <c r="B12" s="16">
-        <v>9</v>
-      </c>
-      <c r="C12" s="16">
-        <v>36727</v>
-      </c>
-      <c r="D12" s="16">
-        <v>7908</v>
-      </c>
-      <c r="E12" s="30"/>
-      <c r="O12" s="25"/>
-      <c r="P12" s="25"/>
-      <c r="Q12" s="25"/>
-    </row>
-    <row r="13" spans="2:19" ht="17.850000000000001" x14ac:dyDescent="0.25">
-      <c r="B13" s="16">
-        <v>10</v>
-      </c>
-      <c r="C13" s="16">
-        <v>36931</v>
-      </c>
-      <c r="D13" s="16">
-        <v>8155</v>
-      </c>
-      <c r="O13" s="25"/>
-      <c r="P13" s="25"/>
-      <c r="Q13" s="25"/>
-    </row>
-    <row r="14" spans="2:19" ht="17.850000000000001" x14ac:dyDescent="0.25">
-      <c r="B14" s="16">
-        <v>11</v>
-      </c>
-      <c r="C14" s="16">
-        <v>38323</v>
-      </c>
-      <c r="D14" s="16">
-        <v>7985</v>
-      </c>
-      <c r="O14" s="25"/>
-      <c r="P14" s="25"/>
-      <c r="Q14" s="25"/>
-    </row>
-    <row r="15" spans="2:19" ht="17.850000000000001" x14ac:dyDescent="0.25">
-      <c r="B15" s="15">
-        <v>12</v>
-      </c>
-      <c r="C15" s="26">
-        <v>40896</v>
-      </c>
-      <c r="D15" s="19">
-        <v>8411</v>
-      </c>
-      <c r="O15" s="31"/>
-      <c r="P15" s="31"/>
-      <c r="Q15" s="31"/>
-    </row>
-    <row r="16" spans="2:19" ht="17.850000000000001" x14ac:dyDescent="0.25">
-      <c r="B16" s="16">
-        <v>13</v>
-      </c>
-      <c r="C16" s="16">
-        <v>38132</v>
-      </c>
-      <c r="D16" s="16">
-        <v>8314</v>
-      </c>
-      <c r="O16" s="25"/>
-      <c r="P16" s="25"/>
-      <c r="Q16" s="25"/>
-    </row>
-    <row r="17" spans="2:17" ht="17.850000000000001" x14ac:dyDescent="0.25">
-      <c r="B17" s="16">
-        <v>14</v>
-      </c>
-      <c r="C17" s="16">
-        <v>38962</v>
-      </c>
-      <c r="D17" s="16">
-        <v>8287</v>
-      </c>
-      <c r="O17" s="25"/>
-      <c r="P17" s="25"/>
-      <c r="Q17" s="25"/>
-    </row>
-    <row r="18" spans="2:17" ht="17.850000000000001" x14ac:dyDescent="0.25">
-      <c r="B18" s="16">
-        <v>15</v>
-      </c>
-      <c r="C18" s="16">
-        <v>38825</v>
-      </c>
-      <c r="D18" s="16">
-        <v>8452</v>
-      </c>
-      <c r="O18" s="25"/>
-      <c r="P18" s="25"/>
-      <c r="Q18" s="25"/>
-    </row>
-    <row r="19" spans="2:17" ht="17.850000000000001" x14ac:dyDescent="0.25">
-      <c r="B19" s="15">
+      <c r="C33" s="24">
+        <v>11424</v>
+      </c>
+      <c r="D33" s="60">
+        <v>2738</v>
+      </c>
+      <c r="E33" s="44"/>
+      <c r="F33" s="44"/>
+      <c r="G33" s="44"/>
+      <c r="H33" s="44"/>
+      <c r="I33" s="44"/>
+      <c r="J33" s="44"/>
+      <c r="K33" s="44"/>
+      <c r="L33" s="44"/>
+      <c r="M33" s="44"/>
+      <c r="N33" s="51"/>
+      <c r="O33" s="57"/>
+    </row>
+    <row r="34" spans="1:15" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="46"/>
+      <c r="B34" s="15">
         <v>16</v>
       </c>
-      <c r="C19" s="26">
-        <v>39364</v>
-      </c>
-      <c r="D19" s="19">
-        <v>7844</v>
-      </c>
-    </row>
-    <row r="20" spans="2:17" ht="17.850000000000001" x14ac:dyDescent="0.2">
-      <c r="C20" s="27">
-        <v>4</v>
-      </c>
-      <c r="D20" s="27">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="24" spans="2:17" ht="17.850000000000001" x14ac:dyDescent="0.25">
-      <c r="B24" s="1" t="s">
-        <v>81</v>
-      </c>
-    </row>
+      <c r="C34" s="24">
+        <v>9939</v>
+      </c>
+      <c r="D34" s="60">
+        <v>2487</v>
+      </c>
+      <c r="E34" s="44"/>
+      <c r="F34" s="44"/>
+      <c r="G34" s="44"/>
+      <c r="H34" s="44"/>
+      <c r="I34" s="44"/>
+      <c r="J34" s="44"/>
+      <c r="K34" s="44"/>
+      <c r="L34" s="44"/>
+      <c r="M34" s="44"/>
+      <c r="N34" s="51"/>
+      <c r="O34" s="57"/>
+    </row>
+    <row r="35" spans="1:15" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="46"/>
+      <c r="B35" s="47" t="s">
+        <v>86</v>
+      </c>
+      <c r="C35" s="48" t="s">
+        <v>93</v>
+      </c>
+      <c r="D35" s="48"/>
+      <c r="E35" s="48"/>
+      <c r="F35" s="48"/>
+      <c r="G35" s="48"/>
+      <c r="H35" s="48"/>
+      <c r="I35" s="48"/>
+      <c r="J35" s="48"/>
+      <c r="K35" s="48"/>
+      <c r="L35" s="48"/>
+      <c r="M35" s="48"/>
+      <c r="N35" s="53"/>
+      <c r="O35" s="57"/>
+    </row>
+    <row r="36" spans="1:15" ht="21.6" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="37" spans="1:15" ht="21.6" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="38" spans="1:15" ht="21.6" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="39" spans="1:15" ht="21.6" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="40" spans="1:15" ht="21.6" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="41" spans="1:15" ht="21.6" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="42" spans="1:15" ht="21.6" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="43" spans="1:15" ht="21.6" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="44" spans="1:15" ht="21.6" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="45" spans="1:15" ht="21.6" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="46" spans="1:15" ht="21.6" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="47" spans="1:15" ht="21.6" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="48" spans="1:15" ht="21.6" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="49" ht="21.6" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="50" ht="21.6" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="14">
+    <mergeCell ref="C22:N23"/>
+    <mergeCell ref="A25:A35"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="C35:N35"/>
+    <mergeCell ref="A24:L24"/>
+    <mergeCell ref="M24:N24"/>
+    <mergeCell ref="M1:N1"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="C13:D13"/>
     <mergeCell ref="C2:D2"/>
-    <mergeCell ref="P2:Q2"/>
+    <mergeCell ref="C12:N12"/>
+    <mergeCell ref="A2:A12"/>
+    <mergeCell ref="A13:A23"/>
+    <mergeCell ref="B22:B23"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="M1" location="Таблица!A44" display="Соотв. таблица" xr:uid="{4CD65288-3286-4AD3-A58F-54F99559607B}"/>
+    <hyperlink ref="M24" location="Таблица!A44" display="Соотв. таблица" xr:uid="{9D7BFC76-831B-45ED-A711-BD69FCBDF5EA}"/>
+    <hyperlink ref="M1:N1" location="Таблица!A31" display="Соотв. таблица" xr:uid="{A11C2496-942C-485E-9C90-BC6832A5FEFB}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4269BDC4-CFAE-4A4A-95F0-395DE59C8746}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Version with old comparation (accuracy 1e-4)
</commit_message>
<xml_diff>
--- a/DecompositionLU/docs/statistics.xlsx
+++ b/DecompositionLU/docs/statistics.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Maxim\source\repos\practice\SECOND_COURSE\FOR_ITLAB\ArchBenchs\DecompositionLU\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D008614A-3AA6-44F3-9329-9BDFFF850BE6}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53BC1C17-75AD-4989-A155-43BF22094778}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-114" yWindow="-114" windowWidth="27602" windowHeight="15027" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-114" yWindow="-114" windowWidth="27602" windowHeight="15027" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Таблица" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="103">
   <si>
     <t>Я не уверен, будет ли это использоваться в готовой презентации и так ли это надо делать, если да, так что пока считаем, что файл для личного пользования.</t>
   </si>
@@ -397,14 +397,26 @@
     <t>Эффективность</t>
   </si>
   <si>
-    <t>Мне нравится, но ускорение могло быть лучше</t>
+    <t>Мне нравится, но ускорение могло быть лучше. Возможно, это связано с энергосберегающими ядрами процессора</t>
+  </si>
+  <si>
+    <t>4 производительных, 8 энергосберегающих ядер</t>
+  </si>
+  <si>
+    <t>Производительные: ~1.7-2.1 GHz, ~4.4 Ghz, hyperthreading</t>
+  </si>
+  <si>
+    <t>Энергосберегающие: ~1.2-1.5 GHz, ~3.3 GHz</t>
+  </si>
+  <si>
+    <t>12 Мб кэша третьего уровня, 10 Мб - второго</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -515,6 +527,14 @@
       <charset val="204"/>
     </font>
     <font>
+      <sz val="18"/>
+      <color theme="1"/>
+      <name val="GOST Common"/>
+      <family val="2"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <b/>
       <sz val="18"/>
       <color theme="1"/>
       <name val="GOST Common"/>
@@ -679,7 +699,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="69">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
@@ -774,6 +794,7 @@
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -816,6 +837,9 @@
     <xf numFmtId="0" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
@@ -824,9 +848,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -2597,28 +2618,28 @@
               <c:strCache>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>#DIV/0!</c:v>
+                  <c:v>#ДЕЛ/0!</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>#DIV/0!</c:v>
+                  <c:v>#ДЕЛ/0!</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>#DIV/0!</c:v>
+                  <c:v>#ДЕЛ/0!</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>#DIV/0!</c:v>
+                  <c:v>#ДЕЛ/0!</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>#DIV/0!</c:v>
+                  <c:v>#ДЕЛ/0!</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>#DIV/0!</c:v>
+                  <c:v>#ДЕЛ/0!</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>#DIV/0!</c:v>
+                  <c:v>#ДЕЛ/0!</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>#DIV/0!</c:v>
+                  <c:v>#ДЕЛ/0!</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -2971,28 +2992,28 @@
               <c:strCache>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>#DIV/0!</c:v>
+                  <c:v>#ДЕЛ/0!</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>#DIV/0!</c:v>
+                  <c:v>#ДЕЛ/0!</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>#DIV/0!</c:v>
+                  <c:v>#ДЕЛ/0!</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>#DIV/0!</c:v>
+                  <c:v>#ДЕЛ/0!</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>#DIV/0!</c:v>
+                  <c:v>#ДЕЛ/0!</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>#DIV/0!</c:v>
+                  <c:v>#ДЕЛ/0!</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>#DIV/0!</c:v>
+                  <c:v>#ДЕЛ/0!</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>#DIV/0!</c:v>
+                  <c:v>#ДЕЛ/0!</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -6935,22 +6956,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>9053</xdr:colOff>
+      <xdr:colOff>208229</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>162962</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>465843</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>21108</xdr:rowOff>
+      <xdr:colOff>57156</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>273426</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Рисунок 1">
+        <xdr:cNvPr id="3" name="Рисунок 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{77F3D0DE-7688-4F41-B6B2-A8862A31AAEF}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8AF8B7F6-D74A-4CDC-B0AF-980BCBE244CF}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -6966,8 +6987,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9053" y="0"/>
-          <a:ext cx="6251008" cy="1424395"/>
+          <a:off x="208229" y="162962"/>
+          <a:ext cx="5643145" cy="5162298"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -6978,23 +6999,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>63374</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>81481</xdr:rowOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>181069</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>262550</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>491723</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>191945</xdr:rowOff>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>176382</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>257032</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Рисунок 2">
+        <xdr:cNvPr id="4" name="Рисунок 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8AF8B7F6-D74A-4CDC-B0AF-980BCBE244CF}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{221F9B8A-2F8A-4250-B9AE-2A1DBD282628}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -7010,51 +7031,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="63374" y="1484768"/>
-          <a:ext cx="5643145" cy="5162298"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>21</xdr:col>
-      <xdr:colOff>574735</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>275139</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Рисунок 3">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{221F9B8A-2F8A-4250-B9AE-2A1DBD282628}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="6373640" y="280657"/>
+          <a:off x="5975287" y="262550"/>
           <a:ext cx="6368952" cy="1678427"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -7408,17 +7385,17 @@
       <c r="N3" s="6"/>
     </row>
     <row r="5" spans="1:23" ht="17.850000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="49" t="s">
+      <c r="A5" s="50" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="50"/>
-      <c r="C5" s="50"/>
-      <c r="D5" s="50"/>
-      <c r="E5" s="51"/>
-      <c r="G5" s="53" t="s">
+      <c r="B5" s="51"/>
+      <c r="C5" s="51"/>
+      <c r="D5" s="51"/>
+      <c r="E5" s="52"/>
+      <c r="G5" s="54" t="s">
         <v>3</v>
       </c>
-      <c r="H5" s="53"/>
+      <c r="H5" s="54"/>
       <c r="S5" s="5"/>
       <c r="T5" s="14"/>
       <c r="U5" s="14"/>
@@ -7429,14 +7406,14 @@
       <c r="A6" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="46" t="s">
+      <c r="B6" s="47" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="46"/>
-      <c r="D6" s="46"/>
-      <c r="E6" s="46"/>
-      <c r="G6" s="53"/>
-      <c r="H6" s="53"/>
+      <c r="C6" s="47"/>
+      <c r="D6" s="47"/>
+      <c r="E6" s="47"/>
+      <c r="G6" s="54"/>
+      <c r="H6" s="54"/>
       <c r="S6" s="14"/>
       <c r="T6" s="14"/>
       <c r="U6" s="14"/>
@@ -7459,8 +7436,8 @@
       <c r="E7" s="8">
         <v>10000</v>
       </c>
-      <c r="G7" s="53"/>
-      <c r="H7" s="53"/>
+      <c r="G7" s="54"/>
+      <c r="H7" s="54"/>
       <c r="S7" s="14"/>
       <c r="T7" s="14"/>
       <c r="U7" s="14"/>
@@ -7468,15 +7445,15 @@
       <c r="W7" s="14"/>
     </row>
     <row r="8" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A8" s="47" t="s">
+      <c r="A8" s="48" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="47"/>
-      <c r="C8" s="47"/>
-      <c r="D8" s="47"/>
-      <c r="E8" s="47"/>
-      <c r="G8" s="53"/>
-      <c r="H8" s="53"/>
+      <c r="B8" s="48"/>
+      <c r="C8" s="48"/>
+      <c r="D8" s="48"/>
+      <c r="E8" s="48"/>
+      <c r="G8" s="54"/>
+      <c r="H8" s="54"/>
       <c r="S8" s="14"/>
       <c r="T8" s="14"/>
       <c r="U8" s="14"/>
@@ -7552,13 +7529,13 @@
       <c r="W11" s="5"/>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A12" s="47" t="s">
+      <c r="A12" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="B12" s="47"/>
-      <c r="C12" s="47"/>
-      <c r="D12" s="47"/>
-      <c r="E12" s="47"/>
+      <c r="B12" s="48"/>
+      <c r="C12" s="48"/>
+      <c r="D12" s="48"/>
+      <c r="E12" s="48"/>
       <c r="F12" s="5"/>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.25">
@@ -7571,7 +7548,7 @@
       <c r="C13" s="10">
         <v>232</v>
       </c>
-      <c r="D13" s="55" t="s">
+      <c r="D13" s="56" t="s">
         <v>21</v>
       </c>
       <c r="E13" s="10">
@@ -7589,7 +7566,7 @@
       <c r="C14" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="D14" s="56"/>
+      <c r="D14" s="57"/>
       <c r="E14" s="10" t="s">
         <v>10</v>
       </c>
@@ -7607,30 +7584,30 @@
       <c r="C15" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="D15" s="57"/>
+      <c r="D15" s="58"/>
       <c r="E15" s="10" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A18" s="58" t="s">
+      <c r="A18" s="59" t="s">
         <v>32</v>
       </c>
-      <c r="B18" s="58"/>
-      <c r="C18" s="58"/>
-      <c r="D18" s="58"/>
-      <c r="E18" s="58"/>
+      <c r="B18" s="59"/>
+      <c r="C18" s="59"/>
+      <c r="D18" s="59"/>
+      <c r="E18" s="59"/>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B19" s="46" t="s">
+      <c r="B19" s="47" t="s">
         <v>5</v>
       </c>
-      <c r="C19" s="46"/>
-      <c r="D19" s="46"/>
-      <c r="E19" s="46"/>
+      <c r="C19" s="47"/>
+      <c r="D19" s="47"/>
+      <c r="E19" s="47"/>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
@@ -7650,13 +7627,13 @@
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A21" s="47" t="s">
+      <c r="A21" s="48" t="s">
         <v>11</v>
       </c>
-      <c r="B21" s="47"/>
-      <c r="C21" s="47"/>
-      <c r="D21" s="47"/>
-      <c r="E21" s="47"/>
+      <c r="B21" s="48"/>
+      <c r="C21" s="48"/>
+      <c r="D21" s="48"/>
+      <c r="E21" s="48"/>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
@@ -7709,17 +7686,17 @@
         <v>35</v>
       </c>
       <c r="G24" s="18"/>
-      <c r="H24" s="52"/>
-      <c r="I24" s="52"/>
+      <c r="H24" s="53"/>
+      <c r="I24" s="53"/>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" s="47" t="s">
+      <c r="A25" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="B25" s="47"/>
-      <c r="C25" s="47"/>
-      <c r="D25" s="47"/>
-      <c r="E25" s="47"/>
+      <c r="B25" s="48"/>
+      <c r="C25" s="48"/>
+      <c r="D25" s="48"/>
+      <c r="E25" s="48"/>
       <c r="G25" s="19"/>
       <c r="H25" s="17"/>
       <c r="I25" s="17"/>
@@ -7804,15 +7781,15 @@
       <c r="I30" s="18"/>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A31" s="49" t="s">
+      <c r="A31" s="50" t="s">
         <v>70</v>
       </c>
-      <c r="B31" s="50"/>
-      <c r="C31" s="51"/>
-      <c r="D31" s="48" t="s">
+      <c r="B31" s="51"/>
+      <c r="C31" s="52"/>
+      <c r="D31" s="49" t="s">
         <v>91</v>
       </c>
-      <c r="E31" s="48" t="s">
+      <c r="E31" s="49" t="s">
         <v>91</v>
       </c>
       <c r="G31" s="20"/>
@@ -7823,12 +7800,12 @@
       <c r="A32" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B32" s="46" t="s">
+      <c r="B32" s="47" t="s">
         <v>5</v>
       </c>
-      <c r="C32" s="46"/>
-      <c r="D32" s="46"/>
-      <c r="E32" s="46"/>
+      <c r="C32" s="47"/>
+      <c r="D32" s="47"/>
+      <c r="E32" s="47"/>
       <c r="G32" s="23"/>
       <c r="H32" s="18"/>
       <c r="I32" s="18"/>
@@ -7854,13 +7831,13 @@
       <c r="I33" s="18"/>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A34" s="47" t="s">
+      <c r="A34" s="48" t="s">
         <v>11</v>
       </c>
-      <c r="B34" s="47"/>
-      <c r="C34" s="47"/>
-      <c r="D34" s="47"/>
-      <c r="E34" s="47"/>
+      <c r="B34" s="48"/>
+      <c r="C34" s="48"/>
+      <c r="D34" s="48"/>
+      <c r="E34" s="48"/>
       <c r="G34" s="23"/>
       <c r="H34" s="18"/>
       <c r="I34" s="18"/>
@@ -7926,13 +7903,13 @@
       <c r="I37" s="18"/>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A38" s="47" t="s">
+      <c r="A38" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="B38" s="47"/>
-      <c r="C38" s="47"/>
-      <c r="D38" s="47"/>
-      <c r="E38" s="47"/>
+      <c r="B38" s="48"/>
+      <c r="C38" s="48"/>
+      <c r="D38" s="48"/>
+      <c r="E38" s="48"/>
       <c r="G38" s="23"/>
       <c r="H38" s="18"/>
       <c r="I38" s="18"/>
@@ -7998,23 +7975,23 @@
       <c r="I41" s="18"/>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B42" s="54" t="s">
+      <c r="B42" s="55" t="s">
         <v>66</v>
       </c>
-      <c r="C42" s="54"/>
-      <c r="D42" s="54"/>
-      <c r="E42" s="54"/>
+      <c r="C42" s="55"/>
+      <c r="D42" s="55"/>
+      <c r="E42" s="55"/>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A44" s="49" t="s">
+      <c r="A44" s="50" t="s">
         <v>82</v>
       </c>
-      <c r="B44" s="50"/>
-      <c r="C44" s="51"/>
-      <c r="D44" s="48" t="s">
+      <c r="B44" s="51"/>
+      <c r="C44" s="52"/>
+      <c r="D44" s="49" t="s">
         <v>92</v>
       </c>
-      <c r="E44" s="48" t="s">
+      <c r="E44" s="49" t="s">
         <v>91</v>
       </c>
     </row>
@@ -8022,12 +7999,12 @@
       <c r="A45" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B45" s="46" t="s">
+      <c r="B45" s="47" t="s">
         <v>5</v>
       </c>
-      <c r="C45" s="46"/>
-      <c r="D45" s="46"/>
-      <c r="E45" s="46"/>
+      <c r="C45" s="47"/>
+      <c r="D45" s="47"/>
+      <c r="E45" s="47"/>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
@@ -8047,13 +8024,13 @@
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A47" s="47" t="s">
+      <c r="A47" s="48" t="s">
         <v>11</v>
       </c>
-      <c r="B47" s="47"/>
-      <c r="C47" s="47"/>
-      <c r="D47" s="47"/>
-      <c r="E47" s="47"/>
+      <c r="B47" s="48"/>
+      <c r="C47" s="48"/>
+      <c r="D47" s="48"/>
+      <c r="E47" s="48"/>
       <c r="G47" s="1" t="s">
         <v>95</v>
       </c>
@@ -8066,16 +8043,16 @@
         <v>7</v>
       </c>
       <c r="B48" s="9">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="C48" s="10">
-        <v>123</v>
+        <v>154</v>
       </c>
       <c r="D48" s="10">
-        <v>378</v>
+        <v>486</v>
       </c>
       <c r="E48" s="10">
-        <v>1131</v>
+        <v>1184</v>
       </c>
       <c r="G48" s="1">
         <v>32</v>
@@ -8089,16 +8066,16 @@
         <v>8</v>
       </c>
       <c r="B49" s="9">
-        <v>122</v>
+        <v>77</v>
       </c>
       <c r="C49" s="10">
-        <v>2103</v>
+        <v>994</v>
       </c>
       <c r="D49" s="10">
-        <v>26833</v>
+        <v>9972</v>
       </c>
       <c r="E49" s="10">
-        <v>73485</v>
+        <v>28809</v>
       </c>
       <c r="G49" s="1">
         <v>128</v>
@@ -8112,16 +8089,16 @@
         <v>9</v>
       </c>
       <c r="B50" s="9">
-        <v>139</v>
+        <v>99</v>
       </c>
       <c r="C50" s="10">
-        <v>2226</v>
+        <v>1149</v>
       </c>
       <c r="D50" s="10">
-        <v>27211</v>
+        <v>10459</v>
       </c>
       <c r="E50" s="10">
-        <v>74635</v>
+        <v>30062</v>
       </c>
       <c r="G50" s="1">
         <v>256</v>
@@ -8131,13 +8108,13 @@
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A51" s="47" t="s">
+      <c r="A51" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="B51" s="47"/>
-      <c r="C51" s="47"/>
-      <c r="D51" s="47"/>
-      <c r="E51" s="47"/>
+      <c r="B51" s="48"/>
+      <c r="C51" s="48"/>
+      <c r="D51" s="48"/>
+      <c r="E51" s="48"/>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" s="3" t="s">
@@ -8245,24 +8222,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="58" t="s">
+      <c r="A1" s="59" t="s">
         <v>84</v>
       </c>
-      <c r="B1" s="58"/>
-      <c r="C1" s="58"/>
-      <c r="D1" s="58"/>
-      <c r="E1" s="58"/>
-      <c r="F1" s="58"/>
-      <c r="G1" s="58"/>
-      <c r="H1" s="58"/>
-      <c r="I1" s="58"/>
-      <c r="J1" s="58"/>
-      <c r="K1" s="58"/>
-      <c r="L1" s="58"/>
-      <c r="M1" s="48" t="s">
+      <c r="B1" s="59"/>
+      <c r="C1" s="59"/>
+      <c r="D1" s="59"/>
+      <c r="E1" s="59"/>
+      <c r="F1" s="59"/>
+      <c r="G1" s="59"/>
+      <c r="H1" s="59"/>
+      <c r="I1" s="59"/>
+      <c r="J1" s="59"/>
+      <c r="K1" s="59"/>
+      <c r="L1" s="59"/>
+      <c r="M1" s="49" t="s">
         <v>90</v>
       </c>
-      <c r="N1" s="48"/>
+      <c r="N1" s="49"/>
       <c r="O1" s="36"/>
       <c r="P1" s="35"/>
       <c r="Q1" s="35"/>
@@ -8277,14 +8254,14 @@
       <c r="Z1" s="35"/>
     </row>
     <row r="2" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="65" t="s">
+      <c r="A2" s="66" t="s">
         <v>85</v>
       </c>
       <c r="B2" s="44"/>
-      <c r="C2" s="59" t="s">
+      <c r="C2" s="60" t="s">
         <v>78</v>
       </c>
-      <c r="D2" s="59"/>
+      <c r="D2" s="60"/>
       <c r="E2" s="31"/>
       <c r="F2" s="31"/>
       <c r="G2" s="31"/>
@@ -8309,7 +8286,7 @@
       <c r="Z2" s="30"/>
     </row>
     <row r="3" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="65"/>
+      <c r="A3" s="66"/>
       <c r="B3" s="29" t="s">
         <v>77</v>
       </c>
@@ -8343,7 +8320,7 @@
       <c r="Z3" s="30"/>
     </row>
     <row r="4" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="65"/>
+      <c r="A4" s="66"/>
       <c r="B4" s="15">
         <v>1</v>
       </c>
@@ -8377,7 +8354,7 @@
       <c r="Z4" s="30"/>
     </row>
     <row r="5" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="65"/>
+      <c r="A5" s="66"/>
       <c r="B5" s="15">
         <v>2</v>
       </c>
@@ -8411,7 +8388,7 @@
       <c r="Z5" s="30"/>
     </row>
     <row r="6" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="65"/>
+      <c r="A6" s="66"/>
       <c r="B6" s="15">
         <v>4</v>
       </c>
@@ -8434,7 +8411,7 @@
       <c r="O6" s="38"/>
     </row>
     <row r="7" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="65"/>
+      <c r="A7" s="66"/>
       <c r="B7" s="15">
         <v>6</v>
       </c>
@@ -8457,7 +8434,7 @@
       <c r="O7" s="38"/>
     </row>
     <row r="8" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="65"/>
+      <c r="A8" s="66"/>
       <c r="B8" s="15">
         <v>8</v>
       </c>
@@ -8480,7 +8457,7 @@
       <c r="O8" s="38"/>
     </row>
     <row r="9" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="65"/>
+      <c r="A9" s="66"/>
       <c r="B9" s="15">
         <v>10</v>
       </c>
@@ -8503,7 +8480,7 @@
       <c r="O9" s="38"/>
     </row>
     <row r="10" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="65"/>
+      <c r="A10" s="66"/>
       <c r="B10" s="15">
         <v>12</v>
       </c>
@@ -8526,7 +8503,7 @@
       <c r="O10" s="38"/>
     </row>
     <row r="11" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="65"/>
+      <c r="A11" s="66"/>
       <c r="B11" s="15">
         <v>16</v>
       </c>
@@ -8551,37 +8528,37 @@
       <c r="Q11" s="27"/>
     </row>
     <row r="12" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="65"/>
+      <c r="A12" s="66"/>
       <c r="B12" s="33" t="s">
         <v>86</v>
       </c>
-      <c r="C12" s="63" t="s">
+      <c r="C12" s="61" t="s">
         <v>81</v>
       </c>
-      <c r="D12" s="63"/>
-      <c r="E12" s="63"/>
-      <c r="F12" s="63"/>
-      <c r="G12" s="63"/>
-      <c r="H12" s="63"/>
-      <c r="I12" s="63"/>
-      <c r="J12" s="63"/>
-      <c r="K12" s="63"/>
-      <c r="L12" s="63"/>
-      <c r="M12" s="63"/>
-      <c r="N12" s="64"/>
+      <c r="D12" s="61"/>
+      <c r="E12" s="61"/>
+      <c r="F12" s="61"/>
+      <c r="G12" s="61"/>
+      <c r="H12" s="61"/>
+      <c r="I12" s="61"/>
+      <c r="J12" s="61"/>
+      <c r="K12" s="61"/>
+      <c r="L12" s="61"/>
+      <c r="M12" s="61"/>
+      <c r="N12" s="65"/>
       <c r="O12" s="39"/>
       <c r="P12" s="23"/>
       <c r="Q12" s="23"/>
     </row>
     <row r="13" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="65" t="s">
+      <c r="A13" s="66" t="s">
         <v>87</v>
       </c>
       <c r="B13" s="44"/>
-      <c r="C13" s="59" t="s">
+      <c r="C13" s="60" t="s">
         <v>78</v>
       </c>
-      <c r="D13" s="59"/>
+      <c r="D13" s="60"/>
       <c r="E13" s="32"/>
       <c r="F13" s="31"/>
       <c r="G13" s="31"/>
@@ -8597,7 +8574,7 @@
       <c r="Q13" s="23"/>
     </row>
     <row r="14" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="65"/>
+      <c r="A14" s="66"/>
       <c r="B14" s="13" t="s">
         <v>77</v>
       </c>
@@ -8622,7 +8599,7 @@
       <c r="Q14" s="23"/>
     </row>
     <row r="15" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="65"/>
+      <c r="A15" s="66"/>
       <c r="B15" s="15">
         <v>1</v>
       </c>
@@ -8647,7 +8624,7 @@
       <c r="Q15" s="27"/>
     </row>
     <row r="16" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="65"/>
+      <c r="A16" s="66"/>
       <c r="B16" s="15">
         <v>2</v>
       </c>
@@ -8672,7 +8649,7 @@
       <c r="Q16" s="23"/>
     </row>
     <row r="17" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="65"/>
+      <c r="A17" s="66"/>
       <c r="B17" s="15">
         <v>4</v>
       </c>
@@ -8697,7 +8674,7 @@
       <c r="Q17" s="23"/>
     </row>
     <row r="18" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="65"/>
+      <c r="A18" s="66"/>
       <c r="B18" s="15">
         <v>6</v>
       </c>
@@ -8722,7 +8699,7 @@
       <c r="Q18" s="23"/>
     </row>
     <row r="19" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="65"/>
+      <c r="A19" s="66"/>
       <c r="B19" s="15">
         <v>8</v>
       </c>
@@ -8745,7 +8722,7 @@
       <c r="O19" s="38"/>
     </row>
     <row r="20" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="65"/>
+      <c r="A20" s="66"/>
       <c r="B20" s="15">
         <v>10</v>
       </c>
@@ -8768,7 +8745,7 @@
       <c r="O20" s="38"/>
     </row>
     <row r="21" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="65"/>
+      <c r="A21" s="66"/>
       <c r="B21" s="15">
         <v>12</v>
       </c>
@@ -8791,73 +8768,73 @@
       <c r="O21" s="38"/>
     </row>
     <row r="22" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="65"/>
-      <c r="B22" s="66" t="s">
+      <c r="A22" s="66"/>
+      <c r="B22" s="67" t="s">
         <v>86</v>
       </c>
-      <c r="C22" s="67" t="s">
+      <c r="C22" s="68" t="s">
         <v>88</v>
       </c>
-      <c r="D22" s="67"/>
-      <c r="E22" s="67"/>
-      <c r="F22" s="67"/>
-      <c r="G22" s="67"/>
-      <c r="H22" s="67"/>
-      <c r="I22" s="67"/>
-      <c r="J22" s="67"/>
-      <c r="K22" s="67"/>
-      <c r="L22" s="67"/>
-      <c r="M22" s="67"/>
-      <c r="N22" s="68"/>
+      <c r="D22" s="68"/>
+      <c r="E22" s="68"/>
+      <c r="F22" s="68"/>
+      <c r="G22" s="68"/>
+      <c r="H22" s="68"/>
+      <c r="I22" s="68"/>
+      <c r="J22" s="68"/>
+      <c r="K22" s="68"/>
+      <c r="L22" s="68"/>
+      <c r="M22" s="68"/>
+      <c r="N22" s="69"/>
       <c r="O22" s="38"/>
     </row>
     <row r="23" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="65"/>
-      <c r="B23" s="66"/>
-      <c r="C23" s="67"/>
-      <c r="D23" s="67"/>
-      <c r="E23" s="67"/>
-      <c r="F23" s="67"/>
-      <c r="G23" s="67"/>
-      <c r="H23" s="67"/>
-      <c r="I23" s="67"/>
-      <c r="J23" s="67"/>
-      <c r="K23" s="67"/>
-      <c r="L23" s="67"/>
-      <c r="M23" s="67"/>
-      <c r="N23" s="68"/>
+      <c r="A23" s="66"/>
+      <c r="B23" s="67"/>
+      <c r="C23" s="68"/>
+      <c r="D23" s="68"/>
+      <c r="E23" s="68"/>
+      <c r="F23" s="68"/>
+      <c r="G23" s="68"/>
+      <c r="H23" s="68"/>
+      <c r="I23" s="68"/>
+      <c r="J23" s="68"/>
+      <c r="K23" s="68"/>
+      <c r="L23" s="68"/>
+      <c r="M23" s="68"/>
+      <c r="N23" s="69"/>
       <c r="O23" s="38"/>
     </row>
     <row r="24" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="58" t="s">
+      <c r="A24" s="59" t="s">
         <v>89</v>
       </c>
-      <c r="B24" s="58"/>
-      <c r="C24" s="58"/>
-      <c r="D24" s="58"/>
-      <c r="E24" s="58"/>
-      <c r="F24" s="58"/>
-      <c r="G24" s="58"/>
-      <c r="H24" s="58"/>
-      <c r="I24" s="58"/>
-      <c r="J24" s="58"/>
-      <c r="K24" s="58"/>
-      <c r="L24" s="58"/>
-      <c r="M24" s="48" t="s">
+      <c r="B24" s="59"/>
+      <c r="C24" s="59"/>
+      <c r="D24" s="59"/>
+      <c r="E24" s="59"/>
+      <c r="F24" s="59"/>
+      <c r="G24" s="59"/>
+      <c r="H24" s="59"/>
+      <c r="I24" s="59"/>
+      <c r="J24" s="59"/>
+      <c r="K24" s="59"/>
+      <c r="L24" s="59"/>
+      <c r="M24" s="49" t="s">
         <v>90</v>
       </c>
-      <c r="N24" s="48"/>
+      <c r="N24" s="49"/>
       <c r="O24" s="38"/>
     </row>
     <row r="25" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="60" t="s">
+      <c r="A25" s="62" t="s">
         <v>85</v>
       </c>
       <c r="B25" s="44"/>
-      <c r="C25" s="59" t="s">
+      <c r="C25" s="60" t="s">
         <v>78</v>
       </c>
-      <c r="D25" s="59"/>
+      <c r="D25" s="60"/>
       <c r="E25" s="31"/>
       <c r="F25" s="31"/>
       <c r="G25" s="31"/>
@@ -8871,7 +8848,7 @@
       <c r="O25" s="27"/>
     </row>
     <row r="26" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="61"/>
+      <c r="A26" s="63"/>
       <c r="B26" s="42" t="s">
         <v>77</v>
       </c>
@@ -8894,7 +8871,7 @@
       <c r="O26" s="27"/>
     </row>
     <row r="27" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="61"/>
+      <c r="A27" s="63"/>
       <c r="B27" s="15">
         <v>1</v>
       </c>
@@ -8917,7 +8894,7 @@
       <c r="O27" s="27"/>
     </row>
     <row r="28" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="61"/>
+      <c r="A28" s="63"/>
       <c r="B28" s="15">
         <v>2</v>
       </c>
@@ -8940,7 +8917,7 @@
       <c r="O28" s="27"/>
     </row>
     <row r="29" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="61"/>
+      <c r="A29" s="63"/>
       <c r="B29" s="15">
         <v>4</v>
       </c>
@@ -8963,7 +8940,7 @@
       <c r="O29" s="27"/>
     </row>
     <row r="30" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="61"/>
+      <c r="A30" s="63"/>
       <c r="B30" s="15">
         <v>6</v>
       </c>
@@ -8986,7 +8963,7 @@
       <c r="O30" s="27"/>
     </row>
     <row r="31" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="61"/>
+      <c r="A31" s="63"/>
       <c r="B31" s="15">
         <v>8</v>
       </c>
@@ -9009,7 +8986,7 @@
       <c r="O31" s="27"/>
     </row>
     <row r="32" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="61"/>
+      <c r="A32" s="63"/>
       <c r="B32" s="15">
         <v>10</v>
       </c>
@@ -9032,7 +9009,7 @@
       <c r="O32" s="27"/>
     </row>
     <row r="33" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="61"/>
+      <c r="A33" s="63"/>
       <c r="B33" s="15">
         <v>12</v>
       </c>
@@ -9055,7 +9032,7 @@
       <c r="O33" s="27"/>
     </row>
     <row r="34" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="61"/>
+      <c r="A34" s="63"/>
       <c r="B34" s="15">
         <v>16</v>
       </c>
@@ -9078,12 +9055,12 @@
       <c r="O34" s="27"/>
     </row>
     <row r="35" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="61"/>
+      <c r="A35" s="63"/>
       <c r="B35" s="45"/>
-      <c r="C35" s="59" t="s">
+      <c r="C35" s="60" t="s">
         <v>96</v>
       </c>
-      <c r="D35" s="59"/>
+      <c r="D35" s="60"/>
       <c r="E35" s="31"/>
       <c r="F35" s="31"/>
       <c r="G35" s="31"/>
@@ -9097,7 +9074,7 @@
       <c r="O35" s="27"/>
     </row>
     <row r="36" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="61"/>
+      <c r="A36" s="63"/>
       <c r="B36" s="42" t="s">
         <v>77</v>
       </c>
@@ -9121,7 +9098,7 @@
       <c r="P36" s="1"/>
     </row>
     <row r="37" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="61"/>
+      <c r="A37" s="63"/>
       <c r="B37" s="42">
         <v>1</v>
       </c>
@@ -9147,7 +9124,7 @@
       <c r="P37" s="1"/>
     </row>
     <row r="38" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="61"/>
+      <c r="A38" s="63"/>
       <c r="B38" s="42">
         <v>2</v>
       </c>
@@ -9173,7 +9150,7 @@
       <c r="P38" s="1"/>
     </row>
     <row r="39" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="61"/>
+      <c r="A39" s="63"/>
       <c r="B39" s="42">
         <v>4</v>
       </c>
@@ -9199,7 +9176,7 @@
       <c r="P39" s="1"/>
     </row>
     <row r="40" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="61"/>
+      <c r="A40" s="63"/>
       <c r="B40" s="42">
         <v>6</v>
       </c>
@@ -9225,7 +9202,7 @@
       <c r="P40" s="1"/>
     </row>
     <row r="41" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="61"/>
+      <c r="A41" s="63"/>
       <c r="B41" s="42">
         <v>8</v>
       </c>
@@ -9251,7 +9228,7 @@
       <c r="P41" s="1"/>
     </row>
     <row r="42" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="61"/>
+      <c r="A42" s="63"/>
       <c r="B42" s="42">
         <v>10</v>
       </c>
@@ -9277,7 +9254,7 @@
       <c r="P42" s="1"/>
     </row>
     <row r="43" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="61"/>
+      <c r="A43" s="63"/>
       <c r="B43" s="42">
         <v>12</v>
       </c>
@@ -9303,7 +9280,7 @@
       <c r="P43" s="1"/>
     </row>
     <row r="44" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="61"/>
+      <c r="A44" s="63"/>
       <c r="B44" s="42">
         <v>16</v>
       </c>
@@ -9329,12 +9306,12 @@
       <c r="P44" s="1"/>
     </row>
     <row r="45" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="61"/>
+      <c r="A45" s="63"/>
       <c r="B45" s="45"/>
-      <c r="C45" s="59" t="s">
+      <c r="C45" s="60" t="s">
         <v>97</v>
       </c>
-      <c r="D45" s="59"/>
+      <c r="D45" s="60"/>
       <c r="E45" s="43"/>
       <c r="F45" s="43"/>
       <c r="G45" s="43"/>
@@ -9349,7 +9326,7 @@
       <c r="P45" s="1"/>
     </row>
     <row r="46" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="61"/>
+      <c r="A46" s="63"/>
       <c r="B46" s="42" t="s">
         <v>77</v>
       </c>
@@ -9373,16 +9350,16 @@
       <c r="P46" s="1"/>
     </row>
     <row r="47" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="61"/>
+      <c r="A47" s="63"/>
       <c r="B47" s="42">
         <v>1</v>
       </c>
       <c r="C47" s="43">
-        <f>C37/B37</f>
+        <f t="shared" ref="C47:C54" si="0">C37/B37</f>
         <v>1</v>
       </c>
       <c r="D47" s="43">
-        <f>D37/B37</f>
+        <f t="shared" ref="D47:D54" si="1">D37/B37</f>
         <v>1</v>
       </c>
       <c r="E47" s="43"/>
@@ -9399,16 +9376,16 @@
       <c r="P47" s="1"/>
     </row>
     <row r="48" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="61"/>
+      <c r="A48" s="63"/>
       <c r="B48" s="42">
         <v>2</v>
       </c>
       <c r="C48" s="43">
-        <f>C38/B38</f>
+        <f t="shared" si="0"/>
         <v>0.98108925869894104</v>
       </c>
       <c r="D48" s="43">
-        <f>D38/B38</f>
+        <f t="shared" si="1"/>
         <v>0.94677230671062429</v>
       </c>
       <c r="E48" s="43"/>
@@ -9425,16 +9402,16 @@
       <c r="P48" s="1"/>
     </row>
     <row r="49" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="61"/>
+      <c r="A49" s="63"/>
       <c r="B49" s="42">
         <v>4</v>
       </c>
       <c r="C49" s="43">
-        <f>C39/B39</f>
+        <f t="shared" si="0"/>
         <v>0.91330112232959226</v>
       </c>
       <c r="D49" s="43">
-        <f>D39/B39</f>
+        <f t="shared" si="1"/>
         <v>0.90472560975609762</v>
       </c>
       <c r="E49" s="43"/>
@@ -9451,16 +9428,16 @@
       <c r="P49" s="1"/>
     </row>
     <row r="50" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="61"/>
+      <c r="A50" s="63"/>
       <c r="B50" s="42">
         <v>6</v>
       </c>
       <c r="C50" s="43">
-        <f>C40/B40</f>
+        <f t="shared" si="0"/>
         <v>0.78055848749143564</v>
       </c>
       <c r="D50" s="43">
-        <f>D40/B40</f>
+        <f t="shared" si="1"/>
         <v>0.73380316518298716</v>
       </c>
       <c r="E50" s="43"/>
@@ -9477,16 +9454,16 @@
       <c r="P50" s="1"/>
     </row>
     <row r="51" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="61"/>
+      <c r="A51" s="63"/>
       <c r="B51" s="42">
         <v>8</v>
       </c>
       <c r="C51" s="43">
-        <f>C41/B41</f>
+        <f t="shared" si="0"/>
         <v>0.73910260906157943</v>
       </c>
       <c r="D51" s="43">
-        <f>D41/B41</f>
+        <f t="shared" si="1"/>
         <v>0.67097527886644559</v>
       </c>
       <c r="E51" s="43"/>
@@ -9502,16 +9479,16 @@
       <c r="O51" s="1"/>
     </row>
     <row r="52" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="61"/>
+      <c r="A52" s="63"/>
       <c r="B52" s="42">
         <v>10</v>
       </c>
       <c r="C52" s="43">
-        <f>C42/B42</f>
+        <f t="shared" si="0"/>
         <v>0.66718106995884774</v>
       </c>
       <c r="D52" s="43">
-        <f>D42/B42</f>
+        <f t="shared" si="1"/>
         <v>0.59608302644794109</v>
       </c>
       <c r="E52" s="43"/>
@@ -9527,16 +9504,16 @@
       <c r="O52" s="1"/>
     </row>
     <row r="53" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="61"/>
+      <c r="A53" s="63"/>
       <c r="B53" s="42">
         <v>12</v>
       </c>
       <c r="C53" s="43">
-        <f>C43/B43</f>
+        <f t="shared" si="0"/>
         <v>0.61496994631185808</v>
       </c>
       <c r="D53" s="43">
-        <f>D43/B43</f>
+        <f t="shared" si="1"/>
         <v>0.54191015339663984</v>
       </c>
       <c r="E53" s="31"/>
@@ -9552,16 +9529,16 @@
       <c r="O53" s="1"/>
     </row>
     <row r="54" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="61"/>
+      <c r="A54" s="63"/>
       <c r="B54" s="42">
         <v>16</v>
       </c>
       <c r="C54" s="43">
-        <f>C44/B44</f>
+        <f t="shared" si="0"/>
         <v>0.53014010463829364</v>
       </c>
       <c r="D54" s="43">
-        <f>D44/B44</f>
+        <f t="shared" si="1"/>
         <v>0.44745174909529556</v>
       </c>
       <c r="E54" s="31"/>
@@ -9577,34 +9554,34 @@
       <c r="O54" s="1"/>
     </row>
     <row r="55" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="62"/>
+      <c r="A55" s="64"/>
       <c r="B55" s="33" t="s">
         <v>86</v>
       </c>
-      <c r="C55" s="63" t="s">
+      <c r="C55" s="61" t="s">
         <v>98</v>
       </c>
-      <c r="D55" s="63"/>
-      <c r="E55" s="63"/>
-      <c r="F55" s="63"/>
-      <c r="G55" s="63"/>
-      <c r="H55" s="63"/>
-      <c r="I55" s="63"/>
-      <c r="J55" s="63"/>
-      <c r="K55" s="63"/>
-      <c r="L55" s="63"/>
-      <c r="M55" s="63"/>
-      <c r="N55" s="63"/>
+      <c r="D55" s="61"/>
+      <c r="E55" s="61"/>
+      <c r="F55" s="61"/>
+      <c r="G55" s="61"/>
+      <c r="H55" s="61"/>
+      <c r="I55" s="61"/>
+      <c r="J55" s="61"/>
+      <c r="K55" s="61"/>
+      <c r="L55" s="61"/>
+      <c r="M55" s="61"/>
+      <c r="N55" s="61"/>
     </row>
     <row r="56" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="60" t="s">
+      <c r="A56" s="62" t="s">
         <v>87</v>
       </c>
       <c r="B56" s="44"/>
-      <c r="C56" s="59" t="s">
+      <c r="C56" s="60" t="s">
         <v>78</v>
       </c>
-      <c r="D56" s="59"/>
+      <c r="D56" s="60"/>
       <c r="E56" s="31"/>
       <c r="F56" s="31"/>
       <c r="G56" s="31"/>
@@ -9617,7 +9594,7 @@
       <c r="N56" s="31"/>
     </row>
     <row r="57" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="61"/>
+      <c r="A57" s="63"/>
       <c r="B57" s="42" t="s">
         <v>77</v>
       </c>
@@ -9639,7 +9616,7 @@
       <c r="N57" s="31"/>
     </row>
     <row r="58" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="61"/>
+      <c r="A58" s="63"/>
       <c r="B58" s="15">
         <v>1</v>
       </c>
@@ -9657,7 +9634,7 @@
       <c r="N58" s="31"/>
     </row>
     <row r="59" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="61"/>
+      <c r="A59" s="63"/>
       <c r="B59" s="15">
         <v>2</v>
       </c>
@@ -9675,7 +9652,7 @@
       <c r="N59" s="31"/>
     </row>
     <row r="60" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="61"/>
+      <c r="A60" s="63"/>
       <c r="B60" s="15">
         <v>4</v>
       </c>
@@ -9693,7 +9670,7 @@
       <c r="N60" s="31"/>
     </row>
     <row r="61" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="61"/>
+      <c r="A61" s="63"/>
       <c r="B61" s="15">
         <v>6</v>
       </c>
@@ -9711,7 +9688,7 @@
       <c r="N61" s="31"/>
     </row>
     <row r="62" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="61"/>
+      <c r="A62" s="63"/>
       <c r="B62" s="15">
         <v>8</v>
       </c>
@@ -9729,7 +9706,7 @@
       <c r="N62" s="31"/>
     </row>
     <row r="63" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="61"/>
+      <c r="A63" s="63"/>
       <c r="B63" s="15">
         <v>10</v>
       </c>
@@ -9747,7 +9724,7 @@
       <c r="N63" s="31"/>
     </row>
     <row r="64" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="61"/>
+      <c r="A64" s="63"/>
       <c r="B64" s="15">
         <v>12</v>
       </c>
@@ -9765,7 +9742,7 @@
       <c r="N64" s="31"/>
     </row>
     <row r="65" spans="1:14" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="61"/>
+      <c r="A65" s="63"/>
       <c r="B65" s="15">
         <v>16</v>
       </c>
@@ -9783,12 +9760,12 @@
       <c r="N65" s="31"/>
     </row>
     <row r="66" spans="1:14" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="61"/>
+      <c r="A66" s="63"/>
       <c r="B66" s="45"/>
-      <c r="C66" s="59" t="s">
+      <c r="C66" s="60" t="s">
         <v>96</v>
       </c>
-      <c r="D66" s="59"/>
+      <c r="D66" s="60"/>
       <c r="E66" s="31"/>
       <c r="F66" s="31"/>
       <c r="G66" s="31"/>
@@ -9801,7 +9778,7 @@
       <c r="N66" s="31"/>
     </row>
     <row r="67" spans="1:14" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="61"/>
+      <c r="A67" s="63"/>
       <c r="B67" s="42" t="s">
         <v>77</v>
       </c>
@@ -9823,7 +9800,7 @@
       <c r="N67" s="16"/>
     </row>
     <row r="68" spans="1:14" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="61"/>
+      <c r="A68" s="63"/>
       <c r="B68" s="42">
         <v>1</v>
       </c>
@@ -9847,7 +9824,7 @@
       <c r="N68" s="16"/>
     </row>
     <row r="69" spans="1:14" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="61"/>
+      <c r="A69" s="63"/>
       <c r="B69" s="42">
         <v>2</v>
       </c>
@@ -9871,7 +9848,7 @@
       <c r="N69" s="16"/>
     </row>
     <row r="70" spans="1:14" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="61"/>
+      <c r="A70" s="63"/>
       <c r="B70" s="42">
         <v>4</v>
       </c>
@@ -9895,7 +9872,7 @@
       <c r="N70" s="16"/>
     </row>
     <row r="71" spans="1:14" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="61"/>
+      <c r="A71" s="63"/>
       <c r="B71" s="42">
         <v>6</v>
       </c>
@@ -9919,7 +9896,7 @@
       <c r="N71" s="16"/>
     </row>
     <row r="72" spans="1:14" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="61"/>
+      <c r="A72" s="63"/>
       <c r="B72" s="42">
         <v>8</v>
       </c>
@@ -9943,7 +9920,7 @@
       <c r="N72" s="16"/>
     </row>
     <row r="73" spans="1:14" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="61"/>
+      <c r="A73" s="63"/>
       <c r="B73" s="42">
         <v>10</v>
       </c>
@@ -9967,7 +9944,7 @@
       <c r="N73" s="16"/>
     </row>
     <row r="74" spans="1:14" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A74" s="61"/>
+      <c r="A74" s="63"/>
       <c r="B74" s="42">
         <v>12</v>
       </c>
@@ -9991,7 +9968,7 @@
       <c r="N74" s="16"/>
     </row>
     <row r="75" spans="1:14" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A75" s="61"/>
+      <c r="A75" s="63"/>
       <c r="B75" s="42">
         <v>16</v>
       </c>
@@ -10015,12 +9992,12 @@
       <c r="N75" s="16"/>
     </row>
     <row r="76" spans="1:14" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="61"/>
+      <c r="A76" s="63"/>
       <c r="B76" s="45"/>
-      <c r="C76" s="59" t="s">
+      <c r="C76" s="60" t="s">
         <v>97</v>
       </c>
-      <c r="D76" s="59"/>
+      <c r="D76" s="60"/>
       <c r="E76" s="43"/>
       <c r="F76" s="43"/>
       <c r="G76" s="43"/>
@@ -10033,7 +10010,7 @@
       <c r="N76" s="16"/>
     </row>
     <row r="77" spans="1:14" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="61"/>
+      <c r="A77" s="63"/>
       <c r="B77" s="42" t="s">
         <v>77</v>
       </c>
@@ -10055,7 +10032,7 @@
       <c r="N77" s="16"/>
     </row>
     <row r="78" spans="1:14" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A78" s="61"/>
+      <c r="A78" s="63"/>
       <c r="B78" s="42">
         <v>1</v>
       </c>
@@ -10079,7 +10056,7 @@
       <c r="N78" s="16"/>
     </row>
     <row r="79" spans="1:14" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A79" s="61"/>
+      <c r="A79" s="63"/>
       <c r="B79" s="42">
         <v>2</v>
       </c>
@@ -10088,7 +10065,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="D79" s="43" t="e">
-        <f t="shared" ref="D79:D85" si="0">D69/B69</f>
+        <f t="shared" ref="D79:D85" si="2">D69/B69</f>
         <v>#DIV/0!</v>
       </c>
       <c r="E79" s="43"/>
@@ -10103,16 +10080,16 @@
       <c r="N79" s="16"/>
     </row>
     <row r="80" spans="1:14" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A80" s="61"/>
+      <c r="A80" s="63"/>
       <c r="B80" s="42">
         <v>4</v>
       </c>
       <c r="C80" s="43" t="e">
-        <f t="shared" ref="C80:C85" si="1">C70/B70</f>
+        <f t="shared" ref="C80:C85" si="3">C70/B70</f>
         <v>#DIV/0!</v>
       </c>
       <c r="D80" s="43" t="e">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="E80" s="43"/>
@@ -10127,16 +10104,16 @@
       <c r="N80" s="16"/>
     </row>
     <row r="81" spans="1:14" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="61"/>
+      <c r="A81" s="63"/>
       <c r="B81" s="42">
         <v>6</v>
       </c>
       <c r="C81" s="43" t="e">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="D81" s="43" t="e">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="E81" s="43"/>
@@ -10151,16 +10128,16 @@
       <c r="N81" s="16"/>
     </row>
     <row r="82" spans="1:14" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A82" s="61"/>
+      <c r="A82" s="63"/>
       <c r="B82" s="42">
         <v>8</v>
       </c>
       <c r="C82" s="43" t="e">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="D82" s="43" t="e">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="E82" s="43"/>
@@ -10175,16 +10152,16 @@
       <c r="N82" s="16"/>
     </row>
     <row r="83" spans="1:14" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="61"/>
+      <c r="A83" s="63"/>
       <c r="B83" s="42">
         <v>10</v>
       </c>
       <c r="C83" s="43" t="e">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="D83" s="43" t="e">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="E83" s="43"/>
@@ -10199,16 +10176,16 @@
       <c r="N83" s="16"/>
     </row>
     <row r="84" spans="1:14" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A84" s="61"/>
+      <c r="A84" s="63"/>
       <c r="B84" s="42">
         <v>12</v>
       </c>
       <c r="C84" s="43" t="e">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="D84" s="43" t="e">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="E84" s="31"/>
@@ -10223,16 +10200,16 @@
       <c r="N84" s="31"/>
     </row>
     <row r="85" spans="1:14" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A85" s="61"/>
+      <c r="A85" s="63"/>
       <c r="B85" s="42">
         <v>16</v>
       </c>
       <c r="C85" s="43" t="e">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="D85" s="43" t="e">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="E85" s="31"/>
@@ -10247,22 +10224,22 @@
       <c r="N85" s="31"/>
     </row>
     <row r="86" spans="1:14" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A86" s="62"/>
+      <c r="A86" s="64"/>
       <c r="B86" s="33" t="s">
         <v>86</v>
       </c>
-      <c r="C86" s="63"/>
-      <c r="D86" s="63"/>
-      <c r="E86" s="63"/>
-      <c r="F86" s="63"/>
-      <c r="G86" s="63"/>
-      <c r="H86" s="63"/>
-      <c r="I86" s="63"/>
-      <c r="J86" s="63"/>
-      <c r="K86" s="63"/>
-      <c r="L86" s="63"/>
-      <c r="M86" s="63"/>
-      <c r="N86" s="63"/>
+      <c r="C86" s="61"/>
+      <c r="D86" s="61"/>
+      <c r="E86" s="61"/>
+      <c r="F86" s="61"/>
+      <c r="G86" s="61"/>
+      <c r="H86" s="61"/>
+      <c r="I86" s="61"/>
+      <c r="J86" s="61"/>
+      <c r="K86" s="61"/>
+      <c r="L86" s="61"/>
+      <c r="M86" s="61"/>
+      <c r="N86" s="61"/>
     </row>
   </sheetData>
   <mergeCells count="21">
@@ -10301,15 +10278,35 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4269BDC4-CFAE-4A4A-95F0-395DE59C8746}">
-  <dimension ref="M10"/>
+  <dimension ref="M10:M14"/>
   <sheetFormatPr defaultRowHeight="22.1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="16384" width="9.140625" style="41"/>
   </cols>
   <sheetData>
     <row r="10" spans="13:13" x14ac:dyDescent="0.3">
-      <c r="M10" s="41" t="s">
+      <c r="M10" s="46" t="s">
         <v>93</v>
+      </c>
+    </row>
+    <row r="11" spans="13:13" x14ac:dyDescent="0.3">
+      <c r="M11" s="41" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="12" spans="13:13" x14ac:dyDescent="0.3">
+      <c r="M12" s="41" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="13" spans="13:13" x14ac:dyDescent="0.3">
+      <c r="M13" s="41" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="14" spans="13:13" x14ac:dyDescent="0.3">
+      <c r="M14" s="41" t="s">
+        <v>102</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Merged L21 and U12 cycles.
</commit_message>
<xml_diff>
--- a/DecompositionLU/docs/statistics.xlsx
+++ b/DecompositionLU/docs/statistics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Maxim\source\repos\practice\SECOND_COURSE\FOR_ITLAB\ArchBenchs\DecompositionLU\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC2A0560-C327-424F-8F5A-116FD11421DC}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19261714-9429-42C2-965A-10FB4931A57B}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-114" yWindow="-114" windowWidth="27602" windowHeight="15027" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4627,7 +4627,7 @@
                   <c:v>4.7108100000000004</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>4.8997400000000004</c:v>
+                  <c:v>5.4617599999999999</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5108,7 +5108,7 @@
                   <c:v>0.39256999999999997</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.30623</c:v>
+                  <c:v>0.34136</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5586,7 +5586,7 @@
                   <c:v>1971</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1895</c:v>
+                  <c:v>1700</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -6287,7 +6287,7 @@
                   <c:v>3.4933100000000001</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>3.4933100000000001</c:v>
+                  <c:v>4.5314500000000004</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -6768,7 +6768,7 @@
                   <c:v>0.29110999999999998</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.21833</c:v>
+                  <c:v>0.28322000000000003</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -7246,7 +7246,7 @@
                   <c:v>598</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>598</c:v>
+                  <c:v>461</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -7616,7 +7616,7 @@
                   <c:v>5.3701999999999996</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>5.5549099999999996</c:v>
+                  <c:v>6.0136599999999998</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -8109,7 +8109,7 @@
                   <c:v>0.44751999999999997</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.34717999999999999</c:v>
+                  <c:v>0.37585000000000002</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -8587,7 +8587,7 @@
                   <c:v>13112</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>12676</c:v>
+                  <c:v>11709</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -35618,13 +35618,13 @@
         <v>13</v>
       </c>
       <c r="C74" s="10">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="D74" s="10">
-        <v>450</v>
+        <v>633</v>
       </c>
       <c r="E74" s="10">
-        <v>1349</v>
+        <v>1101</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
@@ -35635,13 +35635,13 @@
         <v>50</v>
       </c>
       <c r="C75" s="10">
-        <v>598</v>
+        <v>461</v>
       </c>
       <c r="D75" s="10">
-        <v>5232</v>
+        <v>4644</v>
       </c>
       <c r="E75" s="10">
-        <v>12676</v>
+        <v>11709</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
@@ -35652,13 +35652,13 @@
         <v>64</v>
       </c>
       <c r="C76" s="10">
-        <v>720</v>
+        <v>582</v>
       </c>
       <c r="D76" s="10">
-        <v>5682</v>
+        <v>5284</v>
       </c>
       <c r="E76" s="10">
-        <v>14026</v>
+        <v>12810</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
@@ -38181,13 +38181,13 @@
         <v>16</v>
       </c>
       <c r="C98" s="40">
-        <v>598</v>
+        <v>461</v>
       </c>
       <c r="D98" s="24">
-        <v>1895</v>
+        <v>1700</v>
       </c>
       <c r="E98" s="24">
-        <v>12676</v>
+        <v>11709</v>
       </c>
       <c r="F98" s="31"/>
       <c r="G98" s="31"/>
@@ -38497,15 +38497,15 @@
       </c>
       <c r="C108" s="40">
         <f>ROUND(C91/C98,5)</f>
-        <v>3.4933100000000001</v>
+        <v>4.5314500000000004</v>
       </c>
       <c r="D108" s="40">
         <f>ROUND(D91/D98,5)</f>
-        <v>4.8997400000000004</v>
+        <v>5.4617599999999999</v>
       </c>
       <c r="E108" s="40">
         <f>ROUND(E91/E98,5)</f>
-        <v>5.5549099999999996</v>
+        <v>6.0136599999999998</v>
       </c>
       <c r="F108" s="43"/>
       <c r="G108" s="16"/>
@@ -38815,15 +38815,15 @@
       </c>
       <c r="C118" s="40">
         <f t="shared" si="4"/>
-        <v>0.21833</v>
+        <v>0.28322000000000003</v>
       </c>
       <c r="D118" s="40">
         <f t="shared" si="5"/>
-        <v>0.30623</v>
+        <v>0.34136</v>
       </c>
       <c r="E118" s="40">
         <f t="shared" si="6"/>
-        <v>0.34717999999999999</v>
+        <v>0.37585000000000002</v>
       </c>
       <c r="F118" s="31"/>
       <c r="G118" s="31"/>

</xml_diff>

<commit_message>
Rollback, it was a bad idea.
</commit_message>
<xml_diff>
--- a/DecompositionLU/docs/statistics.xlsx
+++ b/DecompositionLU/docs/statistics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Maxim\source\repos\practice\SECOND_COURSE\FOR_ITLAB\ArchBenchs\DecompositionLU\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC2A0560-C327-424F-8F5A-116FD11421DC}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8730C858-ED17-4A5F-A6F0-5B7E2934BBAA}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-114" yWindow="-114" windowWidth="27602" windowHeight="15027" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1005,45 +1005,6 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="18" fillId="5" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1079,6 +1040,45 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -4627,7 +4627,7 @@
                   <c:v>4.7108100000000004</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>4.8997400000000004</c:v>
+                  <c:v>5.4617599999999999</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5108,7 +5108,7 @@
                   <c:v>0.39256999999999997</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.30623</c:v>
+                  <c:v>0.34136</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5586,7 +5586,7 @@
                   <c:v>1971</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1895</c:v>
+                  <c:v>1700</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -6287,7 +6287,7 @@
                   <c:v>3.4933100000000001</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>3.4933100000000001</c:v>
+                  <c:v>4.5314500000000004</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -6768,7 +6768,7 @@
                   <c:v>0.29110999999999998</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.21833</c:v>
+                  <c:v>0.28322000000000003</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -7246,7 +7246,7 @@
                   <c:v>598</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>598</c:v>
+                  <c:v>461</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -7616,7 +7616,7 @@
                   <c:v>5.3701999999999996</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>5.5549099999999996</c:v>
+                  <c:v>5.4314999999999998</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -8109,7 +8109,7 @@
                   <c:v>0.44751999999999997</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.34717999999999999</c:v>
+                  <c:v>0.33946999999999999</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -8587,7 +8587,7 @@
                   <c:v>13112</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>12676</c:v>
+                  <c:v>12964</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -9092,34 +9092,34 @@
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.7688250272826482</c:v>
+                  <c:v>1.7688299999999999</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>3.1615734720416127</c:v>
+                  <c:v>3.1615700000000002</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>4.1524338172502135</c:v>
+                  <c:v>4.1524299999999998</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>5.1728723404255321</c:v>
+                  <c:v>5.1728699999999996</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>5.8939393939393936</c:v>
+                  <c:v>5.8939399999999997</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>6.7770034843205575</c:v>
+                  <c:v>6.7770000000000001</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>7.3786039453717756</c:v>
+                  <c:v>7.3785999999999996</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>7.9517579721995091</c:v>
+                  <c:v>7.9517600000000002</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>8.2695578231292526</c:v>
+                  <c:v>8.2695600000000002</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>9.1143392689784442</c:v>
+                  <c:v>9.1143400000000003</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -9620,34 +9620,34 @@
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.88441251364132412</c:v>
+                  <c:v>0.88441999999999998</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.79039336801040316</c:v>
+                  <c:v>0.79039000000000004</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.69207230287503563</c:v>
+                  <c:v>0.69206999999999996</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.64660904255319152</c:v>
+                  <c:v>0.64661000000000002</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.58939393939393936</c:v>
+                  <c:v>0.58938999999999997</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.56475029036004643</c:v>
+                  <c:v>0.56474999999999997</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.52704313895512678</c:v>
+                  <c:v>0.52703999999999995</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.49698487326246932</c:v>
+                  <c:v>0.49698999999999999</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.45941987906273624</c:v>
+                  <c:v>0.45942</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.45571696344892221</c:v>
+                  <c:v>0.45572000000000001</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -11553,34 +11553,34 @@
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.970216806941498</c:v>
+                  <c:v>1.9702200000000001</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>3.8754067245119308</c:v>
+                  <c:v>3.87541</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5.5921095533094229</c:v>
+                  <c:v>5.5921099999999999</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>7.2291848146795177</c:v>
+                  <c:v>7.2291800000000004</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>8.6001537741525702</c:v>
+                  <c:v>8.6001499999999993</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>10.19719370565619</c:v>
+                  <c:v>10.197190000000001</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>10.873415046491969</c:v>
+                  <c:v>10.873419999999999</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>12.214651979868957</c:v>
+                  <c:v>12.214650000000001</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>12.466201482773659</c:v>
+                  <c:v>12.466200000000001</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>14.049751515482496</c:v>
+                  <c:v>14.04975</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -12084,37 +12084,37 @@
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.9492718384479537</c:v>
+                  <c:v>1.9492700000000001</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>3.7886777435081087</c:v>
+                  <c:v>3.7886799999999998</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5.4156296665007471</c:v>
+                  <c:v>5.4156300000000002</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>6.5149700598802394</c:v>
+                  <c:v>6.5149699999999999</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>7.4953252632614902</c:v>
+                  <c:v>7.49533</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>9.4797112272840423</c:v>
+                  <c:v>9.4797100000000007</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>10.431447746883988</c:v>
+                  <c:v>10.43145</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>11.165518252455652</c:v>
+                  <c:v>11.165520000000001</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>12.281890017739075</c:v>
+                  <c:v>12.281890000000001</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>12.575957727873183</c:v>
+                  <c:v>12.57596</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>11.124744376278118</c:v>
+                  <c:v>11.124739999999999</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -12615,34 +12615,34 @@
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.98510840347074902</c:v>
+                  <c:v>0.98511000000000004</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.9688516811279827</c:v>
+                  <c:v>0.96885250000000001</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.93201825888490386</c:v>
+                  <c:v>0.93201833333333328</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.90364810183493971</c:v>
+                  <c:v>0.90364750000000005</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.86001537741525702</c:v>
+                  <c:v>0.86001499999999997</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.84976614213801582</c:v>
+                  <c:v>0.84976583333333344</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.77667250332085491</c:v>
+                  <c:v>0.77667285714285705</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.76341574874180984</c:v>
+                  <c:v>0.76341562500000004</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.6925667490429811</c:v>
+                  <c:v>0.69256666666666666</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.7024875757741248</c:v>
+                  <c:v>0.70248749999999993</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -13145,34 +13145,34 @@
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.97463591922397685</c:v>
+                  <c:v>0.97463500000000003</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.94716943587702718</c:v>
+                  <c:v>0.94716999999999996</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.90260494441679118</c:v>
+                  <c:v>0.90260499999999999</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.81437125748502992</c:v>
+                  <c:v>0.81437124999999999</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.74953252632614897</c:v>
+                  <c:v>0.749533</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.78997593560700352</c:v>
+                  <c:v>0.78997583333333343</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.74510341049171347</c:v>
+                  <c:v>0.74510357142857142</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.69784489077847822</c:v>
+                  <c:v>0.69784500000000005</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.68232722320772643</c:v>
+                  <c:v>0.68232722222222231</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.62879788639365919</c:v>
+                  <c:v>0.62879799999999997</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -35618,13 +35618,13 @@
         <v>13</v>
       </c>
       <c r="C74" s="10">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="D74" s="10">
-        <v>450</v>
+        <v>633</v>
       </c>
       <c r="E74" s="10">
-        <v>1349</v>
+        <v>1101</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
@@ -35635,13 +35635,13 @@
         <v>50</v>
       </c>
       <c r="C75" s="10">
-        <v>598</v>
+        <v>461</v>
       </c>
       <c r="D75" s="10">
-        <v>5232</v>
+        <v>4644</v>
       </c>
       <c r="E75" s="10">
-        <v>12676</v>
+        <v>11709</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
@@ -35652,13 +35652,13 @@
         <v>64</v>
       </c>
       <c r="C76" s="10">
-        <v>720</v>
+        <v>582</v>
       </c>
       <c r="D76" s="10">
-        <v>5682</v>
+        <v>5284</v>
       </c>
       <c r="E76" s="10">
-        <v>14026</v>
+        <v>12810</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
@@ -35716,18 +35716,11 @@
     </row>
   </sheetData>
   <mergeCells count="32">
-    <mergeCell ref="A57:C57"/>
-    <mergeCell ref="D57:E57"/>
-    <mergeCell ref="B58:E58"/>
-    <mergeCell ref="A60:E60"/>
-    <mergeCell ref="A64:E64"/>
-    <mergeCell ref="B45:E45"/>
-    <mergeCell ref="A47:E47"/>
-    <mergeCell ref="A51:E51"/>
-    <mergeCell ref="D44:E44"/>
-    <mergeCell ref="D31:E31"/>
-    <mergeCell ref="A44:C44"/>
-    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="A70:C70"/>
+    <mergeCell ref="D70:E70"/>
+    <mergeCell ref="B71:E71"/>
+    <mergeCell ref="A72:E72"/>
+    <mergeCell ref="A77:E77"/>
     <mergeCell ref="H24:I24"/>
     <mergeCell ref="G5:H8"/>
     <mergeCell ref="B42:E42"/>
@@ -35743,11 +35736,18 @@
     <mergeCell ref="B19:E19"/>
     <mergeCell ref="A21:E21"/>
     <mergeCell ref="A25:E25"/>
-    <mergeCell ref="A70:C70"/>
-    <mergeCell ref="D70:E70"/>
-    <mergeCell ref="B71:E71"/>
-    <mergeCell ref="A72:E72"/>
-    <mergeCell ref="A77:E77"/>
+    <mergeCell ref="B45:E45"/>
+    <mergeCell ref="A47:E47"/>
+    <mergeCell ref="A51:E51"/>
+    <mergeCell ref="D44:E44"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="A44:C44"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="A57:C57"/>
+    <mergeCell ref="D57:E57"/>
+    <mergeCell ref="B58:E58"/>
+    <mergeCell ref="A60:E60"/>
+    <mergeCell ref="A64:E64"/>
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <hyperlinks>
@@ -35811,14 +35811,14 @@
       <c r="Z1" s="35"/>
     </row>
     <row r="2" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="73" t="s">
+      <c r="A2" s="82" t="s">
         <v>85</v>
       </c>
-      <c r="B2" s="65" t="s">
+      <c r="B2" s="77" t="s">
         <v>78</v>
       </c>
-      <c r="C2" s="66"/>
-      <c r="D2" s="67"/>
+      <c r="C2" s="78"/>
+      <c r="D2" s="79"/>
       <c r="E2" s="31"/>
       <c r="F2" s="31"/>
       <c r="G2" s="31"/>
@@ -35843,7 +35843,7 @@
       <c r="Z2" s="30"/>
     </row>
     <row r="3" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="73"/>
+      <c r="A3" s="82"/>
       <c r="B3" s="29" t="s">
         <v>77</v>
       </c>
@@ -35877,7 +35877,7 @@
       <c r="Z3" s="30"/>
     </row>
     <row r="4" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="73"/>
+      <c r="A4" s="82"/>
       <c r="B4" s="15">
         <v>1</v>
       </c>
@@ -35911,7 +35911,7 @@
       <c r="Z4" s="30"/>
     </row>
     <row r="5" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="73"/>
+      <c r="A5" s="82"/>
       <c r="B5" s="15">
         <v>2</v>
       </c>
@@ -35945,7 +35945,7 @@
       <c r="Z5" s="30"/>
     </row>
     <row r="6" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="73"/>
+      <c r="A6" s="82"/>
       <c r="B6" s="15">
         <v>4</v>
       </c>
@@ -35968,7 +35968,7 @@
       <c r="O6" s="38"/>
     </row>
     <row r="7" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="73"/>
+      <c r="A7" s="82"/>
       <c r="B7" s="15">
         <v>6</v>
       </c>
@@ -35991,7 +35991,7 @@
       <c r="O7" s="38"/>
     </row>
     <row r="8" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="73"/>
+      <c r="A8" s="82"/>
       <c r="B8" s="15">
         <v>8</v>
       </c>
@@ -36014,7 +36014,7 @@
       <c r="O8" s="38"/>
     </row>
     <row r="9" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="73"/>
+      <c r="A9" s="82"/>
       <c r="B9" s="15">
         <v>10</v>
       </c>
@@ -36037,7 +36037,7 @@
       <c r="O9" s="38"/>
     </row>
     <row r="10" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="73"/>
+      <c r="A10" s="82"/>
       <c r="B10" s="15">
         <v>12</v>
       </c>
@@ -36060,7 +36060,7 @@
       <c r="O10" s="38"/>
     </row>
     <row r="11" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="73"/>
+      <c r="A11" s="82"/>
       <c r="B11" s="15">
         <v>16</v>
       </c>
@@ -36085,37 +36085,37 @@
       <c r="Q11" s="27"/>
     </row>
     <row r="12" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="73"/>
+      <c r="A12" s="82"/>
       <c r="B12" s="33" t="s">
         <v>86</v>
       </c>
-      <c r="C12" s="74" t="s">
+      <c r="C12" s="80" t="s">
         <v>81</v>
       </c>
-      <c r="D12" s="74"/>
-      <c r="E12" s="74"/>
-      <c r="F12" s="74"/>
-      <c r="G12" s="74"/>
-      <c r="H12" s="74"/>
-      <c r="I12" s="74"/>
-      <c r="J12" s="74"/>
-      <c r="K12" s="74"/>
-      <c r="L12" s="74"/>
-      <c r="M12" s="74"/>
-      <c r="N12" s="70"/>
+      <c r="D12" s="80"/>
+      <c r="E12" s="80"/>
+      <c r="F12" s="80"/>
+      <c r="G12" s="80"/>
+      <c r="H12" s="80"/>
+      <c r="I12" s="80"/>
+      <c r="J12" s="80"/>
+      <c r="K12" s="80"/>
+      <c r="L12" s="80"/>
+      <c r="M12" s="80"/>
+      <c r="N12" s="81"/>
       <c r="O12" s="39"/>
       <c r="P12" s="23"/>
       <c r="Q12" s="23"/>
     </row>
     <row r="13" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="73" t="s">
+      <c r="A13" s="82" t="s">
         <v>87</v>
       </c>
-      <c r="B13" s="65" t="s">
+      <c r="B13" s="77" t="s">
         <v>78</v>
       </c>
-      <c r="C13" s="66"/>
-      <c r="D13" s="67"/>
+      <c r="C13" s="78"/>
+      <c r="D13" s="79"/>
       <c r="E13" s="32"/>
       <c r="F13" s="31"/>
       <c r="G13" s="31"/>
@@ -36131,7 +36131,7 @@
       <c r="Q13" s="23"/>
     </row>
     <row r="14" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="73"/>
+      <c r="A14" s="82"/>
       <c r="B14" s="13" t="s">
         <v>77</v>
       </c>
@@ -36156,7 +36156,7 @@
       <c r="Q14" s="23"/>
     </row>
     <row r="15" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="73"/>
+      <c r="A15" s="82"/>
       <c r="B15" s="15">
         <v>1</v>
       </c>
@@ -36181,7 +36181,7 @@
       <c r="Q15" s="27"/>
     </row>
     <row r="16" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="73"/>
+      <c r="A16" s="82"/>
       <c r="B16" s="15">
         <v>2</v>
       </c>
@@ -36206,7 +36206,7 @@
       <c r="Q16" s="23"/>
     </row>
     <row r="17" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="73"/>
+      <c r="A17" s="82"/>
       <c r="B17" s="15">
         <v>4</v>
       </c>
@@ -36231,7 +36231,7 @@
       <c r="Q17" s="23"/>
     </row>
     <row r="18" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="73"/>
+      <c r="A18" s="82"/>
       <c r="B18" s="15">
         <v>6</v>
       </c>
@@ -36256,7 +36256,7 @@
       <c r="Q18" s="23"/>
     </row>
     <row r="19" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="73"/>
+      <c r="A19" s="82"/>
       <c r="B19" s="15">
         <v>8</v>
       </c>
@@ -36279,7 +36279,7 @@
       <c r="O19" s="38"/>
     </row>
     <row r="20" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="73"/>
+      <c r="A20" s="82"/>
       <c r="B20" s="15">
         <v>10</v>
       </c>
@@ -36302,7 +36302,7 @@
       <c r="O20" s="38"/>
     </row>
     <row r="21" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="73"/>
+      <c r="A21" s="82"/>
       <c r="B21" s="15">
         <v>12</v>
       </c>
@@ -36325,41 +36325,41 @@
       <c r="O21" s="38"/>
     </row>
     <row r="22" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="73"/>
-      <c r="B22" s="75" t="s">
+      <c r="A22" s="82"/>
+      <c r="B22" s="83" t="s">
         <v>86</v>
       </c>
-      <c r="C22" s="76" t="s">
+      <c r="C22" s="84" t="s">
         <v>88</v>
       </c>
-      <c r="D22" s="76"/>
-      <c r="E22" s="76"/>
-      <c r="F22" s="76"/>
-      <c r="G22" s="76"/>
-      <c r="H22" s="76"/>
-      <c r="I22" s="76"/>
-      <c r="J22" s="76"/>
-      <c r="K22" s="76"/>
-      <c r="L22" s="76"/>
-      <c r="M22" s="76"/>
-      <c r="N22" s="77"/>
+      <c r="D22" s="84"/>
+      <c r="E22" s="84"/>
+      <c r="F22" s="84"/>
+      <c r="G22" s="84"/>
+      <c r="H22" s="84"/>
+      <c r="I22" s="84"/>
+      <c r="J22" s="84"/>
+      <c r="K22" s="84"/>
+      <c r="L22" s="84"/>
+      <c r="M22" s="84"/>
+      <c r="N22" s="85"/>
       <c r="O22" s="38"/>
     </row>
     <row r="23" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="73"/>
-      <c r="B23" s="75"/>
-      <c r="C23" s="76"/>
-      <c r="D23" s="76"/>
-      <c r="E23" s="76"/>
-      <c r="F23" s="76"/>
-      <c r="G23" s="76"/>
-      <c r="H23" s="76"/>
-      <c r="I23" s="76"/>
-      <c r="J23" s="76"/>
-      <c r="K23" s="76"/>
-      <c r="L23" s="76"/>
-      <c r="M23" s="76"/>
-      <c r="N23" s="77"/>
+      <c r="A23" s="82"/>
+      <c r="B23" s="83"/>
+      <c r="C23" s="84"/>
+      <c r="D23" s="84"/>
+      <c r="E23" s="84"/>
+      <c r="F23" s="84"/>
+      <c r="G23" s="84"/>
+      <c r="H23" s="84"/>
+      <c r="I23" s="84"/>
+      <c r="J23" s="84"/>
+      <c r="K23" s="84"/>
+      <c r="L23" s="84"/>
+      <c r="M23" s="84"/>
+      <c r="N23" s="85"/>
       <c r="O23" s="38"/>
     </row>
     <row r="24" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -36384,14 +36384,14 @@
       <c r="O24" s="38"/>
     </row>
     <row r="25" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="81" t="s">
+      <c r="A25" s="68" t="s">
         <v>85</v>
       </c>
-      <c r="B25" s="65" t="s">
+      <c r="B25" s="77" t="s">
         <v>78</v>
       </c>
-      <c r="C25" s="66"/>
-      <c r="D25" s="67"/>
+      <c r="C25" s="78"/>
+      <c r="D25" s="79"/>
       <c r="E25" s="31"/>
       <c r="F25" s="31"/>
       <c r="G25" s="31"/>
@@ -36405,7 +36405,7 @@
       <c r="O25" s="27"/>
     </row>
     <row r="26" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="82"/>
+      <c r="A26" s="69"/>
       <c r="B26" s="42" t="s">
         <v>77</v>
       </c>
@@ -36428,7 +36428,7 @@
       <c r="O26" s="27"/>
     </row>
     <row r="27" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="82"/>
+      <c r="A27" s="69"/>
       <c r="B27" s="15">
         <v>1</v>
       </c>
@@ -36451,7 +36451,7 @@
       <c r="O27" s="27"/>
     </row>
     <row r="28" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="82"/>
+      <c r="A28" s="69"/>
       <c r="B28" s="15">
         <v>2</v>
       </c>
@@ -36474,7 +36474,7 @@
       <c r="O28" s="27"/>
     </row>
     <row r="29" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="82"/>
+      <c r="A29" s="69"/>
       <c r="B29" s="15">
         <v>4</v>
       </c>
@@ -36497,7 +36497,7 @@
       <c r="O29" s="27"/>
     </row>
     <row r="30" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="82"/>
+      <c r="A30" s="69"/>
       <c r="B30" s="15">
         <v>6</v>
       </c>
@@ -36520,7 +36520,7 @@
       <c r="O30" s="27"/>
     </row>
     <row r="31" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="82"/>
+      <c r="A31" s="69"/>
       <c r="B31" s="15">
         <v>8</v>
       </c>
@@ -36543,7 +36543,7 @@
       <c r="O31" s="27"/>
     </row>
     <row r="32" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="82"/>
+      <c r="A32" s="69"/>
       <c r="B32" s="15">
         <v>10</v>
       </c>
@@ -36566,7 +36566,7 @@
       <c r="O32" s="27"/>
     </row>
     <row r="33" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="82"/>
+      <c r="A33" s="69"/>
       <c r="B33" s="15">
         <v>12</v>
       </c>
@@ -36589,7 +36589,7 @@
       <c r="O33" s="27"/>
     </row>
     <row r="34" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="82"/>
+      <c r="A34" s="69"/>
       <c r="B34" s="15">
         <v>16</v>
       </c>
@@ -36612,12 +36612,12 @@
       <c r="O34" s="27"/>
     </row>
     <row r="35" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="82"/>
-      <c r="B35" s="65" t="s">
+      <c r="A35" s="69"/>
+      <c r="B35" s="77" t="s">
         <v>96</v>
       </c>
-      <c r="C35" s="66"/>
-      <c r="D35" s="67"/>
+      <c r="C35" s="78"/>
+      <c r="D35" s="79"/>
       <c r="E35" s="31"/>
       <c r="F35" s="31"/>
       <c r="G35" s="31"/>
@@ -36631,7 +36631,7 @@
       <c r="O35" s="27"/>
     </row>
     <row r="36" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="82"/>
+      <c r="A36" s="69"/>
       <c r="B36" s="42" t="s">
         <v>77</v>
       </c>
@@ -36655,7 +36655,7 @@
       <c r="P36" s="1"/>
     </row>
     <row r="37" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="82"/>
+      <c r="A37" s="69"/>
       <c r="B37" s="42">
         <v>1</v>
       </c>
@@ -36681,7 +36681,7 @@
       <c r="P37" s="1"/>
     </row>
     <row r="38" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="82"/>
+      <c r="A38" s="69"/>
       <c r="B38" s="42">
         <v>2</v>
       </c>
@@ -36707,7 +36707,7 @@
       <c r="P38" s="1"/>
     </row>
     <row r="39" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="82"/>
+      <c r="A39" s="69"/>
       <c r="B39" s="42">
         <v>4</v>
       </c>
@@ -36733,7 +36733,7 @@
       <c r="P39" s="1"/>
     </row>
     <row r="40" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="82"/>
+      <c r="A40" s="69"/>
       <c r="B40" s="42">
         <v>6</v>
       </c>
@@ -36759,7 +36759,7 @@
       <c r="P40" s="1"/>
     </row>
     <row r="41" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="82"/>
+      <c r="A41" s="69"/>
       <c r="B41" s="42">
         <v>8</v>
       </c>
@@ -36785,7 +36785,7 @@
       <c r="P41" s="1"/>
     </row>
     <row r="42" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="82"/>
+      <c r="A42" s="69"/>
       <c r="B42" s="42">
         <v>10</v>
       </c>
@@ -36811,7 +36811,7 @@
       <c r="P42" s="1"/>
     </row>
     <row r="43" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="82"/>
+      <c r="A43" s="69"/>
       <c r="B43" s="42">
         <v>12</v>
       </c>
@@ -36837,7 +36837,7 @@
       <c r="P43" s="1"/>
     </row>
     <row r="44" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="82"/>
+      <c r="A44" s="69"/>
       <c r="B44" s="42">
         <v>16</v>
       </c>
@@ -36863,12 +36863,12 @@
       <c r="P44" s="1"/>
     </row>
     <row r="45" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="82"/>
-      <c r="B45" s="65" t="s">
+      <c r="A45" s="69"/>
+      <c r="B45" s="77" t="s">
         <v>97</v>
       </c>
-      <c r="C45" s="66"/>
-      <c r="D45" s="67"/>
+      <c r="C45" s="78"/>
+      <c r="D45" s="79"/>
       <c r="E45" s="43"/>
       <c r="F45" s="43"/>
       <c r="G45" s="43"/>
@@ -36883,7 +36883,7 @@
       <c r="P45" s="1"/>
     </row>
     <row r="46" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="82"/>
+      <c r="A46" s="69"/>
       <c r="B46" s="42" t="s">
         <v>77</v>
       </c>
@@ -36907,7 +36907,7 @@
       <c r="P46" s="1"/>
     </row>
     <row r="47" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="82"/>
+      <c r="A47" s="69"/>
       <c r="B47" s="42">
         <v>1</v>
       </c>
@@ -36933,7 +36933,7 @@
       <c r="P47" s="1"/>
     </row>
     <row r="48" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="82"/>
+      <c r="A48" s="69"/>
       <c r="B48" s="42">
         <v>2</v>
       </c>
@@ -36959,7 +36959,7 @@
       <c r="P48" s="1"/>
     </row>
     <row r="49" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="82"/>
+      <c r="A49" s="69"/>
       <c r="B49" s="42">
         <v>4</v>
       </c>
@@ -36985,7 +36985,7 @@
       <c r="P49" s="1"/>
     </row>
     <row r="50" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="82"/>
+      <c r="A50" s="69"/>
       <c r="B50" s="42">
         <v>6</v>
       </c>
@@ -37011,7 +37011,7 @@
       <c r="P50" s="1"/>
     </row>
     <row r="51" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="82"/>
+      <c r="A51" s="69"/>
       <c r="B51" s="42">
         <v>8</v>
       </c>
@@ -37036,7 +37036,7 @@
       <c r="O51" s="1"/>
     </row>
     <row r="52" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="82"/>
+      <c r="A52" s="69"/>
       <c r="B52" s="42">
         <v>10</v>
       </c>
@@ -37061,7 +37061,7 @@
       <c r="O52" s="1"/>
     </row>
     <row r="53" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="82"/>
+      <c r="A53" s="69"/>
       <c r="B53" s="42">
         <v>12</v>
       </c>
@@ -37086,7 +37086,7 @@
       <c r="O53" s="1"/>
     </row>
     <row r="54" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="82"/>
+      <c r="A54" s="69"/>
       <c r="B54" s="42">
         <v>16</v>
       </c>
@@ -37111,40 +37111,40 @@
       <c r="O54" s="1"/>
     </row>
     <row r="55" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="82"/>
+      <c r="A55" s="69"/>
       <c r="B55" s="46" t="s">
         <v>86</v>
       </c>
-      <c r="C55" s="86" t="s">
+      <c r="C55" s="73" t="s">
         <v>102</v>
       </c>
-      <c r="D55" s="86"/>
-      <c r="E55" s="86"/>
-      <c r="F55" s="86"/>
-      <c r="G55" s="86"/>
-      <c r="H55" s="86"/>
-      <c r="I55" s="86"/>
-      <c r="J55" s="86"/>
-      <c r="K55" s="86"/>
-      <c r="L55" s="86"/>
-      <c r="M55" s="86"/>
-      <c r="N55" s="86"/>
+      <c r="D55" s="73"/>
+      <c r="E55" s="73"/>
+      <c r="F55" s="73"/>
+      <c r="G55" s="73"/>
+      <c r="H55" s="73"/>
+      <c r="I55" s="73"/>
+      <c r="J55" s="73"/>
+      <c r="K55" s="73"/>
+      <c r="L55" s="73"/>
+      <c r="M55" s="73"/>
+      <c r="N55" s="73"/>
     </row>
     <row r="56" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="87" t="s">
+      <c r="A56" s="74" t="s">
         <v>103</v>
       </c>
-      <c r="B56" s="88"/>
-      <c r="C56" s="88"/>
-      <c r="D56" s="88"/>
-      <c r="E56" s="88"/>
-      <c r="F56" s="88"/>
-      <c r="G56" s="88"/>
-      <c r="H56" s="88"/>
-      <c r="I56" s="88"/>
-      <c r="J56" s="88"/>
-      <c r="K56" s="88"/>
-      <c r="L56" s="89"/>
+      <c r="B56" s="75"/>
+      <c r="C56" s="75"/>
+      <c r="D56" s="75"/>
+      <c r="E56" s="75"/>
+      <c r="F56" s="75"/>
+      <c r="G56" s="75"/>
+      <c r="H56" s="75"/>
+      <c r="I56" s="75"/>
+      <c r="J56" s="75"/>
+      <c r="K56" s="75"/>
+      <c r="L56" s="76"/>
       <c r="M56" s="55" t="s">
         <v>90</v>
       </c>
@@ -37152,14 +37152,14 @@
       <c r="O56" s="30"/>
     </row>
     <row r="57" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="81" t="s">
+      <c r="A57" s="68" t="s">
         <v>85</v>
       </c>
-      <c r="B57" s="65" t="s">
+      <c r="B57" s="77" t="s">
         <v>78</v>
       </c>
-      <c r="C57" s="66"/>
-      <c r="D57" s="67"/>
+      <c r="C57" s="78"/>
+      <c r="D57" s="79"/>
       <c r="E57" s="31"/>
       <c r="F57" s="31"/>
       <c r="G57" s="31"/>
@@ -37173,7 +37173,7 @@
       <c r="O57" s="30"/>
     </row>
     <row r="58" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="82"/>
+      <c r="A58" s="69"/>
       <c r="B58" s="42" t="s">
         <v>77</v>
       </c>
@@ -37196,7 +37196,7 @@
       <c r="O58" s="30"/>
     </row>
     <row r="59" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="82"/>
+      <c r="A59" s="69"/>
       <c r="B59" s="15">
         <v>1</v>
       </c>
@@ -37219,7 +37219,7 @@
       <c r="O59" s="30"/>
     </row>
     <row r="60" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="82"/>
+      <c r="A60" s="69"/>
       <c r="B60" s="15">
         <v>2</v>
       </c>
@@ -37242,7 +37242,7 @@
       <c r="O60" s="30"/>
     </row>
     <row r="61" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="82"/>
+      <c r="A61" s="69"/>
       <c r="B61" s="15">
         <v>4</v>
       </c>
@@ -37265,7 +37265,7 @@
       <c r="O61" s="30"/>
     </row>
     <row r="62" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="82"/>
+      <c r="A62" s="69"/>
       <c r="B62" s="15">
         <v>6</v>
       </c>
@@ -37288,7 +37288,7 @@
       <c r="O62" s="30"/>
     </row>
     <row r="63" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="82"/>
+      <c r="A63" s="69"/>
       <c r="B63" s="15">
         <v>8</v>
       </c>
@@ -37311,7 +37311,7 @@
       <c r="O63" s="30"/>
     </row>
     <row r="64" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="82"/>
+      <c r="A64" s="69"/>
       <c r="B64" s="15">
         <v>10</v>
       </c>
@@ -37334,7 +37334,7 @@
       <c r="O64" s="30"/>
     </row>
     <row r="65" spans="1:15" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="82"/>
+      <c r="A65" s="69"/>
       <c r="B65" s="15">
         <v>12</v>
       </c>
@@ -37357,7 +37357,7 @@
       <c r="O65" s="30"/>
     </row>
     <row r="66" spans="1:15" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="82"/>
+      <c r="A66" s="69"/>
       <c r="B66" s="15">
         <v>16</v>
       </c>
@@ -37380,12 +37380,12 @@
       <c r="O66" s="30"/>
     </row>
     <row r="67" spans="1:15" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="82"/>
-      <c r="B67" s="65" t="s">
+      <c r="A67" s="69"/>
+      <c r="B67" s="77" t="s">
         <v>96</v>
       </c>
-      <c r="C67" s="66"/>
-      <c r="D67" s="67"/>
+      <c r="C67" s="78"/>
+      <c r="D67" s="79"/>
       <c r="E67" s="31"/>
       <c r="F67" s="31"/>
       <c r="G67" s="31"/>
@@ -37399,7 +37399,7 @@
       <c r="O67" s="30"/>
     </row>
     <row r="68" spans="1:15" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="82"/>
+      <c r="A68" s="69"/>
       <c r="B68" s="42" t="s">
         <v>77</v>
       </c>
@@ -37422,7 +37422,7 @@
       <c r="O68" s="30"/>
     </row>
     <row r="69" spans="1:15" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="82"/>
+      <c r="A69" s="69"/>
       <c r="B69" s="42">
         <v>1</v>
       </c>
@@ -37447,7 +37447,7 @@
       <c r="O69" s="30"/>
     </row>
     <row r="70" spans="1:15" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="82"/>
+      <c r="A70" s="69"/>
       <c r="B70" s="42">
         <v>2</v>
       </c>
@@ -37472,7 +37472,7 @@
       <c r="O70" s="30"/>
     </row>
     <row r="71" spans="1:15" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="82"/>
+      <c r="A71" s="69"/>
       <c r="B71" s="42">
         <v>4</v>
       </c>
@@ -37497,7 +37497,7 @@
       <c r="O71" s="30"/>
     </row>
     <row r="72" spans="1:15" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="82"/>
+      <c r="A72" s="69"/>
       <c r="B72" s="42">
         <v>6</v>
       </c>
@@ -37522,7 +37522,7 @@
       <c r="O72" s="30"/>
     </row>
     <row r="73" spans="1:15" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="82"/>
+      <c r="A73" s="69"/>
       <c r="B73" s="42">
         <v>8</v>
       </c>
@@ -37547,7 +37547,7 @@
       <c r="O73" s="30"/>
     </row>
     <row r="74" spans="1:15" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A74" s="82"/>
+      <c r="A74" s="69"/>
       <c r="B74" s="42">
         <v>10</v>
       </c>
@@ -37572,7 +37572,7 @@
       <c r="O74" s="30"/>
     </row>
     <row r="75" spans="1:15" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A75" s="82"/>
+      <c r="A75" s="69"/>
       <c r="B75" s="42">
         <v>12</v>
       </c>
@@ -37597,7 +37597,7 @@
       <c r="O75" s="30"/>
     </row>
     <row r="76" spans="1:15" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="82"/>
+      <c r="A76" s="69"/>
       <c r="B76" s="42">
         <v>16</v>
       </c>
@@ -37622,12 +37622,12 @@
       <c r="O76" s="30"/>
     </row>
     <row r="77" spans="1:15" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="82"/>
-      <c r="B77" s="65" t="s">
+      <c r="A77" s="69"/>
+      <c r="B77" s="77" t="s">
         <v>97</v>
       </c>
-      <c r="C77" s="66"/>
-      <c r="D77" s="67"/>
+      <c r="C77" s="78"/>
+      <c r="D77" s="79"/>
       <c r="E77" s="43"/>
       <c r="F77" s="43"/>
       <c r="G77" s="43"/>
@@ -37641,7 +37641,7 @@
       <c r="O77" s="30"/>
     </row>
     <row r="78" spans="1:15" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A78" s="82"/>
+      <c r="A78" s="69"/>
       <c r="B78" s="42" t="s">
         <v>77</v>
       </c>
@@ -37664,7 +37664,7 @@
       <c r="O78" s="30"/>
     </row>
     <row r="79" spans="1:15" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A79" s="82"/>
+      <c r="A79" s="69"/>
       <c r="B79" s="42">
         <v>1</v>
       </c>
@@ -37689,7 +37689,7 @@
       <c r="O79" s="30"/>
     </row>
     <row r="80" spans="1:15" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A80" s="82"/>
+      <c r="A80" s="69"/>
       <c r="B80" s="42">
         <v>2</v>
       </c>
@@ -37714,7 +37714,7 @@
       <c r="O80" s="30"/>
     </row>
     <row r="81" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="82"/>
+      <c r="A81" s="69"/>
       <c r="B81" s="42">
         <v>4</v>
       </c>
@@ -37739,7 +37739,7 @@
       <c r="O81" s="30"/>
     </row>
     <row r="82" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A82" s="82"/>
+      <c r="A82" s="69"/>
       <c r="B82" s="42">
         <v>6</v>
       </c>
@@ -37764,7 +37764,7 @@
       <c r="O82" s="30"/>
     </row>
     <row r="83" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="82"/>
+      <c r="A83" s="69"/>
       <c r="B83" s="42">
         <v>8</v>
       </c>
@@ -37789,7 +37789,7 @@
       <c r="O83" s="30"/>
     </row>
     <row r="84" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A84" s="82"/>
+      <c r="A84" s="69"/>
       <c r="B84" s="42">
         <v>10</v>
       </c>
@@ -37814,7 +37814,7 @@
       <c r="O84" s="30"/>
     </row>
     <row r="85" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A85" s="82"/>
+      <c r="A85" s="69"/>
       <c r="B85" s="42">
         <v>12</v>
       </c>
@@ -37839,7 +37839,7 @@
       <c r="O85" s="30"/>
     </row>
     <row r="86" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A86" s="82"/>
+      <c r="A86" s="69"/>
       <c r="B86" s="42">
         <v>16</v>
       </c>
@@ -37864,24 +37864,24 @@
       <c r="O86" s="30"/>
     </row>
     <row r="87" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A87" s="82"/>
+      <c r="A87" s="69"/>
       <c r="B87" s="46" t="s">
         <v>86</v>
       </c>
-      <c r="C87" s="83" t="s">
+      <c r="C87" s="70" t="s">
         <v>106</v>
       </c>
-      <c r="D87" s="84"/>
-      <c r="E87" s="84"/>
-      <c r="F87" s="84"/>
-      <c r="G87" s="84"/>
-      <c r="H87" s="84"/>
-      <c r="I87" s="84"/>
-      <c r="J87" s="84"/>
-      <c r="K87" s="84"/>
-      <c r="L87" s="84"/>
-      <c r="M87" s="84"/>
-      <c r="N87" s="85"/>
+      <c r="D87" s="71"/>
+      <c r="E87" s="71"/>
+      <c r="F87" s="71"/>
+      <c r="G87" s="71"/>
+      <c r="H87" s="71"/>
+      <c r="I87" s="71"/>
+      <c r="J87" s="71"/>
+      <c r="K87" s="71"/>
+      <c r="L87" s="71"/>
+      <c r="M87" s="71"/>
+      <c r="N87" s="72"/>
     </row>
     <row r="88" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A88" s="52" t="s">
@@ -37900,25 +37900,25 @@
       <c r="L88" s="53"/>
       <c r="M88" s="53"/>
       <c r="N88" s="53"/>
-      <c r="O88" s="78" t="s">
+      <c r="O88" s="65" t="s">
         <v>112</v>
       </c>
-      <c r="P88" s="79"/>
-      <c r="Q88" s="79"/>
-      <c r="R88" s="79"/>
-      <c r="S88" s="79"/>
-      <c r="T88" s="80"/>
+      <c r="P88" s="66"/>
+      <c r="Q88" s="66"/>
+      <c r="R88" s="66"/>
+      <c r="S88" s="66"/>
+      <c r="T88" s="67"/>
     </row>
     <row r="89" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A89" s="73" t="s">
+      <c r="A89" s="82" t="s">
         <v>85</v>
       </c>
-      <c r="B89" s="65" t="s">
+      <c r="B89" s="77" t="s">
         <v>78</v>
       </c>
-      <c r="C89" s="66"/>
-      <c r="D89" s="66"/>
-      <c r="E89" s="67"/>
+      <c r="C89" s="78"/>
+      <c r="D89" s="78"/>
+      <c r="E89" s="79"/>
       <c r="F89" s="31"/>
       <c r="G89" s="31"/>
       <c r="H89" s="31"/>
@@ -37936,7 +37936,7 @@
       <c r="T89" s="31"/>
     </row>
     <row r="90" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A90" s="73"/>
+      <c r="A90" s="82"/>
       <c r="B90" s="42" t="s">
         <v>77</v>
       </c>
@@ -37966,7 +37966,7 @@
       <c r="T90" s="31"/>
     </row>
     <row r="91" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A91" s="73"/>
+      <c r="A91" s="82"/>
       <c r="B91" s="15">
         <v>1</v>
       </c>
@@ -37996,7 +37996,7 @@
       <c r="T91" s="31"/>
     </row>
     <row r="92" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A92" s="73"/>
+      <c r="A92" s="82"/>
       <c r="B92" s="15">
         <v>2</v>
       </c>
@@ -38026,7 +38026,7 @@
       <c r="T92" s="31"/>
     </row>
     <row r="93" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A93" s="73"/>
+      <c r="A93" s="82"/>
       <c r="B93" s="15">
         <v>4</v>
       </c>
@@ -38056,7 +38056,7 @@
       <c r="T93" s="31"/>
     </row>
     <row r="94" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A94" s="73"/>
+      <c r="A94" s="82"/>
       <c r="B94" s="15">
         <v>6</v>
       </c>
@@ -38086,7 +38086,7 @@
       <c r="T94" s="31"/>
     </row>
     <row r="95" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A95" s="73"/>
+      <c r="A95" s="82"/>
       <c r="B95" s="15">
         <v>8</v>
       </c>
@@ -38116,7 +38116,7 @@
       <c r="T95" s="31"/>
     </row>
     <row r="96" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A96" s="73"/>
+      <c r="A96" s="82"/>
       <c r="B96" s="15">
         <v>10</v>
       </c>
@@ -38146,7 +38146,7 @@
       <c r="T96" s="31"/>
     </row>
     <row r="97" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A97" s="73"/>
+      <c r="A97" s="82"/>
       <c r="B97" s="15">
         <v>12</v>
       </c>
@@ -38176,18 +38176,18 @@
       <c r="T97" s="31"/>
     </row>
     <row r="98" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A98" s="73"/>
+      <c r="A98" s="82"/>
       <c r="B98" s="15">
         <v>16</v>
       </c>
       <c r="C98" s="40">
-        <v>598</v>
+        <v>461</v>
       </c>
       <c r="D98" s="24">
-        <v>1895</v>
+        <v>1700</v>
       </c>
       <c r="E98" s="24">
-        <v>12676</v>
+        <v>12964</v>
       </c>
       <c r="F98" s="31"/>
       <c r="G98" s="31"/>
@@ -38206,13 +38206,13 @@
       <c r="T98" s="31"/>
     </row>
     <row r="99" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A99" s="73"/>
-      <c r="B99" s="65" t="s">
+      <c r="A99" s="82"/>
+      <c r="B99" s="77" t="s">
         <v>96</v>
       </c>
-      <c r="C99" s="66"/>
-      <c r="D99" s="66"/>
-      <c r="E99" s="67"/>
+      <c r="C99" s="78"/>
+      <c r="D99" s="78"/>
+      <c r="E99" s="79"/>
       <c r="F99" s="31"/>
       <c r="G99" s="31"/>
       <c r="H99" s="31"/>
@@ -38230,7 +38230,7 @@
       <c r="T99" s="31"/>
     </row>
     <row r="100" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A100" s="73"/>
+      <c r="A100" s="82"/>
       <c r="B100" s="42" t="s">
         <v>77</v>
       </c>
@@ -38260,7 +38260,7 @@
       <c r="T100" s="16"/>
     </row>
     <row r="101" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A101" s="73"/>
+      <c r="A101" s="82"/>
       <c r="B101" s="42">
         <v>1</v>
       </c>
@@ -38293,7 +38293,7 @@
       <c r="T101" s="16"/>
     </row>
     <row r="102" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A102" s="73"/>
+      <c r="A102" s="82"/>
       <c r="B102" s="42">
         <v>2</v>
       </c>
@@ -38326,7 +38326,7 @@
       <c r="T102" s="16"/>
     </row>
     <row r="103" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A103" s="73"/>
+      <c r="A103" s="82"/>
       <c r="B103" s="42">
         <v>4</v>
       </c>
@@ -38359,7 +38359,7 @@
       <c r="T103" s="16"/>
     </row>
     <row r="104" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A104" s="73"/>
+      <c r="A104" s="82"/>
       <c r="B104" s="42">
         <v>6</v>
       </c>
@@ -38392,7 +38392,7 @@
       <c r="T104" s="16"/>
     </row>
     <row r="105" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A105" s="73"/>
+      <c r="A105" s="82"/>
       <c r="B105" s="42">
         <v>8</v>
       </c>
@@ -38425,7 +38425,7 @@
       <c r="T105" s="16"/>
     </row>
     <row r="106" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A106" s="73"/>
+      <c r="A106" s="82"/>
       <c r="B106" s="42">
         <v>10</v>
       </c>
@@ -38458,7 +38458,7 @@
       <c r="T106" s="16"/>
     </row>
     <row r="107" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A107" s="73"/>
+      <c r="A107" s="82"/>
       <c r="B107" s="42">
         <v>12</v>
       </c>
@@ -38491,21 +38491,21 @@
       <c r="T107" s="16"/>
     </row>
     <row r="108" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A108" s="73"/>
+      <c r="A108" s="82"/>
       <c r="B108" s="42">
         <v>16</v>
       </c>
       <c r="C108" s="40">
         <f>ROUND(C91/C98,5)</f>
-        <v>3.4933100000000001</v>
+        <v>4.5314500000000004</v>
       </c>
       <c r="D108" s="40">
         <f>ROUND(D91/D98,5)</f>
-        <v>4.8997400000000004</v>
+        <v>5.4617599999999999</v>
       </c>
       <c r="E108" s="40">
         <f>ROUND(E91/E98,5)</f>
-        <v>5.5549099999999996</v>
+        <v>5.4314999999999998</v>
       </c>
       <c r="F108" s="43"/>
       <c r="G108" s="16"/>
@@ -38524,13 +38524,13 @@
       <c r="T108" s="16"/>
     </row>
     <row r="109" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A109" s="73"/>
-      <c r="B109" s="65" t="s">
+      <c r="A109" s="82"/>
+      <c r="B109" s="77" t="s">
         <v>97</v>
       </c>
-      <c r="C109" s="66"/>
-      <c r="D109" s="66"/>
-      <c r="E109" s="67"/>
+      <c r="C109" s="78"/>
+      <c r="D109" s="78"/>
+      <c r="E109" s="79"/>
       <c r="F109" s="43"/>
       <c r="G109" s="16"/>
       <c r="H109" s="16"/>
@@ -38548,7 +38548,7 @@
       <c r="T109" s="16"/>
     </row>
     <row r="110" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A110" s="73"/>
+      <c r="A110" s="82"/>
       <c r="B110" s="42" t="s">
         <v>77</v>
       </c>
@@ -38578,7 +38578,7 @@
       <c r="T110" s="16"/>
     </row>
     <row r="111" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A111" s="73"/>
+      <c r="A111" s="82"/>
       <c r="B111" s="42">
         <v>1</v>
       </c>
@@ -38611,7 +38611,7 @@
       <c r="T111" s="16"/>
     </row>
     <row r="112" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A112" s="73"/>
+      <c r="A112" s="82"/>
       <c r="B112" s="42">
         <v>2</v>
       </c>
@@ -38644,7 +38644,7 @@
       <c r="T112" s="16"/>
     </row>
     <row r="113" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A113" s="73"/>
+      <c r="A113" s="82"/>
       <c r="B113" s="42">
         <v>4</v>
       </c>
@@ -38677,7 +38677,7 @@
       <c r="T113" s="16"/>
     </row>
     <row r="114" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A114" s="73"/>
+      <c r="A114" s="82"/>
       <c r="B114" s="42">
         <v>6</v>
       </c>
@@ -38710,7 +38710,7 @@
       <c r="T114" s="16"/>
     </row>
     <row r="115" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A115" s="73"/>
+      <c r="A115" s="82"/>
       <c r="B115" s="42">
         <v>8</v>
       </c>
@@ -38743,7 +38743,7 @@
       <c r="T115" s="16"/>
     </row>
     <row r="116" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A116" s="73"/>
+      <c r="A116" s="82"/>
       <c r="B116" s="42">
         <v>10</v>
       </c>
@@ -38776,7 +38776,7 @@
       <c r="T116" s="16"/>
     </row>
     <row r="117" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A117" s="73"/>
+      <c r="A117" s="82"/>
       <c r="B117" s="42">
         <v>12</v>
       </c>
@@ -38809,21 +38809,21 @@
       <c r="T117" s="31"/>
     </row>
     <row r="118" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A118" s="73"/>
+      <c r="A118" s="82"/>
       <c r="B118" s="42">
         <v>16</v>
       </c>
       <c r="C118" s="40">
         <f t="shared" si="4"/>
-        <v>0.21833</v>
+        <v>0.28322000000000003</v>
       </c>
       <c r="D118" s="40">
         <f t="shared" si="5"/>
-        <v>0.30623</v>
+        <v>0.34136</v>
       </c>
       <c r="E118" s="40">
         <f t="shared" si="6"/>
-        <v>0.34717999999999999</v>
+        <v>0.33946999999999999</v>
       </c>
       <c r="F118" s="31"/>
       <c r="G118" s="31"/>
@@ -38842,41 +38842,41 @@
       <c r="T118" s="31"/>
     </row>
     <row r="119" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A119" s="73"/>
+      <c r="A119" s="82"/>
       <c r="B119" s="33" t="s">
         <v>86</v>
       </c>
-      <c r="C119" s="70" t="s">
+      <c r="C119" s="81" t="s">
         <v>113</v>
       </c>
-      <c r="D119" s="71"/>
-      <c r="E119" s="71"/>
-      <c r="F119" s="71"/>
-      <c r="G119" s="71"/>
-      <c r="H119" s="71"/>
-      <c r="I119" s="71"/>
-      <c r="J119" s="71"/>
-      <c r="K119" s="71"/>
-      <c r="L119" s="71"/>
-      <c r="M119" s="71"/>
-      <c r="N119" s="71"/>
-      <c r="O119" s="71"/>
-      <c r="P119" s="71"/>
-      <c r="Q119" s="71"/>
-      <c r="R119" s="71"/>
-      <c r="S119" s="71"/>
-      <c r="T119" s="72"/>
+      <c r="D119" s="86"/>
+      <c r="E119" s="86"/>
+      <c r="F119" s="86"/>
+      <c r="G119" s="86"/>
+      <c r="H119" s="86"/>
+      <c r="I119" s="86"/>
+      <c r="J119" s="86"/>
+      <c r="K119" s="86"/>
+      <c r="L119" s="86"/>
+      <c r="M119" s="86"/>
+      <c r="N119" s="86"/>
+      <c r="O119" s="86"/>
+      <c r="P119" s="86"/>
+      <c r="Q119" s="86"/>
+      <c r="R119" s="86"/>
+      <c r="S119" s="86"/>
+      <c r="T119" s="87"/>
     </row>
     <row r="120" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A120" s="68" t="s">
+      <c r="A120" s="88" t="s">
         <v>116</v>
       </c>
-      <c r="B120" s="65" t="s">
+      <c r="B120" s="77" t="s">
         <v>78</v>
       </c>
-      <c r="C120" s="66"/>
-      <c r="D120" s="66"/>
-      <c r="E120" s="67"/>
+      <c r="C120" s="78"/>
+      <c r="D120" s="78"/>
+      <c r="E120" s="79"/>
       <c r="F120" s="31"/>
       <c r="G120" s="31"/>
       <c r="H120" s="31"/>
@@ -38903,7 +38903,7 @@
       <c r="AC120" s="31"/>
     </row>
     <row r="121" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A121" s="69"/>
+      <c r="A121" s="89"/>
       <c r="B121" s="42" t="s">
         <v>77</v>
       </c>
@@ -38942,7 +38942,7 @@
       <c r="AC121" s="31"/>
     </row>
     <row r="122" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A122" s="69"/>
+      <c r="A122" s="89"/>
       <c r="B122" s="15">
         <v>1</v>
       </c>
@@ -38981,7 +38981,7 @@
       <c r="AC122" s="31"/>
     </row>
     <row r="123" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A123" s="69"/>
+      <c r="A123" s="89"/>
       <c r="B123" s="15">
         <v>2</v>
       </c>
@@ -39020,7 +39020,7 @@
       <c r="AC123" s="31"/>
     </row>
     <row r="124" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A124" s="69"/>
+      <c r="A124" s="89"/>
       <c r="B124" s="15">
         <v>4</v>
       </c>
@@ -39059,7 +39059,7 @@
       <c r="AC124" s="31"/>
     </row>
     <row r="125" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A125" s="69"/>
+      <c r="A125" s="89"/>
       <c r="B125" s="15">
         <v>6</v>
       </c>
@@ -39098,7 +39098,7 @@
       <c r="AC125" s="31"/>
     </row>
     <row r="126" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A126" s="69"/>
+      <c r="A126" s="89"/>
       <c r="B126" s="15">
         <v>8</v>
       </c>
@@ -39137,7 +39137,7 @@
       <c r="AC126" s="31"/>
     </row>
     <row r="127" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A127" s="69"/>
+      <c r="A127" s="89"/>
       <c r="B127" s="15">
         <v>10</v>
       </c>
@@ -39176,7 +39176,7 @@
       <c r="AC127" s="31"/>
     </row>
     <row r="128" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A128" s="69"/>
+      <c r="A128" s="89"/>
       <c r="B128" s="15">
         <v>12</v>
       </c>
@@ -39215,7 +39215,7 @@
       <c r="AC128" s="31"/>
     </row>
     <row r="129" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A129" s="69"/>
+      <c r="A129" s="89"/>
       <c r="B129" s="15">
         <v>14</v>
       </c>
@@ -39254,7 +39254,7 @@
       <c r="AC129" s="31"/>
     </row>
     <row r="130" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A130" s="69"/>
+      <c r="A130" s="89"/>
       <c r="B130" s="15">
         <v>16</v>
       </c>
@@ -39293,7 +39293,7 @@
       <c r="AC130" s="31"/>
     </row>
     <row r="131" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A131" s="69"/>
+      <c r="A131" s="89"/>
       <c r="B131" s="15">
         <v>18</v>
       </c>
@@ -39332,7 +39332,7 @@
       <c r="AC131" s="31"/>
     </row>
     <row r="132" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A132" s="69"/>
+      <c r="A132" s="89"/>
       <c r="B132" s="15">
         <v>20</v>
       </c>
@@ -39371,7 +39371,7 @@
       <c r="AC132" s="31"/>
     </row>
     <row r="133" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A133" s="69"/>
+      <c r="A133" s="89"/>
       <c r="B133" s="49">
         <v>40</v>
       </c>
@@ -39410,13 +39410,13 @@
       <c r="AC133" s="31"/>
     </row>
     <row r="134" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A134" s="69"/>
-      <c r="B134" s="65" t="s">
+      <c r="A134" s="89"/>
+      <c r="B134" s="77" t="s">
         <v>96</v>
       </c>
-      <c r="C134" s="66"/>
-      <c r="D134" s="66"/>
-      <c r="E134" s="67"/>
+      <c r="C134" s="78"/>
+      <c r="D134" s="78"/>
+      <c r="E134" s="79"/>
       <c r="F134" s="31"/>
       <c r="G134" s="31"/>
       <c r="H134" s="31"/>
@@ -39443,7 +39443,7 @@
       <c r="AC134" s="31"/>
     </row>
     <row r="135" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A135" s="69"/>
+      <c r="A135" s="89"/>
       <c r="B135" s="42" t="s">
         <v>77</v>
       </c>
@@ -39482,7 +39482,7 @@
       <c r="AC135" s="16"/>
     </row>
     <row r="136" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A136" s="69"/>
+      <c r="A136" s="89"/>
       <c r="B136" s="15">
         <v>1</v>
       </c>
@@ -39495,7 +39495,7 @@
         <v>1</v>
       </c>
       <c r="E136" s="40">
-        <f>E122/E122</f>
+        <f>ROUND(E122/E122,5)</f>
         <v>1</v>
       </c>
       <c r="F136" s="16"/>
@@ -39524,21 +39524,21 @@
       <c r="AC136" s="16"/>
     </row>
     <row r="137" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A137" s="69"/>
+      <c r="A137" s="89"/>
       <c r="B137" s="15">
         <v>2</v>
       </c>
       <c r="C137" s="40">
-        <f>C122/C123</f>
-        <v>1.7688250272826482</v>
+        <f>ROUND(C122/C123,5)</f>
+        <v>1.7688299999999999</v>
       </c>
       <c r="D137" s="40">
-        <f>D122/D123</f>
-        <v>1.9492718384479537</v>
+        <f>ROUND(D122/D123,5)</f>
+        <v>1.9492700000000001</v>
       </c>
       <c r="E137" s="40">
-        <f>E122/E123</f>
-        <v>1.970216806941498</v>
+        <f>ROUND(E122/E123,5)</f>
+        <v>1.9702200000000001</v>
       </c>
       <c r="F137" s="16"/>
       <c r="G137" s="16"/>
@@ -39566,21 +39566,21 @@
       <c r="AC137" s="16"/>
     </row>
     <row r="138" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A138" s="69"/>
+      <c r="A138" s="89"/>
       <c r="B138" s="15">
         <v>4</v>
       </c>
       <c r="C138" s="40">
-        <f>C122/C124</f>
-        <v>3.1615734720416127</v>
+        <f>ROUND(C122/C124,5)</f>
+        <v>3.1615700000000002</v>
       </c>
       <c r="D138" s="40">
-        <f>D122/D124</f>
-        <v>3.7886777435081087</v>
+        <f>ROUND(D122/D124,5)</f>
+        <v>3.7886799999999998</v>
       </c>
       <c r="E138" s="40">
-        <f>E122/E124</f>
-        <v>3.8754067245119308</v>
+        <f>ROUND(E122/E124,5)</f>
+        <v>3.87541</v>
       </c>
       <c r="F138" s="16"/>
       <c r="G138" s="16"/>
@@ -39608,21 +39608,21 @@
       <c r="AC138" s="16"/>
     </row>
     <row r="139" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A139" s="69"/>
+      <c r="A139" s="89"/>
       <c r="B139" s="15">
         <v>6</v>
       </c>
       <c r="C139" s="40">
-        <f>C122/C125</f>
-        <v>4.1524338172502135</v>
+        <f>ROUND(C122/C125,5)</f>
+        <v>4.1524299999999998</v>
       </c>
       <c r="D139" s="40">
-        <f>D122/D125</f>
-        <v>5.4156296665007471</v>
+        <f>ROUND(D122/D125,5)</f>
+        <v>5.4156300000000002</v>
       </c>
       <c r="E139" s="40">
-        <f>E122/E125</f>
-        <v>5.5921095533094229</v>
+        <f>ROUND(E122/E125,5)</f>
+        <v>5.5921099999999999</v>
       </c>
       <c r="F139" s="16"/>
       <c r="G139" s="16"/>
@@ -39650,21 +39650,21 @@
       <c r="AC139" s="16"/>
     </row>
     <row r="140" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A140" s="69"/>
+      <c r="A140" s="89"/>
       <c r="B140" s="15">
         <v>8</v>
       </c>
       <c r="C140" s="40">
-        <f>C122/C126</f>
-        <v>5.1728723404255321</v>
+        <f>ROUND(C122/C126,5)</f>
+        <v>5.1728699999999996</v>
       </c>
       <c r="D140" s="40">
-        <f>D122/D126</f>
-        <v>6.5149700598802394</v>
+        <f>ROUND(D122/D126,5)</f>
+        <v>6.5149699999999999</v>
       </c>
       <c r="E140" s="40">
-        <f>E122/E126</f>
-        <v>7.2291848146795177</v>
+        <f>ROUND(E122/E126,5)</f>
+        <v>7.2291800000000004</v>
       </c>
       <c r="F140" s="16"/>
       <c r="G140" s="16"/>
@@ -39692,21 +39692,21 @@
       <c r="AC140" s="16"/>
     </row>
     <row r="141" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A141" s="69"/>
+      <c r="A141" s="89"/>
       <c r="B141" s="15">
         <v>10</v>
       </c>
       <c r="C141" s="40">
-        <f>C122/C127</f>
-        <v>5.8939393939393936</v>
+        <f>ROUND(C122/C127,5)</f>
+        <v>5.8939399999999997</v>
       </c>
       <c r="D141" s="40">
-        <f>D122/D127</f>
-        <v>7.4953252632614902</v>
+        <f>ROUND(D122/D127,5)</f>
+        <v>7.49533</v>
       </c>
       <c r="E141" s="40">
-        <f>E122/E127</f>
-        <v>8.6001537741525702</v>
+        <f>ROUND(E122/E127,5)</f>
+        <v>8.6001499999999993</v>
       </c>
       <c r="F141" s="16"/>
       <c r="G141" s="16"/>
@@ -39734,21 +39734,21 @@
       <c r="AC141" s="16"/>
     </row>
     <row r="142" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A142" s="69"/>
+      <c r="A142" s="89"/>
       <c r="B142" s="15">
         <v>12</v>
       </c>
       <c r="C142" s="40">
-        <f>C122/C128</f>
-        <v>6.7770034843205575</v>
+        <f>ROUND(C122/C128,5)</f>
+        <v>6.7770000000000001</v>
       </c>
       <c r="D142" s="40">
-        <f>D122/D128</f>
-        <v>9.4797112272840423</v>
+        <f>ROUND(D122/D128,5)</f>
+        <v>9.4797100000000007</v>
       </c>
       <c r="E142" s="40">
-        <f>E122/E128</f>
-        <v>10.19719370565619</v>
+        <f>ROUND(E122/E128,5)</f>
+        <v>10.197190000000001</v>
       </c>
       <c r="F142" s="16"/>
       <c r="G142" s="16"/>
@@ -39776,21 +39776,21 @@
       <c r="AC142" s="16"/>
     </row>
     <row r="143" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A143" s="69"/>
+      <c r="A143" s="89"/>
       <c r="B143" s="15">
         <v>14</v>
       </c>
       <c r="C143" s="40">
-        <f>C$122/C129</f>
-        <v>7.3786039453717756</v>
+        <f t="shared" ref="C143:E147" si="7">ROUND(C$122/C129,5)</f>
+        <v>7.3785999999999996</v>
       </c>
       <c r="D143" s="40">
-        <f>D$122/D129</f>
-        <v>10.431447746883988</v>
+        <f t="shared" si="7"/>
+        <v>10.43145</v>
       </c>
       <c r="E143" s="40">
-        <f>E$122/E129</f>
-        <v>10.873415046491969</v>
+        <f t="shared" si="7"/>
+        <v>10.873419999999999</v>
       </c>
       <c r="F143" s="16"/>
       <c r="G143" s="16"/>
@@ -39818,21 +39818,21 @@
       <c r="AC143" s="16"/>
     </row>
     <row r="144" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A144" s="69"/>
+      <c r="A144" s="89"/>
       <c r="B144" s="15">
         <v>16</v>
       </c>
       <c r="C144" s="40">
-        <f t="shared" ref="C144:D147" si="7">C$122/C130</f>
-        <v>7.9517579721995091</v>
+        <f t="shared" si="7"/>
+        <v>7.9517600000000002</v>
       </c>
       <c r="D144" s="40">
         <f t="shared" si="7"/>
-        <v>11.165518252455652</v>
+        <v>11.165520000000001</v>
       </c>
       <c r="E144" s="40">
-        <f t="shared" ref="E144" si="8">E$122/E130</f>
-        <v>12.214651979868957</v>
+        <f t="shared" si="7"/>
+        <v>12.214650000000001</v>
       </c>
       <c r="F144" s="31"/>
       <c r="G144" s="31"/>
@@ -39860,21 +39860,21 @@
       <c r="AC144" s="31"/>
     </row>
     <row r="145" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A145" s="69"/>
+      <c r="A145" s="89"/>
       <c r="B145" s="15">
         <v>18</v>
       </c>
       <c r="C145" s="40">
         <f t="shared" si="7"/>
-        <v>8.2695578231292526</v>
+        <v>8.2695600000000002</v>
       </c>
       <c r="D145" s="40">
         <f t="shared" si="7"/>
-        <v>12.281890017739075</v>
+        <v>12.281890000000001</v>
       </c>
       <c r="E145" s="40">
-        <f t="shared" ref="E145" si="9">E$122/E131</f>
-        <v>12.466201482773659</v>
+        <f t="shared" si="7"/>
+        <v>12.466200000000001</v>
       </c>
       <c r="F145" s="16"/>
       <c r="G145" s="16"/>
@@ -39902,21 +39902,21 @@
       <c r="AC145" s="16"/>
     </row>
     <row r="146" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A146" s="69"/>
+      <c r="A146" s="89"/>
       <c r="B146" s="15">
         <v>20</v>
       </c>
       <c r="C146" s="40">
         <f t="shared" si="7"/>
-        <v>9.1143392689784442</v>
+        <v>9.1143400000000003</v>
       </c>
       <c r="D146" s="40">
         <f t="shared" si="7"/>
-        <v>12.575957727873183</v>
+        <v>12.57596</v>
       </c>
       <c r="E146" s="40">
-        <f t="shared" ref="E146" si="10">E$122/E132</f>
-        <v>14.049751515482496</v>
+        <f t="shared" si="7"/>
+        <v>14.04975</v>
       </c>
       <c r="F146" s="16"/>
       <c r="G146" s="16"/>
@@ -39944,21 +39944,21 @@
       <c r="AC146" s="16"/>
     </row>
     <row r="147" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A147" s="69"/>
+      <c r="A147" s="89"/>
       <c r="B147" s="49">
         <v>40</v>
       </c>
       <c r="C147" s="50">
         <f t="shared" si="7"/>
-        <v>8.0974188176519561</v>
+        <v>8.0974199999999996</v>
       </c>
       <c r="D147" s="50">
         <f t="shared" si="7"/>
-        <v>11.124744376278118</v>
+        <v>11.124739999999999</v>
       </c>
       <c r="E147" s="50">
-        <f>E$122/E133</f>
-        <v>12.471035920306365</v>
+        <f t="shared" si="7"/>
+        <v>12.47104</v>
       </c>
       <c r="F147" s="16"/>
       <c r="G147" s="16"/>
@@ -39986,13 +39986,13 @@
       <c r="AC147" s="16"/>
     </row>
     <row r="148" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A148" s="69"/>
-      <c r="B148" s="65" t="s">
+      <c r="A148" s="89"/>
+      <c r="B148" s="77" t="s">
         <v>97</v>
       </c>
-      <c r="C148" s="66"/>
-      <c r="D148" s="66"/>
-      <c r="E148" s="67"/>
+      <c r="C148" s="78"/>
+      <c r="D148" s="78"/>
+      <c r="E148" s="79"/>
       <c r="F148" s="16"/>
       <c r="G148" s="16"/>
       <c r="H148" s="16"/>
@@ -40019,7 +40019,7 @@
       <c r="AC148" s="16"/>
     </row>
     <row r="149" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A149" s="69"/>
+      <c r="A149" s="89"/>
       <c r="B149" s="42" t="s">
         <v>77</v>
       </c>
@@ -40058,20 +40058,20 @@
       <c r="AC149" s="16"/>
     </row>
     <row r="150" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A150" s="69"/>
+      <c r="A150" s="89"/>
       <c r="B150" s="15">
         <v>1</v>
       </c>
       <c r="C150" s="40">
-        <f t="shared" ref="C150:E154" si="11">C136/$B136</f>
+        <f t="shared" ref="C150:C161" si="8">ROUND(C136/$B136,5)</f>
         <v>1</v>
       </c>
       <c r="D150" s="40">
-        <f t="shared" si="11"/>
+        <f t="shared" ref="D150:E154" si="9">D136/$B136</f>
         <v>1</v>
       </c>
       <c r="E150" s="40">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>1</v>
       </c>
       <c r="F150" s="16"/>
@@ -40100,21 +40100,21 @@
       <c r="AC150" s="16"/>
     </row>
     <row r="151" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A151" s="69"/>
+      <c r="A151" s="89"/>
       <c r="B151" s="15">
         <v>2</v>
       </c>
       <c r="C151" s="40">
-        <f t="shared" si="11"/>
-        <v>0.88441251364132412</v>
+        <f t="shared" si="8"/>
+        <v>0.88441999999999998</v>
       </c>
       <c r="D151" s="40">
-        <f t="shared" si="11"/>
-        <v>0.97463591922397685</v>
+        <f t="shared" si="9"/>
+        <v>0.97463500000000003</v>
       </c>
       <c r="E151" s="40">
-        <f t="shared" si="11"/>
-        <v>0.98510840347074902</v>
+        <f t="shared" si="9"/>
+        <v>0.98511000000000004</v>
       </c>
       <c r="F151" s="16"/>
       <c r="G151" s="16"/>
@@ -40142,21 +40142,21 @@
       <c r="AC151" s="16"/>
     </row>
     <row r="152" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A152" s="69"/>
+      <c r="A152" s="89"/>
       <c r="B152" s="15">
         <v>4</v>
       </c>
       <c r="C152" s="40">
-        <f t="shared" si="11"/>
-        <v>0.79039336801040316</v>
+        <f t="shared" si="8"/>
+        <v>0.79039000000000004</v>
       </c>
       <c r="D152" s="40">
-        <f t="shared" si="11"/>
-        <v>0.94716943587702718</v>
+        <f t="shared" si="9"/>
+        <v>0.94716999999999996</v>
       </c>
       <c r="E152" s="40">
-        <f t="shared" si="11"/>
-        <v>0.9688516811279827</v>
+        <f t="shared" si="9"/>
+        <v>0.96885250000000001</v>
       </c>
       <c r="F152" s="16"/>
       <c r="G152" s="16"/>
@@ -40184,21 +40184,21 @@
       <c r="AC152" s="16"/>
     </row>
     <row r="153" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A153" s="69"/>
+      <c r="A153" s="89"/>
       <c r="B153" s="15">
         <v>6</v>
       </c>
       <c r="C153" s="40">
-        <f t="shared" si="11"/>
-        <v>0.69207230287503563</v>
+        <f t="shared" si="8"/>
+        <v>0.69206999999999996</v>
       </c>
       <c r="D153" s="40">
-        <f t="shared" si="11"/>
-        <v>0.90260494441679118</v>
+        <f t="shared" si="9"/>
+        <v>0.90260499999999999</v>
       </c>
       <c r="E153" s="40">
-        <f t="shared" si="11"/>
-        <v>0.93201825888490386</v>
+        <f t="shared" si="9"/>
+        <v>0.93201833333333328</v>
       </c>
       <c r="F153" s="16"/>
       <c r="G153" s="16"/>
@@ -40226,21 +40226,21 @@
       <c r="AC153" s="16"/>
     </row>
     <row r="154" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A154" s="69"/>
+      <c r="A154" s="89"/>
       <c r="B154" s="15">
         <v>8</v>
       </c>
       <c r="C154" s="40">
-        <f t="shared" si="11"/>
-        <v>0.64660904255319152</v>
+        <f t="shared" si="8"/>
+        <v>0.64661000000000002</v>
       </c>
       <c r="D154" s="40">
-        <f t="shared" si="11"/>
-        <v>0.81437125748502992</v>
+        <f t="shared" si="9"/>
+        <v>0.81437124999999999</v>
       </c>
       <c r="E154" s="40">
-        <f t="shared" si="11"/>
-        <v>0.90364810183493971</v>
+        <f t="shared" si="9"/>
+        <v>0.90364750000000005</v>
       </c>
       <c r="F154" s="16"/>
       <c r="G154" s="16"/>
@@ -40268,21 +40268,21 @@
       <c r="AC154" s="16"/>
     </row>
     <row r="155" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A155" s="69"/>
+      <c r="A155" s="89"/>
       <c r="B155" s="15">
         <v>10</v>
       </c>
       <c r="C155" s="40">
-        <f>C141/B141</f>
-        <v>0.58939393939393936</v>
+        <f t="shared" si="8"/>
+        <v>0.58938999999999997</v>
       </c>
       <c r="D155" s="40">
-        <f t="shared" ref="D155:E161" si="12">D141/$B141</f>
-        <v>0.74953252632614897</v>
+        <f t="shared" ref="D155:E161" si="10">D141/$B141</f>
+        <v>0.749533</v>
       </c>
       <c r="E155" s="40">
-        <f t="shared" si="12"/>
-        <v>0.86001537741525702</v>
+        <f t="shared" si="10"/>
+        <v>0.86001499999999997</v>
       </c>
       <c r="F155" s="16"/>
       <c r="G155" s="16"/>
@@ -40310,21 +40310,21 @@
       <c r="AC155" s="16"/>
     </row>
     <row r="156" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A156" s="69"/>
+      <c r="A156" s="89"/>
       <c r="B156" s="15">
         <v>12</v>
       </c>
       <c r="C156" s="40">
-        <f t="shared" ref="C156:C161" si="13">C142/$B142</f>
-        <v>0.56475029036004643</v>
+        <f t="shared" si="8"/>
+        <v>0.56474999999999997</v>
       </c>
       <c r="D156" s="40">
-        <f t="shared" si="12"/>
-        <v>0.78997593560700352</v>
+        <f t="shared" si="10"/>
+        <v>0.78997583333333343</v>
       </c>
       <c r="E156" s="40">
-        <f t="shared" si="12"/>
-        <v>0.84976614213801582</v>
+        <f t="shared" si="10"/>
+        <v>0.84976583333333344</v>
       </c>
       <c r="F156" s="31"/>
       <c r="G156" s="31"/>
@@ -40352,21 +40352,21 @@
       <c r="AC156" s="31"/>
     </row>
     <row r="157" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A157" s="69"/>
+      <c r="A157" s="89"/>
       <c r="B157" s="15">
         <v>14</v>
       </c>
       <c r="C157" s="40">
-        <f t="shared" si="13"/>
-        <v>0.52704313895512678</v>
+        <f t="shared" si="8"/>
+        <v>0.52703999999999995</v>
       </c>
       <c r="D157" s="40">
-        <f t="shared" si="12"/>
-        <v>0.74510341049171347</v>
+        <f t="shared" si="10"/>
+        <v>0.74510357142857142</v>
       </c>
       <c r="E157" s="40">
-        <f t="shared" si="12"/>
-        <v>0.77667250332085491</v>
+        <f t="shared" si="10"/>
+        <v>0.77667285714285705</v>
       </c>
       <c r="F157" s="31"/>
       <c r="G157" s="31"/>
@@ -40394,21 +40394,21 @@
       <c r="AC157" s="31"/>
     </row>
     <row r="158" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A158" s="69"/>
+      <c r="A158" s="89"/>
       <c r="B158" s="15">
         <v>16</v>
       </c>
       <c r="C158" s="40">
-        <f t="shared" si="13"/>
-        <v>0.49698487326246932</v>
+        <f t="shared" si="8"/>
+        <v>0.49698999999999999</v>
       </c>
       <c r="D158" s="40">
-        <f t="shared" si="12"/>
-        <v>0.69784489077847822</v>
+        <f t="shared" si="10"/>
+        <v>0.69784500000000005</v>
       </c>
       <c r="E158" s="40">
-        <f t="shared" si="12"/>
-        <v>0.76341574874180984</v>
+        <f t="shared" si="10"/>
+        <v>0.76341562500000004</v>
       </c>
       <c r="F158" s="16"/>
       <c r="G158" s="16"/>
@@ -40436,21 +40436,21 @@
       <c r="AC158" s="16"/>
     </row>
     <row r="159" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A159" s="69"/>
+      <c r="A159" s="89"/>
       <c r="B159" s="15">
         <v>18</v>
       </c>
       <c r="C159" s="40">
-        <f t="shared" si="13"/>
-        <v>0.45941987906273624</v>
+        <f t="shared" si="8"/>
+        <v>0.45942</v>
       </c>
       <c r="D159" s="40">
-        <f t="shared" si="12"/>
-        <v>0.68232722320772643</v>
+        <f t="shared" si="10"/>
+        <v>0.68232722222222231</v>
       </c>
       <c r="E159" s="40">
-        <f t="shared" si="12"/>
-        <v>0.6925667490429811</v>
+        <f t="shared" si="10"/>
+        <v>0.69256666666666666</v>
       </c>
       <c r="F159" s="16"/>
       <c r="G159" s="16"/>
@@ -40478,21 +40478,21 @@
       <c r="AC159" s="16"/>
     </row>
     <row r="160" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A160" s="69"/>
+      <c r="A160" s="89"/>
       <c r="B160" s="15">
         <v>20</v>
       </c>
       <c r="C160" s="40">
-        <f t="shared" si="13"/>
-        <v>0.45571696344892221</v>
+        <f t="shared" si="8"/>
+        <v>0.45572000000000001</v>
       </c>
       <c r="D160" s="40">
-        <f t="shared" si="12"/>
-        <v>0.62879788639365919</v>
+        <f t="shared" si="10"/>
+        <v>0.62879799999999997</v>
       </c>
       <c r="E160" s="40">
-        <f t="shared" si="12"/>
-        <v>0.7024875757741248</v>
+        <f t="shared" si="10"/>
+        <v>0.70248749999999993</v>
       </c>
       <c r="F160" s="16"/>
       <c r="G160" s="16"/>
@@ -40520,21 +40520,21 @@
       <c r="AC160" s="16"/>
     </row>
     <row r="161" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A161" s="69"/>
+      <c r="A161" s="89"/>
       <c r="B161" s="49">
         <v>40</v>
       </c>
       <c r="C161" s="50">
-        <f t="shared" si="13"/>
-        <v>0.20243547044129889</v>
+        <f t="shared" si="8"/>
+        <v>0.20244000000000001</v>
       </c>
       <c r="D161" s="50">
-        <f t="shared" si="12"/>
-        <v>0.27811860940695293</v>
+        <f t="shared" si="10"/>
+        <v>0.27811849999999999</v>
       </c>
       <c r="E161" s="50">
-        <f t="shared" si="12"/>
-        <v>0.31177589800765915</v>
+        <f t="shared" si="10"/>
+        <v>0.311776</v>
       </c>
       <c r="F161" s="16"/>
       <c r="G161" s="16"/>
@@ -40562,42 +40562,63 @@
       <c r="AC161" s="16"/>
     </row>
     <row r="162" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A162" s="69"/>
+      <c r="A162" s="89"/>
       <c r="B162" s="33" t="s">
         <v>86</v>
       </c>
-      <c r="C162" s="70" t="s">
+      <c r="C162" s="81" t="s">
         <v>115</v>
       </c>
-      <c r="D162" s="71"/>
-      <c r="E162" s="71"/>
-      <c r="F162" s="71"/>
-      <c r="G162" s="71"/>
-      <c r="H162" s="71"/>
-      <c r="I162" s="71"/>
-      <c r="J162" s="71"/>
-      <c r="K162" s="71"/>
-      <c r="L162" s="71"/>
-      <c r="M162" s="71"/>
-      <c r="N162" s="71"/>
-      <c r="O162" s="71"/>
-      <c r="P162" s="71"/>
-      <c r="Q162" s="71"/>
-      <c r="R162" s="71"/>
-      <c r="S162" s="71"/>
-      <c r="T162" s="71"/>
-      <c r="U162" s="71"/>
-      <c r="V162" s="71"/>
-      <c r="W162" s="71"/>
-      <c r="X162" s="71"/>
-      <c r="Y162" s="71"/>
-      <c r="Z162" s="71"/>
-      <c r="AA162" s="71"/>
-      <c r="AB162" s="71"/>
-      <c r="AC162" s="72"/>
+      <c r="D162" s="86"/>
+      <c r="E162" s="86"/>
+      <c r="F162" s="86"/>
+      <c r="G162" s="86"/>
+      <c r="H162" s="86"/>
+      <c r="I162" s="86"/>
+      <c r="J162" s="86"/>
+      <c r="K162" s="86"/>
+      <c r="L162" s="86"/>
+      <c r="M162" s="86"/>
+      <c r="N162" s="86"/>
+      <c r="O162" s="86"/>
+      <c r="P162" s="86"/>
+      <c r="Q162" s="86"/>
+      <c r="R162" s="86"/>
+      <c r="S162" s="86"/>
+      <c r="T162" s="86"/>
+      <c r="U162" s="86"/>
+      <c r="V162" s="86"/>
+      <c r="W162" s="86"/>
+      <c r="X162" s="86"/>
+      <c r="Y162" s="86"/>
+      <c r="Z162" s="86"/>
+      <c r="AA162" s="86"/>
+      <c r="AB162" s="86"/>
+      <c r="AC162" s="87"/>
     </row>
   </sheetData>
   <mergeCells count="35">
+    <mergeCell ref="B148:E148"/>
+    <mergeCell ref="B134:E134"/>
+    <mergeCell ref="B120:E120"/>
+    <mergeCell ref="A120:A162"/>
+    <mergeCell ref="C162:AC162"/>
+    <mergeCell ref="A89:A119"/>
+    <mergeCell ref="C119:T119"/>
+    <mergeCell ref="B89:E89"/>
+    <mergeCell ref="B99:E99"/>
+    <mergeCell ref="B109:E109"/>
+    <mergeCell ref="A24:L24"/>
+    <mergeCell ref="M24:N24"/>
+    <mergeCell ref="M1:N1"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="C12:N12"/>
+    <mergeCell ref="A2:A12"/>
+    <mergeCell ref="A13:A23"/>
+    <mergeCell ref="B22:B23"/>
+    <mergeCell ref="C22:N23"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="B2:D2"/>
     <mergeCell ref="O88:T88"/>
     <mergeCell ref="A88:N88"/>
     <mergeCell ref="A57:A87"/>
@@ -40612,27 +40633,6 @@
     <mergeCell ref="B45:D45"/>
     <mergeCell ref="B35:D35"/>
     <mergeCell ref="B25:D25"/>
-    <mergeCell ref="A24:L24"/>
-    <mergeCell ref="M24:N24"/>
-    <mergeCell ref="M1:N1"/>
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="C12:N12"/>
-    <mergeCell ref="A2:A12"/>
-    <mergeCell ref="A13:A23"/>
-    <mergeCell ref="B22:B23"/>
-    <mergeCell ref="C22:N23"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="A89:A119"/>
-    <mergeCell ref="C119:T119"/>
-    <mergeCell ref="B89:E89"/>
-    <mergeCell ref="B99:E99"/>
-    <mergeCell ref="B109:E109"/>
-    <mergeCell ref="B148:E148"/>
-    <mergeCell ref="B134:E134"/>
-    <mergeCell ref="B120:E120"/>
-    <mergeCell ref="A120:A162"/>
-    <mergeCell ref="C162:AC162"/>
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <hyperlinks>

</xml_diff>

<commit_message>
Added simple diagonaly dominant constructor for faster init.
</commit_message>
<xml_diff>
--- a/DecompositionLU/docs/statistics.xlsx
+++ b/DecompositionLU/docs/statistics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Maxim\source\repos\practice\SECOND_COURSE\FOR_ITLAB\ArchBenchs\DecompositionLU\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8730C858-ED17-4A5F-A6F0-5B7E2934BBAA}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EF867C6-078C-45FB-8D57-EF0D3112A1F6}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-114" yWindow="-114" windowWidth="27602" windowHeight="15027" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="119">
   <si>
     <t>Я не уверен, будет ли это использоваться в готовой презентации и так ли это надо делать, если да, так что пока считаем, что файл для личного пользования.</t>
   </si>
@@ -478,6 +478,12 @@
   </si>
   <si>
     <t>Замеры на кластере, данные, аналогично, вкладке "Про процессор"</t>
+  </si>
+  <si>
+    <t>icpx -g -O2 -fopenmp -march=icelake-server ./test.cpp -o test</t>
+  </si>
+  <si>
+    <t>srun -N 1 advisor --collect=roofline …</t>
   </si>
 </sst>
 </file>
@@ -35691,28 +35697,52 @@
       <c r="A79" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B79" s="9"/>
-      <c r="C79" s="10"/>
-      <c r="D79" s="10"/>
-      <c r="E79" s="10"/>
+      <c r="B79" s="9">
+        <v>1179</v>
+      </c>
+      <c r="C79" s="10">
+        <v>2737</v>
+      </c>
+      <c r="D79" s="10">
+        <v>4927</v>
+      </c>
+      <c r="E79" s="10">
+        <v>9248</v>
+      </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B80" s="9"/>
-      <c r="C80" s="10"/>
-      <c r="D80" s="10"/>
-      <c r="E80" s="10"/>
+      <c r="B80" s="9">
+        <v>459</v>
+      </c>
+      <c r="C80" s="10">
+        <v>1310</v>
+      </c>
+      <c r="D80" s="10">
+        <v>2689</v>
+      </c>
+      <c r="E80" s="10">
+        <v>6665</v>
+      </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B81" s="9"/>
-      <c r="C81" s="10"/>
-      <c r="D81" s="10"/>
-      <c r="E81" s="10"/>
+      <c r="B81" s="9">
+        <v>1638</v>
+      </c>
+      <c r="C81" s="10">
+        <v>4048</v>
+      </c>
+      <c r="D81" s="10">
+        <v>7636</v>
+      </c>
+      <c r="E81" s="10">
+        <v>15914</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="32">
@@ -35766,7 +35796,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:AC162"/>
+  <dimension ref="A1:AC167"/>
   <sheetFormatPr defaultRowHeight="21.6" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.28515625" style="26" customWidth="1"/>
@@ -40595,6 +40625,16 @@
       <c r="AA162" s="86"/>
       <c r="AB162" s="86"/>
       <c r="AC162" s="87"/>
+    </row>
+    <row r="165" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B165" s="26" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="167" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B167" s="26" t="s">
+        <v>118</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="35">

</xml_diff>

<commit_message>
Toolchains for risk-V, eng comments, some changes in cmd args
</commit_message>
<xml_diff>
--- a/DecompositionLU/docs/statistics.xlsx
+++ b/DecompositionLU/docs/statistics.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Maxim\source\repos\practice\SECOND_COURSE\FOR_ITLAB\ArchBenchs\DecompositionLU\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EF867C6-078C-45FB-8D57-EF0D3112A1F6}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7569BE9-6E9F-4482-B87C-E87E23EA383E}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-114" yWindow="-114" windowWidth="27602" windowHeight="15027" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-114" yWindow="-114" windowWidth="27602" windowHeight="15027" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Таблица" sheetId="1" r:id="rId1"/>
     <sheet name="Графики" sheetId="2" r:id="rId2"/>
-    <sheet name="Про процессор" sheetId="3" r:id="rId3"/>
+    <sheet name="Про ноутбук" sheetId="3" r:id="rId3"/>
+    <sheet name="Про кластер" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="125">
   <si>
     <t>Я не уверен, будет ли это использоваться в готовой презентации и так ли это надо делать, если да, так что пока считаем, что файл для личного пользования.</t>
   </si>
@@ -474,9 +475,6 @@
     <t>n = 15000</t>
   </si>
   <si>
-    <t>В ходе работы выяснил следующее - на миникластере 2 процессора по 10 физ ядер, балансировать их надо поровну, но на каждом четное количество (чем больше размер матрицы, тем более заметно, например, при n=10000 и числе потоков &lt;= 10, это незаметно)</t>
-  </si>
-  <si>
     <t>Замеры на кластере, данные, аналогично, вкладке "Про процессор"</t>
   </si>
   <si>
@@ -485,12 +483,33 @@
   <si>
     <t>srun -N 1 advisor --collect=roofline …</t>
   </si>
+  <si>
+    <t>на 20000:</t>
+  </si>
+  <si>
+    <t>1 поток</t>
+  </si>
+  <si>
+    <t>20 потоков</t>
+  </si>
+  <si>
+    <t>время</t>
+  </si>
+  <si>
+    <t>ускорение</t>
+  </si>
+  <si>
+    <t>эффективность</t>
+  </si>
+  <si>
+    <t>с ключом -march=icelake-server программа ускорилась вдвое, но потеряла в ускорении.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -631,6 +650,13 @@
       <family val="2"/>
       <charset val="204"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="GOST Common"/>
+      <family val="2"/>
+      <charset val="204"/>
     </font>
   </fonts>
   <fills count="8">
@@ -859,7 +885,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="90">
+  <cellXfs count="98">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
@@ -972,6 +998,27 @@
     <xf numFmtId="0" fontId="12" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1011,6 +1058,48 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="5" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1046,45 +1135,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -9098,34 +9148,34 @@
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.7688299999999999</c:v>
+                  <c:v>1.9660200000000001</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>3.1615700000000002</c:v>
+                  <c:v>3.7708499999999998</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>4.1524299999999998</c:v>
+                  <c:v>5.16411</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>5.1728699999999996</c:v>
+                  <c:v>6.5782400000000001</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>5.8939399999999997</c:v>
+                  <c:v>7.8900300000000003</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>6.7770000000000001</c:v>
+                  <c:v>9.0895299999999999</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>7.3785999999999996</c:v>
+                  <c:v>9.7836400000000001</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>7.9517600000000002</c:v>
+                  <c:v>10.21063</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>8.2695600000000002</c:v>
+                  <c:v>10.82696</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>9.1143400000000003</c:v>
+                  <c:v>11.23382</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -9626,34 +9676,34 @@
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.88441999999999998</c:v>
+                  <c:v>0.98301000000000005</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.79039000000000004</c:v>
+                  <c:v>0.94271000000000005</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.69206999999999996</c:v>
+                  <c:v>0.86068999999999996</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.64661000000000002</c:v>
+                  <c:v>0.82228000000000001</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.58938999999999997</c:v>
+                  <c:v>0.78900000000000003</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.56474999999999997</c:v>
+                  <c:v>0.75746000000000002</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.52703999999999995</c:v>
+                  <c:v>0.69882999999999995</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.49698999999999999</c:v>
+                  <c:v>0.63815999999999995</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.45942</c:v>
+                  <c:v>0.60150000000000003</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.45572000000000001</c:v>
+                  <c:v>0.56169000000000002</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -10024,37 +10074,37 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="11"/>
                 <c:pt idx="0">
-                  <c:v>9725</c:v>
+                  <c:v>5381</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>5498</c:v>
+                  <c:v>2737</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>3076</c:v>
+                  <c:v>1427</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2342</c:v>
+                  <c:v>1042</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1880</c:v>
+                  <c:v>818</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1650</c:v>
+                  <c:v>682</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1435</c:v>
+                  <c:v>592</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1318</c:v>
+                  <c:v>550</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1223</c:v>
+                  <c:v>527</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>1176</c:v>
+                  <c:v>497</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1067</c:v>
+                  <c:v>479</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -10425,37 +10475,37 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="11"/>
                 <c:pt idx="0">
-                  <c:v>76160</c:v>
+                  <c:v>41829</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>39071</c:v>
+                  <c:v>21202</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>20102</c:v>
+                  <c:v>11078</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>14063</c:v>
+                  <c:v>7787</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>11690</c:v>
+                  <c:v>6260</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>10161</c:v>
+                  <c:v>5372</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>8034</c:v>
+                  <c:v>4574</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>7301</c:v>
+                  <c:v>4295</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>6821</c:v>
+                  <c:v>3969</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>6201</c:v>
+                  <c:v>3709</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>6056</c:v>
+                  <c:v>3554</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -11026,37 +11076,37 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="11"/>
                 <c:pt idx="0">
-                  <c:v>257265</c:v>
+                  <c:v>142216</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>130577</c:v>
+                  <c:v>70771</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>66384</c:v>
+                  <c:v>36194</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>46005</c:v>
+                  <c:v>25435</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>35587</c:v>
+                  <c:v>19632</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>29914</c:v>
+                  <c:v>16476</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>25229</c:v>
+                  <c:v>14220</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>23660</c:v>
+                  <c:v>13252</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>21062</c:v>
+                  <c:v>12007</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>20637</c:v>
+                  <c:v>11351</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>18311</c:v>
+                  <c:v>10884</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -11559,34 +11609,34 @@
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.9702200000000001</c:v>
+                  <c:v>2.0095200000000002</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>3.87541</c:v>
+                  <c:v>3.9292699999999998</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5.5921099999999999</c:v>
+                  <c:v>5.5913500000000003</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>7.2291800000000004</c:v>
+                  <c:v>7.2440899999999999</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>8.6001499999999993</c:v>
+                  <c:v>8.63171</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>10.197190000000001</c:v>
+                  <c:v>10.00113</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>10.873419999999999</c:v>
+                  <c:v>10.73166</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>12.214650000000001</c:v>
+                  <c:v>11.84442</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>12.466200000000001</c:v>
+                  <c:v>12.52894</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>14.04975</c:v>
+                  <c:v>13.066520000000001</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -12090,37 +12140,37 @@
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.9492700000000001</c:v>
+                  <c:v>1.97288</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>3.7886799999999998</c:v>
+                  <c:v>3.7758600000000002</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5.4156300000000002</c:v>
+                  <c:v>5.3716499999999998</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>6.5149699999999999</c:v>
+                  <c:v>6.6819499999999996</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>7.49533</c:v>
+                  <c:v>7.7864899999999997</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>9.4797100000000007</c:v>
+                  <c:v>9.1449499999999997</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>10.43145</c:v>
+                  <c:v>9.7390000000000008</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>11.165520000000001</c:v>
+                  <c:v>10.538930000000001</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>12.281890000000001</c:v>
+                  <c:v>11.277699999999999</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>12.57596</c:v>
+                  <c:v>11.76956</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>11.124739999999999</c:v>
+                  <c:v>11.314310000000001</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -12621,34 +12671,34 @@
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.98511000000000004</c:v>
+                  <c:v>1.0047600000000001</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.96885250000000001</c:v>
+                  <c:v>0.98231999999999997</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.93201833333333328</c:v>
+                  <c:v>0.93189</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.90364750000000005</c:v>
+                  <c:v>0.90551000000000004</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.86001499999999997</c:v>
+                  <c:v>0.86316999999999999</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.84976583333333344</c:v>
+                  <c:v>0.83343</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.77667285714285705</c:v>
+                  <c:v>0.76654999999999995</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.76341562500000004</c:v>
+                  <c:v>0.74028000000000005</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.69256666666666666</c:v>
+                  <c:v>0.69604999999999995</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.70248749999999993</c:v>
+                  <c:v>0.65332999999999997</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -13151,34 +13201,34 @@
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.97463500000000003</c:v>
+                  <c:v>0.98643999999999998</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.94716999999999996</c:v>
+                  <c:v>0.94396999999999998</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.90260499999999999</c:v>
+                  <c:v>0.89527999999999996</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.81437124999999999</c:v>
+                  <c:v>0.83523999999999998</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.749533</c:v>
+                  <c:v>0.77864999999999995</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.78997583333333343</c:v>
+                  <c:v>0.76207999999999998</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.74510357142857142</c:v>
+                  <c:v>0.69564000000000004</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.69784500000000005</c:v>
+                  <c:v>0.65868000000000004</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.68232722222222231</c:v>
+                  <c:v>0.62653999999999999</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.62879799999999997</c:v>
+                  <c:v>0.58848</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -34272,6 +34322,55 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>314076</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>93477</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Рисунок 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{737DEF32-62D1-4C14-BC14-417238EFD225}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="579422" y="280657"/>
+          <a:ext cx="7267137" cy="1496765"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -34613,17 +34712,17 @@
       <c r="N3" s="6"/>
     </row>
     <row r="5" spans="1:23" ht="17.850000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="52" t="s">
+      <c r="A5" s="59" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="53"/>
-      <c r="C5" s="53"/>
-      <c r="D5" s="53"/>
-      <c r="E5" s="54"/>
-      <c r="G5" s="59" t="s">
+      <c r="B5" s="60"/>
+      <c r="C5" s="60"/>
+      <c r="D5" s="60"/>
+      <c r="E5" s="61"/>
+      <c r="G5" s="66" t="s">
         <v>3</v>
       </c>
-      <c r="H5" s="59"/>
+      <c r="H5" s="66"/>
       <c r="S5" s="5"/>
       <c r="T5" s="14"/>
       <c r="U5" s="14"/>
@@ -34634,14 +34733,14 @@
       <c r="A6" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="56" t="s">
+      <c r="B6" s="63" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="56"/>
-      <c r="D6" s="56"/>
-      <c r="E6" s="56"/>
-      <c r="G6" s="59"/>
-      <c r="H6" s="59"/>
+      <c r="C6" s="63"/>
+      <c r="D6" s="63"/>
+      <c r="E6" s="63"/>
+      <c r="G6" s="66"/>
+      <c r="H6" s="66"/>
       <c r="S6" s="14"/>
       <c r="T6" s="14"/>
       <c r="U6" s="14"/>
@@ -34664,8 +34763,8 @@
       <c r="E7" s="8">
         <v>10000</v>
       </c>
-      <c r="G7" s="59"/>
-      <c r="H7" s="59"/>
+      <c r="G7" s="66"/>
+      <c r="H7" s="66"/>
       <c r="S7" s="14"/>
       <c r="T7" s="14"/>
       <c r="U7" s="14"/>
@@ -34673,15 +34772,15 @@
       <c r="W7" s="14"/>
     </row>
     <row r="8" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A8" s="57" t="s">
+      <c r="A8" s="64" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="57"/>
-      <c r="C8" s="57"/>
-      <c r="D8" s="57"/>
-      <c r="E8" s="57"/>
-      <c r="G8" s="59"/>
-      <c r="H8" s="59"/>
+      <c r="B8" s="64"/>
+      <c r="C8" s="64"/>
+      <c r="D8" s="64"/>
+      <c r="E8" s="64"/>
+      <c r="G8" s="66"/>
+      <c r="H8" s="66"/>
       <c r="S8" s="14"/>
       <c r="T8" s="14"/>
       <c r="U8" s="14"/>
@@ -34757,13 +34856,13 @@
       <c r="W11" s="5"/>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A12" s="57" t="s">
+      <c r="A12" s="64" t="s">
         <v>12</v>
       </c>
-      <c r="B12" s="57"/>
-      <c r="C12" s="57"/>
-      <c r="D12" s="57"/>
-      <c r="E12" s="57"/>
+      <c r="B12" s="64"/>
+      <c r="C12" s="64"/>
+      <c r="D12" s="64"/>
+      <c r="E12" s="64"/>
       <c r="F12" s="5"/>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.25">
@@ -34776,7 +34875,7 @@
       <c r="C13" s="10">
         <v>232</v>
       </c>
-      <c r="D13" s="61" t="s">
+      <c r="D13" s="68" t="s">
         <v>21</v>
       </c>
       <c r="E13" s="10">
@@ -34794,7 +34893,7 @@
       <c r="C14" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="D14" s="62"/>
+      <c r="D14" s="69"/>
       <c r="E14" s="10" t="s">
         <v>10</v>
       </c>
@@ -34812,30 +34911,30 @@
       <c r="C15" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="D15" s="63"/>
+      <c r="D15" s="70"/>
       <c r="E15" s="10" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A18" s="64" t="s">
+      <c r="A18" s="71" t="s">
         <v>32</v>
       </c>
-      <c r="B18" s="64"/>
-      <c r="C18" s="64"/>
-      <c r="D18" s="64"/>
-      <c r="E18" s="64"/>
+      <c r="B18" s="71"/>
+      <c r="C18" s="71"/>
+      <c r="D18" s="71"/>
+      <c r="E18" s="71"/>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B19" s="56" t="s">
+      <c r="B19" s="63" t="s">
         <v>5</v>
       </c>
-      <c r="C19" s="56"/>
-      <c r="D19" s="56"/>
-      <c r="E19" s="56"/>
+      <c r="C19" s="63"/>
+      <c r="D19" s="63"/>
+      <c r="E19" s="63"/>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
@@ -34855,13 +34954,13 @@
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A21" s="57" t="s">
+      <c r="A21" s="64" t="s">
         <v>11</v>
       </c>
-      <c r="B21" s="57"/>
-      <c r="C21" s="57"/>
-      <c r="D21" s="57"/>
-      <c r="E21" s="57"/>
+      <c r="B21" s="64"/>
+      <c r="C21" s="64"/>
+      <c r="D21" s="64"/>
+      <c r="E21" s="64"/>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
@@ -34914,17 +35013,17 @@
         <v>35</v>
       </c>
       <c r="G24" s="18"/>
-      <c r="H24" s="58"/>
-      <c r="I24" s="58"/>
+      <c r="H24" s="65"/>
+      <c r="I24" s="65"/>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" s="57" t="s">
+      <c r="A25" s="64" t="s">
         <v>12</v>
       </c>
-      <c r="B25" s="57"/>
-      <c r="C25" s="57"/>
-      <c r="D25" s="57"/>
-      <c r="E25" s="57"/>
+      <c r="B25" s="64"/>
+      <c r="C25" s="64"/>
+      <c r="D25" s="64"/>
+      <c r="E25" s="64"/>
       <c r="G25" s="19"/>
       <c r="H25" s="17"/>
       <c r="I25" s="17"/>
@@ -35009,15 +35108,15 @@
       <c r="I30" s="18"/>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A31" s="52" t="s">
+      <c r="A31" s="59" t="s">
         <v>70</v>
       </c>
-      <c r="B31" s="53"/>
-      <c r="C31" s="54"/>
-      <c r="D31" s="55" t="s">
+      <c r="B31" s="60"/>
+      <c r="C31" s="61"/>
+      <c r="D31" s="62" t="s">
         <v>91</v>
       </c>
-      <c r="E31" s="55" t="s">
+      <c r="E31" s="62" t="s">
         <v>91</v>
       </c>
       <c r="G31" s="20"/>
@@ -35028,12 +35127,12 @@
       <c r="A32" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B32" s="56" t="s">
+      <c r="B32" s="63" t="s">
         <v>5</v>
       </c>
-      <c r="C32" s="56"/>
-      <c r="D32" s="56"/>
-      <c r="E32" s="56"/>
+      <c r="C32" s="63"/>
+      <c r="D32" s="63"/>
+      <c r="E32" s="63"/>
       <c r="G32" s="23"/>
       <c r="H32" s="18"/>
       <c r="I32" s="18"/>
@@ -35059,13 +35158,13 @@
       <c r="I33" s="18"/>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A34" s="57" t="s">
+      <c r="A34" s="64" t="s">
         <v>11</v>
       </c>
-      <c r="B34" s="57"/>
-      <c r="C34" s="57"/>
-      <c r="D34" s="57"/>
-      <c r="E34" s="57"/>
+      <c r="B34" s="64"/>
+      <c r="C34" s="64"/>
+      <c r="D34" s="64"/>
+      <c r="E34" s="64"/>
       <c r="G34" s="23"/>
       <c r="H34" s="18"/>
       <c r="I34" s="18"/>
@@ -35131,13 +35230,13 @@
       <c r="I37" s="18"/>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A38" s="57" t="s">
+      <c r="A38" s="64" t="s">
         <v>12</v>
       </c>
-      <c r="B38" s="57"/>
-      <c r="C38" s="57"/>
-      <c r="D38" s="57"/>
-      <c r="E38" s="57"/>
+      <c r="B38" s="64"/>
+      <c r="C38" s="64"/>
+      <c r="D38" s="64"/>
+      <c r="E38" s="64"/>
       <c r="G38" s="23"/>
       <c r="H38" s="18"/>
       <c r="I38" s="18"/>
@@ -35203,23 +35302,23 @@
       <c r="I41" s="18"/>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B42" s="60" t="s">
+      <c r="B42" s="67" t="s">
         <v>66</v>
       </c>
-      <c r="C42" s="60"/>
-      <c r="D42" s="60"/>
-      <c r="E42" s="60"/>
+      <c r="C42" s="67"/>
+      <c r="D42" s="67"/>
+      <c r="E42" s="67"/>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A44" s="52" t="s">
+      <c r="A44" s="59" t="s">
         <v>82</v>
       </c>
-      <c r="B44" s="53"/>
-      <c r="C44" s="54"/>
-      <c r="D44" s="55" t="s">
+      <c r="B44" s="60"/>
+      <c r="C44" s="61"/>
+      <c r="D44" s="62" t="s">
         <v>92</v>
       </c>
-      <c r="E44" s="55" t="s">
+      <c r="E44" s="62" t="s">
         <v>91</v>
       </c>
     </row>
@@ -35227,12 +35326,12 @@
       <c r="A45" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B45" s="56" t="s">
+      <c r="B45" s="63" t="s">
         <v>5</v>
       </c>
-      <c r="C45" s="56"/>
-      <c r="D45" s="56"/>
-      <c r="E45" s="56"/>
+      <c r="C45" s="63"/>
+      <c r="D45" s="63"/>
+      <c r="E45" s="63"/>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
@@ -35252,13 +35351,13 @@
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A47" s="57" t="s">
+      <c r="A47" s="64" t="s">
         <v>11</v>
       </c>
-      <c r="B47" s="57"/>
-      <c r="C47" s="57"/>
-      <c r="D47" s="57"/>
-      <c r="E47" s="57"/>
+      <c r="B47" s="64"/>
+      <c r="C47" s="64"/>
+      <c r="D47" s="64"/>
+      <c r="E47" s="64"/>
       <c r="G47" s="1" t="s">
         <v>95</v>
       </c>
@@ -35336,13 +35435,13 @@
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A51" s="57" t="s">
+      <c r="A51" s="64" t="s">
         <v>12</v>
       </c>
-      <c r="B51" s="57"/>
-      <c r="C51" s="57"/>
-      <c r="D51" s="57"/>
-      <c r="E51" s="57"/>
+      <c r="B51" s="64"/>
+      <c r="C51" s="64"/>
+      <c r="D51" s="64"/>
+      <c r="E51" s="64"/>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" s="3" t="s">
@@ -35401,15 +35500,15 @@
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A57" s="52" t="s">
+      <c r="A57" s="59" t="s">
         <v>104</v>
       </c>
-      <c r="B57" s="53"/>
-      <c r="C57" s="54"/>
-      <c r="D57" s="55" t="s">
+      <c r="B57" s="60"/>
+      <c r="C57" s="61"/>
+      <c r="D57" s="62" t="s">
         <v>92</v>
       </c>
-      <c r="E57" s="55" t="s">
+      <c r="E57" s="62" t="s">
         <v>91</v>
       </c>
     </row>
@@ -35417,12 +35516,12 @@
       <c r="A58" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B58" s="56" t="s">
+      <c r="B58" s="63" t="s">
         <v>5</v>
       </c>
-      <c r="C58" s="56"/>
-      <c r="D58" s="56"/>
-      <c r="E58" s="56"/>
+      <c r="C58" s="63"/>
+      <c r="D58" s="63"/>
+      <c r="E58" s="63"/>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" s="3" t="s">
@@ -35442,13 +35541,13 @@
       </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A60" s="57" t="s">
+      <c r="A60" s="64" t="s">
         <v>11</v>
       </c>
-      <c r="B60" s="57"/>
-      <c r="C60" s="57"/>
-      <c r="D60" s="57"/>
-      <c r="E60" s="57"/>
+      <c r="B60" s="64"/>
+      <c r="C60" s="64"/>
+      <c r="D60" s="64"/>
+      <c r="E60" s="64"/>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" s="3" t="s">
@@ -35502,13 +35601,13 @@
       </c>
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A64" s="57" t="s">
+      <c r="A64" s="64" t="s">
         <v>12</v>
       </c>
-      <c r="B64" s="57"/>
-      <c r="C64" s="57"/>
-      <c r="D64" s="57"/>
-      <c r="E64" s="57"/>
+      <c r="B64" s="64"/>
+      <c r="C64" s="64"/>
+      <c r="D64" s="64"/>
+      <c r="E64" s="64"/>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="3" t="s">
@@ -35567,15 +35666,15 @@
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A70" s="52" t="s">
+      <c r="A70" s="59" t="s">
         <v>108</v>
       </c>
-      <c r="B70" s="53"/>
-      <c r="C70" s="54"/>
-      <c r="D70" s="55" t="s">
+      <c r="B70" s="60"/>
+      <c r="C70" s="61"/>
+      <c r="D70" s="62" t="s">
         <v>92</v>
       </c>
-      <c r="E70" s="55" t="s">
+      <c r="E70" s="62" t="s">
         <v>91</v>
       </c>
     </row>
@@ -35583,21 +35682,21 @@
       <c r="A71" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B71" s="56" t="s">
+      <c r="B71" s="63" t="s">
         <v>5</v>
       </c>
-      <c r="C71" s="56"/>
-      <c r="D71" s="56"/>
-      <c r="E71" s="56"/>
+      <c r="C71" s="63"/>
+      <c r="D71" s="63"/>
+      <c r="E71" s="63"/>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A72" s="57" t="s">
+      <c r="A72" s="64" t="s">
         <v>109</v>
       </c>
-      <c r="B72" s="57"/>
-      <c r="C72" s="57"/>
-      <c r="D72" s="57"/>
-      <c r="E72" s="57"/>
+      <c r="B72" s="64"/>
+      <c r="C72" s="64"/>
+      <c r="D72" s="64"/>
+      <c r="E72" s="64"/>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" s="3" t="s">
@@ -35668,13 +35767,13 @@
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A77" s="57" t="s">
+      <c r="A77" s="64" t="s">
         <v>110</v>
       </c>
-      <c r="B77" s="57"/>
-      <c r="C77" s="57"/>
-      <c r="D77" s="57"/>
-      <c r="E77" s="57"/>
+      <c r="B77" s="64"/>
+      <c r="C77" s="64"/>
+      <c r="D77" s="64"/>
+      <c r="E77" s="64"/>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" s="3" t="s">
@@ -35746,11 +35845,18 @@
     </row>
   </sheetData>
   <mergeCells count="32">
-    <mergeCell ref="A70:C70"/>
-    <mergeCell ref="D70:E70"/>
-    <mergeCell ref="B71:E71"/>
-    <mergeCell ref="A72:E72"/>
-    <mergeCell ref="A77:E77"/>
+    <mergeCell ref="A57:C57"/>
+    <mergeCell ref="D57:E57"/>
+    <mergeCell ref="B58:E58"/>
+    <mergeCell ref="A60:E60"/>
+    <mergeCell ref="A64:E64"/>
+    <mergeCell ref="B45:E45"/>
+    <mergeCell ref="A47:E47"/>
+    <mergeCell ref="A51:E51"/>
+    <mergeCell ref="D44:E44"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="A44:C44"/>
+    <mergeCell ref="A31:C31"/>
     <mergeCell ref="H24:I24"/>
     <mergeCell ref="G5:H8"/>
     <mergeCell ref="B42:E42"/>
@@ -35766,18 +35872,11 @@
     <mergeCell ref="B19:E19"/>
     <mergeCell ref="A21:E21"/>
     <mergeCell ref="A25:E25"/>
-    <mergeCell ref="B45:E45"/>
-    <mergeCell ref="A47:E47"/>
-    <mergeCell ref="A51:E51"/>
-    <mergeCell ref="D44:E44"/>
-    <mergeCell ref="D31:E31"/>
-    <mergeCell ref="A44:C44"/>
-    <mergeCell ref="A31:C31"/>
-    <mergeCell ref="A57:C57"/>
-    <mergeCell ref="D57:E57"/>
-    <mergeCell ref="B58:E58"/>
-    <mergeCell ref="A60:E60"/>
-    <mergeCell ref="A64:E64"/>
+    <mergeCell ref="A70:C70"/>
+    <mergeCell ref="D70:E70"/>
+    <mergeCell ref="B71:E71"/>
+    <mergeCell ref="A72:E72"/>
+    <mergeCell ref="A77:E77"/>
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <hyperlinks>
@@ -35796,7 +35895,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:AC167"/>
+  <dimension ref="A1:AC175"/>
   <sheetFormatPr defaultRowHeight="21.6" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.28515625" style="26" customWidth="1"/>
@@ -35809,24 +35908,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="64" t="s">
+      <c r="A1" s="71" t="s">
         <v>84</v>
       </c>
-      <c r="B1" s="64"/>
-      <c r="C1" s="64"/>
-      <c r="D1" s="64"/>
-      <c r="E1" s="64"/>
-      <c r="F1" s="64"/>
-      <c r="G1" s="64"/>
-      <c r="H1" s="64"/>
-      <c r="I1" s="64"/>
-      <c r="J1" s="64"/>
-      <c r="K1" s="64"/>
-      <c r="L1" s="64"/>
-      <c r="M1" s="55" t="s">
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="71"/>
+      <c r="K1" s="71"/>
+      <c r="L1" s="71"/>
+      <c r="M1" s="62" t="s">
         <v>90</v>
       </c>
-      <c r="N1" s="55"/>
+      <c r="N1" s="62"/>
       <c r="O1" s="36"/>
       <c r="P1" s="35"/>
       <c r="Q1" s="35"/>
@@ -35841,14 +35940,14 @@
       <c r="Z1" s="35"/>
     </row>
     <row r="2" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="82" t="s">
+      <c r="A2" s="81" t="s">
         <v>85</v>
       </c>
-      <c r="B2" s="77" t="s">
+      <c r="B2" s="73" t="s">
         <v>78</v>
       </c>
-      <c r="C2" s="78"/>
-      <c r="D2" s="79"/>
+      <c r="C2" s="74"/>
+      <c r="D2" s="75"/>
       <c r="E2" s="31"/>
       <c r="F2" s="31"/>
       <c r="G2" s="31"/>
@@ -35873,7 +35972,7 @@
       <c r="Z2" s="30"/>
     </row>
     <row r="3" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="82"/>
+      <c r="A3" s="81"/>
       <c r="B3" s="29" t="s">
         <v>77</v>
       </c>
@@ -35907,7 +36006,7 @@
       <c r="Z3" s="30"/>
     </row>
     <row r="4" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="82"/>
+      <c r="A4" s="81"/>
       <c r="B4" s="15">
         <v>1</v>
       </c>
@@ -35941,7 +36040,7 @@
       <c r="Z4" s="30"/>
     </row>
     <row r="5" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="82"/>
+      <c r="A5" s="81"/>
       <c r="B5" s="15">
         <v>2</v>
       </c>
@@ -35975,7 +36074,7 @@
       <c r="Z5" s="30"/>
     </row>
     <row r="6" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="82"/>
+      <c r="A6" s="81"/>
       <c r="B6" s="15">
         <v>4</v>
       </c>
@@ -35998,7 +36097,7 @@
       <c r="O6" s="38"/>
     </row>
     <row r="7" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="82"/>
+      <c r="A7" s="81"/>
       <c r="B7" s="15">
         <v>6</v>
       </c>
@@ -36021,7 +36120,7 @@
       <c r="O7" s="38"/>
     </row>
     <row r="8" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="82"/>
+      <c r="A8" s="81"/>
       <c r="B8" s="15">
         <v>8</v>
       </c>
@@ -36044,7 +36143,7 @@
       <c r="O8" s="38"/>
     </row>
     <row r="9" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="82"/>
+      <c r="A9" s="81"/>
       <c r="B9" s="15">
         <v>10</v>
       </c>
@@ -36067,7 +36166,7 @@
       <c r="O9" s="38"/>
     </row>
     <row r="10" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="82"/>
+      <c r="A10" s="81"/>
       <c r="B10" s="15">
         <v>12</v>
       </c>
@@ -36090,7 +36189,7 @@
       <c r="O10" s="38"/>
     </row>
     <row r="11" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="82"/>
+      <c r="A11" s="81"/>
       <c r="B11" s="15">
         <v>16</v>
       </c>
@@ -36115,37 +36214,37 @@
       <c r="Q11" s="27"/>
     </row>
     <row r="12" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="82"/>
+      <c r="A12" s="81"/>
       <c r="B12" s="33" t="s">
         <v>86</v>
       </c>
-      <c r="C12" s="80" t="s">
+      <c r="C12" s="82" t="s">
         <v>81</v>
       </c>
-      <c r="D12" s="80"/>
-      <c r="E12" s="80"/>
-      <c r="F12" s="80"/>
-      <c r="G12" s="80"/>
-      <c r="H12" s="80"/>
-      <c r="I12" s="80"/>
-      <c r="J12" s="80"/>
-      <c r="K12" s="80"/>
-      <c r="L12" s="80"/>
-      <c r="M12" s="80"/>
-      <c r="N12" s="81"/>
+      <c r="D12" s="82"/>
+      <c r="E12" s="82"/>
+      <c r="F12" s="82"/>
+      <c r="G12" s="82"/>
+      <c r="H12" s="82"/>
+      <c r="I12" s="82"/>
+      <c r="J12" s="82"/>
+      <c r="K12" s="82"/>
+      <c r="L12" s="82"/>
+      <c r="M12" s="82"/>
+      <c r="N12" s="78"/>
       <c r="O12" s="39"/>
       <c r="P12" s="23"/>
       <c r="Q12" s="23"/>
     </row>
     <row r="13" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="82" t="s">
+      <c r="A13" s="81" t="s">
         <v>87</v>
       </c>
-      <c r="B13" s="77" t="s">
+      <c r="B13" s="73" t="s">
         <v>78</v>
       </c>
-      <c r="C13" s="78"/>
-      <c r="D13" s="79"/>
+      <c r="C13" s="74"/>
+      <c r="D13" s="75"/>
       <c r="E13" s="32"/>
       <c r="F13" s="31"/>
       <c r="G13" s="31"/>
@@ -36161,7 +36260,7 @@
       <c r="Q13" s="23"/>
     </row>
     <row r="14" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="82"/>
+      <c r="A14" s="81"/>
       <c r="B14" s="13" t="s">
         <v>77</v>
       </c>
@@ -36186,7 +36285,7 @@
       <c r="Q14" s="23"/>
     </row>
     <row r="15" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="82"/>
+      <c r="A15" s="81"/>
       <c r="B15" s="15">
         <v>1</v>
       </c>
@@ -36211,7 +36310,7 @@
       <c r="Q15" s="27"/>
     </row>
     <row r="16" spans="1:26" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="82"/>
+      <c r="A16" s="81"/>
       <c r="B16" s="15">
         <v>2</v>
       </c>
@@ -36236,7 +36335,7 @@
       <c r="Q16" s="23"/>
     </row>
     <row r="17" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="82"/>
+      <c r="A17" s="81"/>
       <c r="B17" s="15">
         <v>4</v>
       </c>
@@ -36261,7 +36360,7 @@
       <c r="Q17" s="23"/>
     </row>
     <row r="18" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="82"/>
+      <c r="A18" s="81"/>
       <c r="B18" s="15">
         <v>6</v>
       </c>
@@ -36286,7 +36385,7 @@
       <c r="Q18" s="23"/>
     </row>
     <row r="19" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="82"/>
+      <c r="A19" s="81"/>
       <c r="B19" s="15">
         <v>8</v>
       </c>
@@ -36309,7 +36408,7 @@
       <c r="O19" s="38"/>
     </row>
     <row r="20" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="82"/>
+      <c r="A20" s="81"/>
       <c r="B20" s="15">
         <v>10</v>
       </c>
@@ -36332,7 +36431,7 @@
       <c r="O20" s="38"/>
     </row>
     <row r="21" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="82"/>
+      <c r="A21" s="81"/>
       <c r="B21" s="15">
         <v>12</v>
       </c>
@@ -36355,7 +36454,7 @@
       <c r="O21" s="38"/>
     </row>
     <row r="22" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="82"/>
+      <c r="A22" s="81"/>
       <c r="B22" s="83" t="s">
         <v>86</v>
       </c>
@@ -36376,7 +36475,7 @@
       <c r="O22" s="38"/>
     </row>
     <row r="23" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="82"/>
+      <c r="A23" s="81"/>
       <c r="B23" s="83"/>
       <c r="C23" s="84"/>
       <c r="D23" s="84"/>
@@ -36393,35 +36492,35 @@
       <c r="O23" s="38"/>
     </row>
     <row r="24" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="64" t="s">
+      <c r="A24" s="71" t="s">
         <v>89</v>
       </c>
-      <c r="B24" s="64"/>
-      <c r="C24" s="64"/>
-      <c r="D24" s="64"/>
-      <c r="E24" s="64"/>
-      <c r="F24" s="64"/>
-      <c r="G24" s="64"/>
-      <c r="H24" s="64"/>
-      <c r="I24" s="64"/>
-      <c r="J24" s="64"/>
-      <c r="K24" s="64"/>
-      <c r="L24" s="64"/>
-      <c r="M24" s="55" t="s">
+      <c r="B24" s="71"/>
+      <c r="C24" s="71"/>
+      <c r="D24" s="71"/>
+      <c r="E24" s="71"/>
+      <c r="F24" s="71"/>
+      <c r="G24" s="71"/>
+      <c r="H24" s="71"/>
+      <c r="I24" s="71"/>
+      <c r="J24" s="71"/>
+      <c r="K24" s="71"/>
+      <c r="L24" s="71"/>
+      <c r="M24" s="62" t="s">
         <v>90</v>
       </c>
-      <c r="N24" s="55"/>
+      <c r="N24" s="62"/>
       <c r="O24" s="38"/>
     </row>
     <row r="25" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="68" t="s">
+      <c r="A25" s="89" t="s">
         <v>85</v>
       </c>
-      <c r="B25" s="77" t="s">
+      <c r="B25" s="73" t="s">
         <v>78</v>
       </c>
-      <c r="C25" s="78"/>
-      <c r="D25" s="79"/>
+      <c r="C25" s="74"/>
+      <c r="D25" s="75"/>
       <c r="E25" s="31"/>
       <c r="F25" s="31"/>
       <c r="G25" s="31"/>
@@ -36435,7 +36534,7 @@
       <c r="O25" s="27"/>
     </row>
     <row r="26" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="69"/>
+      <c r="A26" s="90"/>
       <c r="B26" s="42" t="s">
         <v>77</v>
       </c>
@@ -36458,7 +36557,7 @@
       <c r="O26" s="27"/>
     </row>
     <row r="27" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="69"/>
+      <c r="A27" s="90"/>
       <c r="B27" s="15">
         <v>1</v>
       </c>
@@ -36481,7 +36580,7 @@
       <c r="O27" s="27"/>
     </row>
     <row r="28" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="69"/>
+      <c r="A28" s="90"/>
       <c r="B28" s="15">
         <v>2</v>
       </c>
@@ -36504,7 +36603,7 @@
       <c r="O28" s="27"/>
     </row>
     <row r="29" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="69"/>
+      <c r="A29" s="90"/>
       <c r="B29" s="15">
         <v>4</v>
       </c>
@@ -36527,7 +36626,7 @@
       <c r="O29" s="27"/>
     </row>
     <row r="30" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="69"/>
+      <c r="A30" s="90"/>
       <c r="B30" s="15">
         <v>6</v>
       </c>
@@ -36550,7 +36649,7 @@
       <c r="O30" s="27"/>
     </row>
     <row r="31" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="69"/>
+      <c r="A31" s="90"/>
       <c r="B31" s="15">
         <v>8</v>
       </c>
@@ -36573,7 +36672,7 @@
       <c r="O31" s="27"/>
     </row>
     <row r="32" spans="1:17" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="69"/>
+      <c r="A32" s="90"/>
       <c r="B32" s="15">
         <v>10</v>
       </c>
@@ -36596,7 +36695,7 @@
       <c r="O32" s="27"/>
     </row>
     <row r="33" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="69"/>
+      <c r="A33" s="90"/>
       <c r="B33" s="15">
         <v>12</v>
       </c>
@@ -36619,7 +36718,7 @@
       <c r="O33" s="27"/>
     </row>
     <row r="34" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="69"/>
+      <c r="A34" s="90"/>
       <c r="B34" s="15">
         <v>16</v>
       </c>
@@ -36642,12 +36741,12 @@
       <c r="O34" s="27"/>
     </row>
     <row r="35" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="69"/>
-      <c r="B35" s="77" t="s">
+      <c r="A35" s="90"/>
+      <c r="B35" s="73" t="s">
         <v>96</v>
       </c>
-      <c r="C35" s="78"/>
-      <c r="D35" s="79"/>
+      <c r="C35" s="74"/>
+      <c r="D35" s="75"/>
       <c r="E35" s="31"/>
       <c r="F35" s="31"/>
       <c r="G35" s="31"/>
@@ -36661,7 +36760,7 @@
       <c r="O35" s="27"/>
     </row>
     <row r="36" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="69"/>
+      <c r="A36" s="90"/>
       <c r="B36" s="42" t="s">
         <v>77</v>
       </c>
@@ -36685,7 +36784,7 @@
       <c r="P36" s="1"/>
     </row>
     <row r="37" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="69"/>
+      <c r="A37" s="90"/>
       <c r="B37" s="42">
         <v>1</v>
       </c>
@@ -36711,7 +36810,7 @@
       <c r="P37" s="1"/>
     </row>
     <row r="38" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="69"/>
+      <c r="A38" s="90"/>
       <c r="B38" s="42">
         <v>2</v>
       </c>
@@ -36737,7 +36836,7 @@
       <c r="P38" s="1"/>
     </row>
     <row r="39" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="69"/>
+      <c r="A39" s="90"/>
       <c r="B39" s="42">
         <v>4</v>
       </c>
@@ -36763,7 +36862,7 @@
       <c r="P39" s="1"/>
     </row>
     <row r="40" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="69"/>
+      <c r="A40" s="90"/>
       <c r="B40" s="42">
         <v>6</v>
       </c>
@@ -36789,7 +36888,7 @@
       <c r="P40" s="1"/>
     </row>
     <row r="41" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="69"/>
+      <c r="A41" s="90"/>
       <c r="B41" s="42">
         <v>8</v>
       </c>
@@ -36815,7 +36914,7 @@
       <c r="P41" s="1"/>
     </row>
     <row r="42" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="69"/>
+      <c r="A42" s="90"/>
       <c r="B42" s="42">
         <v>10</v>
       </c>
@@ -36841,7 +36940,7 @@
       <c r="P42" s="1"/>
     </row>
     <row r="43" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="69"/>
+      <c r="A43" s="90"/>
       <c r="B43" s="42">
         <v>12</v>
       </c>
@@ -36867,7 +36966,7 @@
       <c r="P43" s="1"/>
     </row>
     <row r="44" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="69"/>
+      <c r="A44" s="90"/>
       <c r="B44" s="42">
         <v>16</v>
       </c>
@@ -36893,12 +36992,12 @@
       <c r="P44" s="1"/>
     </row>
     <row r="45" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="69"/>
-      <c r="B45" s="77" t="s">
+      <c r="A45" s="90"/>
+      <c r="B45" s="73" t="s">
         <v>97</v>
       </c>
-      <c r="C45" s="78"/>
-      <c r="D45" s="79"/>
+      <c r="C45" s="74"/>
+      <c r="D45" s="75"/>
       <c r="E45" s="43"/>
       <c r="F45" s="43"/>
       <c r="G45" s="43"/>
@@ -36913,7 +37012,7 @@
       <c r="P45" s="1"/>
     </row>
     <row r="46" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="69"/>
+      <c r="A46" s="90"/>
       <c r="B46" s="42" t="s">
         <v>77</v>
       </c>
@@ -36937,7 +37036,7 @@
       <c r="P46" s="1"/>
     </row>
     <row r="47" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="69"/>
+      <c r="A47" s="90"/>
       <c r="B47" s="42">
         <v>1</v>
       </c>
@@ -36963,7 +37062,7 @@
       <c r="P47" s="1"/>
     </row>
     <row r="48" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="69"/>
+      <c r="A48" s="90"/>
       <c r="B48" s="42">
         <v>2</v>
       </c>
@@ -36989,7 +37088,7 @@
       <c r="P48" s="1"/>
     </row>
     <row r="49" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="69"/>
+      <c r="A49" s="90"/>
       <c r="B49" s="42">
         <v>4</v>
       </c>
@@ -37015,7 +37114,7 @@
       <c r="P49" s="1"/>
     </row>
     <row r="50" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="69"/>
+      <c r="A50" s="90"/>
       <c r="B50" s="42">
         <v>6</v>
       </c>
@@ -37041,7 +37140,7 @@
       <c r="P50" s="1"/>
     </row>
     <row r="51" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="69"/>
+      <c r="A51" s="90"/>
       <c r="B51" s="42">
         <v>8</v>
       </c>
@@ -37066,7 +37165,7 @@
       <c r="O51" s="1"/>
     </row>
     <row r="52" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="69"/>
+      <c r="A52" s="90"/>
       <c r="B52" s="42">
         <v>10</v>
       </c>
@@ -37091,7 +37190,7 @@
       <c r="O52" s="1"/>
     </row>
     <row r="53" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="69"/>
+      <c r="A53" s="90"/>
       <c r="B53" s="42">
         <v>12</v>
       </c>
@@ -37116,7 +37215,7 @@
       <c r="O53" s="1"/>
     </row>
     <row r="54" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="69"/>
+      <c r="A54" s="90"/>
       <c r="B54" s="42">
         <v>16</v>
       </c>
@@ -37141,55 +37240,55 @@
       <c r="O54" s="1"/>
     </row>
     <row r="55" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="69"/>
+      <c r="A55" s="90"/>
       <c r="B55" s="46" t="s">
         <v>86</v>
       </c>
-      <c r="C55" s="73" t="s">
+      <c r="C55" s="94" t="s">
         <v>102</v>
       </c>
-      <c r="D55" s="73"/>
-      <c r="E55" s="73"/>
-      <c r="F55" s="73"/>
-      <c r="G55" s="73"/>
-      <c r="H55" s="73"/>
-      <c r="I55" s="73"/>
-      <c r="J55" s="73"/>
-      <c r="K55" s="73"/>
-      <c r="L55" s="73"/>
-      <c r="M55" s="73"/>
-      <c r="N55" s="73"/>
+      <c r="D55" s="94"/>
+      <c r="E55" s="94"/>
+      <c r="F55" s="94"/>
+      <c r="G55" s="94"/>
+      <c r="H55" s="94"/>
+      <c r="I55" s="94"/>
+      <c r="J55" s="94"/>
+      <c r="K55" s="94"/>
+      <c r="L55" s="94"/>
+      <c r="M55" s="94"/>
+      <c r="N55" s="94"/>
     </row>
     <row r="56" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="74" t="s">
+      <c r="A56" s="95" t="s">
         <v>103</v>
       </c>
-      <c r="B56" s="75"/>
-      <c r="C56" s="75"/>
-      <c r="D56" s="75"/>
-      <c r="E56" s="75"/>
-      <c r="F56" s="75"/>
-      <c r="G56" s="75"/>
-      <c r="H56" s="75"/>
-      <c r="I56" s="75"/>
-      <c r="J56" s="75"/>
-      <c r="K56" s="75"/>
-      <c r="L56" s="76"/>
-      <c r="M56" s="55" t="s">
+      <c r="B56" s="96"/>
+      <c r="C56" s="96"/>
+      <c r="D56" s="96"/>
+      <c r="E56" s="96"/>
+      <c r="F56" s="96"/>
+      <c r="G56" s="96"/>
+      <c r="H56" s="96"/>
+      <c r="I56" s="96"/>
+      <c r="J56" s="96"/>
+      <c r="K56" s="96"/>
+      <c r="L56" s="97"/>
+      <c r="M56" s="62" t="s">
         <v>90</v>
       </c>
-      <c r="N56" s="55"/>
+      <c r="N56" s="62"/>
       <c r="O56" s="30"/>
     </row>
     <row r="57" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="68" t="s">
+      <c r="A57" s="89" t="s">
         <v>85</v>
       </c>
-      <c r="B57" s="77" t="s">
+      <c r="B57" s="73" t="s">
         <v>78</v>
       </c>
-      <c r="C57" s="78"/>
-      <c r="D57" s="79"/>
+      <c r="C57" s="74"/>
+      <c r="D57" s="75"/>
       <c r="E57" s="31"/>
       <c r="F57" s="31"/>
       <c r="G57" s="31"/>
@@ -37203,7 +37302,7 @@
       <c r="O57" s="30"/>
     </row>
     <row r="58" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="69"/>
+      <c r="A58" s="90"/>
       <c r="B58" s="42" t="s">
         <v>77</v>
       </c>
@@ -37226,7 +37325,7 @@
       <c r="O58" s="30"/>
     </row>
     <row r="59" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="69"/>
+      <c r="A59" s="90"/>
       <c r="B59" s="15">
         <v>1</v>
       </c>
@@ -37249,7 +37348,7 @@
       <c r="O59" s="30"/>
     </row>
     <row r="60" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="69"/>
+      <c r="A60" s="90"/>
       <c r="B60" s="15">
         <v>2</v>
       </c>
@@ -37272,7 +37371,7 @@
       <c r="O60" s="30"/>
     </row>
     <row r="61" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="69"/>
+      <c r="A61" s="90"/>
       <c r="B61" s="15">
         <v>4</v>
       </c>
@@ -37295,7 +37394,7 @@
       <c r="O61" s="30"/>
     </row>
     <row r="62" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="69"/>
+      <c r="A62" s="90"/>
       <c r="B62" s="15">
         <v>6</v>
       </c>
@@ -37318,7 +37417,7 @@
       <c r="O62" s="30"/>
     </row>
     <row r="63" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="69"/>
+      <c r="A63" s="90"/>
       <c r="B63" s="15">
         <v>8</v>
       </c>
@@ -37341,7 +37440,7 @@
       <c r="O63" s="30"/>
     </row>
     <row r="64" spans="1:16" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="69"/>
+      <c r="A64" s="90"/>
       <c r="B64" s="15">
         <v>10</v>
       </c>
@@ -37364,7 +37463,7 @@
       <c r="O64" s="30"/>
     </row>
     <row r="65" spans="1:15" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="69"/>
+      <c r="A65" s="90"/>
       <c r="B65" s="15">
         <v>12</v>
       </c>
@@ -37387,7 +37486,7 @@
       <c r="O65" s="30"/>
     </row>
     <row r="66" spans="1:15" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="69"/>
+      <c r="A66" s="90"/>
       <c r="B66" s="15">
         <v>16</v>
       </c>
@@ -37410,12 +37509,12 @@
       <c r="O66" s="30"/>
     </row>
     <row r="67" spans="1:15" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="69"/>
-      <c r="B67" s="77" t="s">
+      <c r="A67" s="90"/>
+      <c r="B67" s="73" t="s">
         <v>96</v>
       </c>
-      <c r="C67" s="78"/>
-      <c r="D67" s="79"/>
+      <c r="C67" s="74"/>
+      <c r="D67" s="75"/>
       <c r="E67" s="31"/>
       <c r="F67" s="31"/>
       <c r="G67" s="31"/>
@@ -37429,7 +37528,7 @@
       <c r="O67" s="30"/>
     </row>
     <row r="68" spans="1:15" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="69"/>
+      <c r="A68" s="90"/>
       <c r="B68" s="42" t="s">
         <v>77</v>
       </c>
@@ -37452,7 +37551,7 @@
       <c r="O68" s="30"/>
     </row>
     <row r="69" spans="1:15" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="69"/>
+      <c r="A69" s="90"/>
       <c r="B69" s="42">
         <v>1</v>
       </c>
@@ -37477,7 +37576,7 @@
       <c r="O69" s="30"/>
     </row>
     <row r="70" spans="1:15" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="69"/>
+      <c r="A70" s="90"/>
       <c r="B70" s="42">
         <v>2</v>
       </c>
@@ -37502,7 +37601,7 @@
       <c r="O70" s="30"/>
     </row>
     <row r="71" spans="1:15" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="69"/>
+      <c r="A71" s="90"/>
       <c r="B71" s="42">
         <v>4</v>
       </c>
@@ -37527,7 +37626,7 @@
       <c r="O71" s="30"/>
     </row>
     <row r="72" spans="1:15" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="69"/>
+      <c r="A72" s="90"/>
       <c r="B72" s="42">
         <v>6</v>
       </c>
@@ -37552,7 +37651,7 @@
       <c r="O72" s="30"/>
     </row>
     <row r="73" spans="1:15" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="69"/>
+      <c r="A73" s="90"/>
       <c r="B73" s="42">
         <v>8</v>
       </c>
@@ -37577,7 +37676,7 @@
       <c r="O73" s="30"/>
     </row>
     <row r="74" spans="1:15" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A74" s="69"/>
+      <c r="A74" s="90"/>
       <c r="B74" s="42">
         <v>10</v>
       </c>
@@ -37602,7 +37701,7 @@
       <c r="O74" s="30"/>
     </row>
     <row r="75" spans="1:15" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A75" s="69"/>
+      <c r="A75" s="90"/>
       <c r="B75" s="42">
         <v>12</v>
       </c>
@@ -37627,7 +37726,7 @@
       <c r="O75" s="30"/>
     </row>
     <row r="76" spans="1:15" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="69"/>
+      <c r="A76" s="90"/>
       <c r="B76" s="42">
         <v>16</v>
       </c>
@@ -37652,12 +37751,12 @@
       <c r="O76" s="30"/>
     </row>
     <row r="77" spans="1:15" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="69"/>
-      <c r="B77" s="77" t="s">
+      <c r="A77" s="90"/>
+      <c r="B77" s="73" t="s">
         <v>97</v>
       </c>
-      <c r="C77" s="78"/>
-      <c r="D77" s="79"/>
+      <c r="C77" s="74"/>
+      <c r="D77" s="75"/>
       <c r="E77" s="43"/>
       <c r="F77" s="43"/>
       <c r="G77" s="43"/>
@@ -37671,7 +37770,7 @@
       <c r="O77" s="30"/>
     </row>
     <row r="78" spans="1:15" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A78" s="69"/>
+      <c r="A78" s="90"/>
       <c r="B78" s="42" t="s">
         <v>77</v>
       </c>
@@ -37694,7 +37793,7 @@
       <c r="O78" s="30"/>
     </row>
     <row r="79" spans="1:15" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A79" s="69"/>
+      <c r="A79" s="90"/>
       <c r="B79" s="42">
         <v>1</v>
       </c>
@@ -37719,7 +37818,7 @@
       <c r="O79" s="30"/>
     </row>
     <row r="80" spans="1:15" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A80" s="69"/>
+      <c r="A80" s="90"/>
       <c r="B80" s="42">
         <v>2</v>
       </c>
@@ -37744,7 +37843,7 @@
       <c r="O80" s="30"/>
     </row>
     <row r="81" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="69"/>
+      <c r="A81" s="90"/>
       <c r="B81" s="42">
         <v>4</v>
       </c>
@@ -37769,7 +37868,7 @@
       <c r="O81" s="30"/>
     </row>
     <row r="82" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A82" s="69"/>
+      <c r="A82" s="90"/>
       <c r="B82" s="42">
         <v>6</v>
       </c>
@@ -37794,7 +37893,7 @@
       <c r="O82" s="30"/>
     </row>
     <row r="83" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="69"/>
+      <c r="A83" s="90"/>
       <c r="B83" s="42">
         <v>8</v>
       </c>
@@ -37819,7 +37918,7 @@
       <c r="O83" s="30"/>
     </row>
     <row r="84" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A84" s="69"/>
+      <c r="A84" s="90"/>
       <c r="B84" s="42">
         <v>10</v>
       </c>
@@ -37844,7 +37943,7 @@
       <c r="O84" s="30"/>
     </row>
     <row r="85" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A85" s="69"/>
+      <c r="A85" s="90"/>
       <c r="B85" s="42">
         <v>12</v>
       </c>
@@ -37869,7 +37968,7 @@
       <c r="O85" s="30"/>
     </row>
     <row r="86" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A86" s="69"/>
+      <c r="A86" s="90"/>
       <c r="B86" s="42">
         <v>16</v>
       </c>
@@ -37894,61 +37993,61 @@
       <c r="O86" s="30"/>
     </row>
     <row r="87" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A87" s="69"/>
+      <c r="A87" s="90"/>
       <c r="B87" s="46" t="s">
         <v>86</v>
       </c>
-      <c r="C87" s="70" t="s">
+      <c r="C87" s="91" t="s">
         <v>106</v>
       </c>
-      <c r="D87" s="71"/>
-      <c r="E87" s="71"/>
-      <c r="F87" s="71"/>
-      <c r="G87" s="71"/>
-      <c r="H87" s="71"/>
-      <c r="I87" s="71"/>
-      <c r="J87" s="71"/>
-      <c r="K87" s="71"/>
-      <c r="L87" s="71"/>
-      <c r="M87" s="71"/>
-      <c r="N87" s="72"/>
+      <c r="D87" s="92"/>
+      <c r="E87" s="92"/>
+      <c r="F87" s="92"/>
+      <c r="G87" s="92"/>
+      <c r="H87" s="92"/>
+      <c r="I87" s="92"/>
+      <c r="J87" s="92"/>
+      <c r="K87" s="92"/>
+      <c r="L87" s="92"/>
+      <c r="M87" s="92"/>
+      <c r="N87" s="93"/>
     </row>
     <row r="88" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A88" s="52" t="s">
+      <c r="A88" s="59" t="s">
         <v>107</v>
       </c>
-      <c r="B88" s="53"/>
-      <c r="C88" s="53"/>
-      <c r="D88" s="53"/>
-      <c r="E88" s="53"/>
-      <c r="F88" s="53"/>
-      <c r="G88" s="53"/>
-      <c r="H88" s="53"/>
-      <c r="I88" s="53"/>
-      <c r="J88" s="53"/>
-      <c r="K88" s="53"/>
-      <c r="L88" s="53"/>
-      <c r="M88" s="53"/>
-      <c r="N88" s="53"/>
-      <c r="O88" s="65" t="s">
+      <c r="B88" s="60"/>
+      <c r="C88" s="60"/>
+      <c r="D88" s="60"/>
+      <c r="E88" s="60"/>
+      <c r="F88" s="60"/>
+      <c r="G88" s="60"/>
+      <c r="H88" s="60"/>
+      <c r="I88" s="60"/>
+      <c r="J88" s="60"/>
+      <c r="K88" s="60"/>
+      <c r="L88" s="60"/>
+      <c r="M88" s="60"/>
+      <c r="N88" s="60"/>
+      <c r="O88" s="86" t="s">
         <v>112</v>
       </c>
-      <c r="P88" s="66"/>
-      <c r="Q88" s="66"/>
-      <c r="R88" s="66"/>
-      <c r="S88" s="66"/>
-      <c r="T88" s="67"/>
+      <c r="P88" s="87"/>
+      <c r="Q88" s="87"/>
+      <c r="R88" s="87"/>
+      <c r="S88" s="87"/>
+      <c r="T88" s="88"/>
     </row>
     <row r="89" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A89" s="82" t="s">
+      <c r="A89" s="81" t="s">
         <v>85</v>
       </c>
-      <c r="B89" s="77" t="s">
+      <c r="B89" s="73" t="s">
         <v>78</v>
       </c>
-      <c r="C89" s="78"/>
-      <c r="D89" s="78"/>
-      <c r="E89" s="79"/>
+      <c r="C89" s="74"/>
+      <c r="D89" s="74"/>
+      <c r="E89" s="75"/>
       <c r="F89" s="31"/>
       <c r="G89" s="31"/>
       <c r="H89" s="31"/>
@@ -37966,7 +38065,7 @@
       <c r="T89" s="31"/>
     </row>
     <row r="90" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A90" s="82"/>
+      <c r="A90" s="81"/>
       <c r="B90" s="42" t="s">
         <v>77</v>
       </c>
@@ -37996,7 +38095,7 @@
       <c r="T90" s="31"/>
     </row>
     <row r="91" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A91" s="82"/>
+      <c r="A91" s="81"/>
       <c r="B91" s="15">
         <v>1</v>
       </c>
@@ -38026,7 +38125,7 @@
       <c r="T91" s="31"/>
     </row>
     <row r="92" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A92" s="82"/>
+      <c r="A92" s="81"/>
       <c r="B92" s="15">
         <v>2</v>
       </c>
@@ -38056,7 +38155,7 @@
       <c r="T92" s="31"/>
     </row>
     <row r="93" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A93" s="82"/>
+      <c r="A93" s="81"/>
       <c r="B93" s="15">
         <v>4</v>
       </c>
@@ -38086,7 +38185,7 @@
       <c r="T93" s="31"/>
     </row>
     <row r="94" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A94" s="82"/>
+      <c r="A94" s="81"/>
       <c r="B94" s="15">
         <v>6</v>
       </c>
@@ -38116,7 +38215,7 @@
       <c r="T94" s="31"/>
     </row>
     <row r="95" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A95" s="82"/>
+      <c r="A95" s="81"/>
       <c r="B95" s="15">
         <v>8</v>
       </c>
@@ -38146,7 +38245,7 @@
       <c r="T95" s="31"/>
     </row>
     <row r="96" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A96" s="82"/>
+      <c r="A96" s="81"/>
       <c r="B96" s="15">
         <v>10</v>
       </c>
@@ -38176,7 +38275,7 @@
       <c r="T96" s="31"/>
     </row>
     <row r="97" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A97" s="82"/>
+      <c r="A97" s="81"/>
       <c r="B97" s="15">
         <v>12</v>
       </c>
@@ -38206,7 +38305,7 @@
       <c r="T97" s="31"/>
     </row>
     <row r="98" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A98" s="82"/>
+      <c r="A98" s="81"/>
       <c r="B98" s="15">
         <v>16</v>
       </c>
@@ -38236,13 +38335,13 @@
       <c r="T98" s="31"/>
     </row>
     <row r="99" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A99" s="82"/>
-      <c r="B99" s="77" t="s">
+      <c r="A99" s="81"/>
+      <c r="B99" s="73" t="s">
         <v>96</v>
       </c>
-      <c r="C99" s="78"/>
-      <c r="D99" s="78"/>
-      <c r="E99" s="79"/>
+      <c r="C99" s="74"/>
+      <c r="D99" s="74"/>
+      <c r="E99" s="75"/>
       <c r="F99" s="31"/>
       <c r="G99" s="31"/>
       <c r="H99" s="31"/>
@@ -38260,7 +38359,7 @@
       <c r="T99" s="31"/>
     </row>
     <row r="100" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A100" s="82"/>
+      <c r="A100" s="81"/>
       <c r="B100" s="42" t="s">
         <v>77</v>
       </c>
@@ -38290,7 +38389,7 @@
       <c r="T100" s="16"/>
     </row>
     <row r="101" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A101" s="82"/>
+      <c r="A101" s="81"/>
       <c r="B101" s="42">
         <v>1</v>
       </c>
@@ -38323,7 +38422,7 @@
       <c r="T101" s="16"/>
     </row>
     <row r="102" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A102" s="82"/>
+      <c r="A102" s="81"/>
       <c r="B102" s="42">
         <v>2</v>
       </c>
@@ -38356,7 +38455,7 @@
       <c r="T102" s="16"/>
     </row>
     <row r="103" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A103" s="82"/>
+      <c r="A103" s="81"/>
       <c r="B103" s="42">
         <v>4</v>
       </c>
@@ -38389,7 +38488,7 @@
       <c r="T103" s="16"/>
     </row>
     <row r="104" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A104" s="82"/>
+      <c r="A104" s="81"/>
       <c r="B104" s="42">
         <v>6</v>
       </c>
@@ -38422,7 +38521,7 @@
       <c r="T104" s="16"/>
     </row>
     <row r="105" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A105" s="82"/>
+      <c r="A105" s="81"/>
       <c r="B105" s="42">
         <v>8</v>
       </c>
@@ -38455,7 +38554,7 @@
       <c r="T105" s="16"/>
     </row>
     <row r="106" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A106" s="82"/>
+      <c r="A106" s="81"/>
       <c r="B106" s="42">
         <v>10</v>
       </c>
@@ -38488,7 +38587,7 @@
       <c r="T106" s="16"/>
     </row>
     <row r="107" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A107" s="82"/>
+      <c r="A107" s="81"/>
       <c r="B107" s="42">
         <v>12</v>
       </c>
@@ -38521,7 +38620,7 @@
       <c r="T107" s="16"/>
     </row>
     <row r="108" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A108" s="82"/>
+      <c r="A108" s="81"/>
       <c r="B108" s="42">
         <v>16</v>
       </c>
@@ -38554,13 +38653,13 @@
       <c r="T108" s="16"/>
     </row>
     <row r="109" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A109" s="82"/>
-      <c r="B109" s="77" t="s">
+      <c r="A109" s="81"/>
+      <c r="B109" s="73" t="s">
         <v>97</v>
       </c>
-      <c r="C109" s="78"/>
-      <c r="D109" s="78"/>
-      <c r="E109" s="79"/>
+      <c r="C109" s="74"/>
+      <c r="D109" s="74"/>
+      <c r="E109" s="75"/>
       <c r="F109" s="43"/>
       <c r="G109" s="16"/>
       <c r="H109" s="16"/>
@@ -38578,7 +38677,7 @@
       <c r="T109" s="16"/>
     </row>
     <row r="110" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A110" s="82"/>
+      <c r="A110" s="81"/>
       <c r="B110" s="42" t="s">
         <v>77</v>
       </c>
@@ -38608,7 +38707,7 @@
       <c r="T110" s="16"/>
     </row>
     <row r="111" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A111" s="82"/>
+      <c r="A111" s="81"/>
       <c r="B111" s="42">
         <v>1</v>
       </c>
@@ -38641,7 +38740,7 @@
       <c r="T111" s="16"/>
     </row>
     <row r="112" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A112" s="82"/>
+      <c r="A112" s="81"/>
       <c r="B112" s="42">
         <v>2</v>
       </c>
@@ -38674,7 +38773,7 @@
       <c r="T112" s="16"/>
     </row>
     <row r="113" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A113" s="82"/>
+      <c r="A113" s="81"/>
       <c r="B113" s="42">
         <v>4</v>
       </c>
@@ -38707,7 +38806,7 @@
       <c r="T113" s="16"/>
     </row>
     <row r="114" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A114" s="82"/>
+      <c r="A114" s="81"/>
       <c r="B114" s="42">
         <v>6</v>
       </c>
@@ -38740,7 +38839,7 @@
       <c r="T114" s="16"/>
     </row>
     <row r="115" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A115" s="82"/>
+      <c r="A115" s="81"/>
       <c r="B115" s="42">
         <v>8</v>
       </c>
@@ -38773,7 +38872,7 @@
       <c r="T115" s="16"/>
     </row>
     <row r="116" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A116" s="82"/>
+      <c r="A116" s="81"/>
       <c r="B116" s="42">
         <v>10</v>
       </c>
@@ -38806,7 +38905,7 @@
       <c r="T116" s="16"/>
     </row>
     <row r="117" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A117" s="82"/>
+      <c r="A117" s="81"/>
       <c r="B117" s="42">
         <v>12</v>
       </c>
@@ -38839,7 +38938,7 @@
       <c r="T117" s="31"/>
     </row>
     <row r="118" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A118" s="82"/>
+      <c r="A118" s="81"/>
       <c r="B118" s="42">
         <v>16</v>
       </c>
@@ -38872,41 +38971,41 @@
       <c r="T118" s="31"/>
     </row>
     <row r="119" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A119" s="82"/>
+      <c r="A119" s="81"/>
       <c r="B119" s="33" t="s">
         <v>86</v>
       </c>
-      <c r="C119" s="81" t="s">
+      <c r="C119" s="78" t="s">
         <v>113</v>
       </c>
-      <c r="D119" s="86"/>
-      <c r="E119" s="86"/>
-      <c r="F119" s="86"/>
-      <c r="G119" s="86"/>
-      <c r="H119" s="86"/>
-      <c r="I119" s="86"/>
-      <c r="J119" s="86"/>
-      <c r="K119" s="86"/>
-      <c r="L119" s="86"/>
-      <c r="M119" s="86"/>
-      <c r="N119" s="86"/>
-      <c r="O119" s="86"/>
-      <c r="P119" s="86"/>
-      <c r="Q119" s="86"/>
-      <c r="R119" s="86"/>
-      <c r="S119" s="86"/>
-      <c r="T119" s="87"/>
+      <c r="D119" s="79"/>
+      <c r="E119" s="79"/>
+      <c r="F119" s="79"/>
+      <c r="G119" s="79"/>
+      <c r="H119" s="79"/>
+      <c r="I119" s="79"/>
+      <c r="J119" s="79"/>
+      <c r="K119" s="79"/>
+      <c r="L119" s="79"/>
+      <c r="M119" s="79"/>
+      <c r="N119" s="79"/>
+      <c r="O119" s="79"/>
+      <c r="P119" s="79"/>
+      <c r="Q119" s="79"/>
+      <c r="R119" s="79"/>
+      <c r="S119" s="79"/>
+      <c r="T119" s="80"/>
     </row>
     <row r="120" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A120" s="88" t="s">
-        <v>116</v>
-      </c>
-      <c r="B120" s="77" t="s">
+      <c r="A120" s="76" t="s">
+        <v>115</v>
+      </c>
+      <c r="B120" s="73" t="s">
         <v>78</v>
       </c>
-      <c r="C120" s="78"/>
-      <c r="D120" s="78"/>
-      <c r="E120" s="79"/>
+      <c r="C120" s="74"/>
+      <c r="D120" s="74"/>
+      <c r="E120" s="75"/>
       <c r="F120" s="31"/>
       <c r="G120" s="31"/>
       <c r="H120" s="31"/>
@@ -38933,7 +39032,7 @@
       <c r="AC120" s="31"/>
     </row>
     <row r="121" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A121" s="89"/>
+      <c r="A121" s="77"/>
       <c r="B121" s="42" t="s">
         <v>77</v>
       </c>
@@ -38972,18 +39071,18 @@
       <c r="AC121" s="31"/>
     </row>
     <row r="122" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A122" s="89"/>
+      <c r="A122" s="77"/>
       <c r="B122" s="15">
         <v>1</v>
       </c>
       <c r="C122" s="24">
-        <v>9725</v>
+        <v>5381</v>
       </c>
       <c r="D122" s="24">
-        <v>76160</v>
+        <v>41829</v>
       </c>
       <c r="E122" s="24">
-        <v>257265</v>
+        <v>142216</v>
       </c>
       <c r="F122" s="31"/>
       <c r="G122" s="31"/>
@@ -39011,18 +39110,18 @@
       <c r="AC122" s="31"/>
     </row>
     <row r="123" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A123" s="89"/>
+      <c r="A123" s="77"/>
       <c r="B123" s="15">
         <v>2</v>
       </c>
       <c r="C123" s="24">
-        <v>5498</v>
+        <v>2737</v>
       </c>
       <c r="D123" s="24">
-        <v>39071</v>
+        <v>21202</v>
       </c>
       <c r="E123" s="24">
-        <v>130577</v>
+        <v>70771</v>
       </c>
       <c r="F123" s="31"/>
       <c r="G123" s="31"/>
@@ -39050,18 +39149,18 @@
       <c r="AC123" s="31"/>
     </row>
     <row r="124" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A124" s="89"/>
+      <c r="A124" s="77"/>
       <c r="B124" s="15">
         <v>4</v>
       </c>
       <c r="C124" s="24">
-        <v>3076</v>
+        <v>1427</v>
       </c>
       <c r="D124" s="24">
-        <v>20102</v>
+        <v>11078</v>
       </c>
       <c r="E124" s="24">
-        <v>66384</v>
+        <v>36194</v>
       </c>
       <c r="F124" s="31"/>
       <c r="G124" s="31"/>
@@ -39089,18 +39188,18 @@
       <c r="AC124" s="31"/>
     </row>
     <row r="125" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A125" s="89"/>
+      <c r="A125" s="77"/>
       <c r="B125" s="15">
         <v>6</v>
       </c>
       <c r="C125" s="24">
-        <v>2342</v>
+        <v>1042</v>
       </c>
       <c r="D125" s="24">
-        <v>14063</v>
+        <v>7787</v>
       </c>
       <c r="E125" s="24">
-        <v>46005</v>
+        <v>25435</v>
       </c>
       <c r="F125" s="31"/>
       <c r="G125" s="31"/>
@@ -39128,18 +39227,18 @@
       <c r="AC125" s="31"/>
     </row>
     <row r="126" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A126" s="89"/>
+      <c r="A126" s="77"/>
       <c r="B126" s="15">
         <v>8</v>
       </c>
       <c r="C126" s="40">
-        <v>1880</v>
+        <v>818</v>
       </c>
       <c r="D126" s="24">
-        <v>11690</v>
+        <v>6260</v>
       </c>
       <c r="E126" s="24">
-        <v>35587</v>
+        <v>19632</v>
       </c>
       <c r="F126" s="31"/>
       <c r="G126" s="31"/>
@@ -39167,18 +39266,18 @@
       <c r="AC126" s="31"/>
     </row>
     <row r="127" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A127" s="89"/>
+      <c r="A127" s="77"/>
       <c r="B127" s="15">
         <v>10</v>
       </c>
       <c r="C127" s="40">
-        <v>1650</v>
+        <v>682</v>
       </c>
       <c r="D127" s="24">
-        <v>10161</v>
+        <v>5372</v>
       </c>
       <c r="E127" s="24">
-        <v>29914</v>
+        <v>16476</v>
       </c>
       <c r="F127" s="31"/>
       <c r="G127" s="31"/>
@@ -39206,18 +39305,18 @@
       <c r="AC127" s="31"/>
     </row>
     <row r="128" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A128" s="89"/>
+      <c r="A128" s="77"/>
       <c r="B128" s="15">
         <v>12</v>
       </c>
       <c r="C128" s="40">
-        <v>1435</v>
+        <v>592</v>
       </c>
       <c r="D128" s="24">
-        <v>8034</v>
+        <v>4574</v>
       </c>
       <c r="E128" s="24">
-        <v>25229</v>
+        <v>14220</v>
       </c>
       <c r="F128" s="31"/>
       <c r="G128" s="31"/>
@@ -39245,18 +39344,18 @@
       <c r="AC128" s="31"/>
     </row>
     <row r="129" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A129" s="89"/>
+      <c r="A129" s="77"/>
       <c r="B129" s="15">
         <v>14</v>
       </c>
       <c r="C129" s="40">
-        <v>1318</v>
+        <v>550</v>
       </c>
       <c r="D129" s="24">
-        <v>7301</v>
+        <v>4295</v>
       </c>
       <c r="E129" s="24">
-        <v>23660</v>
+        <v>13252</v>
       </c>
       <c r="F129" s="31"/>
       <c r="G129" s="31"/>
@@ -39284,18 +39383,18 @@
       <c r="AC129" s="31"/>
     </row>
     <row r="130" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A130" s="89"/>
+      <c r="A130" s="77"/>
       <c r="B130" s="15">
         <v>16</v>
       </c>
       <c r="C130" s="40">
-        <v>1223</v>
+        <v>527</v>
       </c>
       <c r="D130" s="24">
-        <v>6821</v>
+        <v>3969</v>
       </c>
       <c r="E130" s="24">
-        <v>21062</v>
+        <v>12007</v>
       </c>
       <c r="F130" s="31"/>
       <c r="G130" s="31"/>
@@ -39323,18 +39422,18 @@
       <c r="AC130" s="31"/>
     </row>
     <row r="131" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A131" s="89"/>
+      <c r="A131" s="77"/>
       <c r="B131" s="15">
         <v>18</v>
       </c>
       <c r="C131" s="40">
-        <v>1176</v>
+        <v>497</v>
       </c>
       <c r="D131" s="24">
-        <v>6201</v>
+        <v>3709</v>
       </c>
       <c r="E131" s="24">
-        <v>20637</v>
+        <v>11351</v>
       </c>
       <c r="F131" s="31"/>
       <c r="G131" s="31"/>
@@ -39362,18 +39461,18 @@
       <c r="AC131" s="31"/>
     </row>
     <row r="132" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A132" s="89"/>
+      <c r="A132" s="77"/>
       <c r="B132" s="15">
         <v>20</v>
       </c>
       <c r="C132" s="40">
-        <v>1067</v>
+        <v>479</v>
       </c>
       <c r="D132" s="24">
-        <v>6056</v>
+        <v>3554</v>
       </c>
       <c r="E132" s="24">
-        <v>18311</v>
+        <v>10884</v>
       </c>
       <c r="F132" s="31"/>
       <c r="G132" s="31"/>
@@ -39401,18 +39500,18 @@
       <c r="AC132" s="31"/>
     </row>
     <row r="133" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A133" s="89"/>
+      <c r="A133" s="77"/>
       <c r="B133" s="49">
         <v>40</v>
       </c>
       <c r="C133" s="50">
-        <v>1201</v>
+        <v>518</v>
       </c>
       <c r="D133" s="51">
-        <v>6846</v>
+        <v>3697</v>
       </c>
       <c r="E133" s="51">
-        <v>20629</v>
+        <v>11163</v>
       </c>
       <c r="F133" s="31"/>
       <c r="G133" s="31"/>
@@ -39440,13 +39539,13 @@
       <c r="AC133" s="31"/>
     </row>
     <row r="134" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A134" s="89"/>
-      <c r="B134" s="77" t="s">
+      <c r="A134" s="77"/>
+      <c r="B134" s="73" t="s">
         <v>96</v>
       </c>
-      <c r="C134" s="78"/>
-      <c r="D134" s="78"/>
-      <c r="E134" s="79"/>
+      <c r="C134" s="74"/>
+      <c r="D134" s="74"/>
+      <c r="E134" s="75"/>
       <c r="F134" s="31"/>
       <c r="G134" s="31"/>
       <c r="H134" s="31"/>
@@ -39473,7 +39572,7 @@
       <c r="AC134" s="31"/>
     </row>
     <row r="135" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A135" s="89"/>
+      <c r="A135" s="77"/>
       <c r="B135" s="42" t="s">
         <v>77</v>
       </c>
@@ -39512,7 +39611,7 @@
       <c r="AC135" s="16"/>
     </row>
     <row r="136" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A136" s="89"/>
+      <c r="A136" s="77"/>
       <c r="B136" s="15">
         <v>1</v>
       </c>
@@ -39554,21 +39653,21 @@
       <c r="AC136" s="16"/>
     </row>
     <row r="137" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A137" s="89"/>
+      <c r="A137" s="77"/>
       <c r="B137" s="15">
         <v>2</v>
       </c>
       <c r="C137" s="40">
         <f>ROUND(C122/C123,5)</f>
-        <v>1.7688299999999999</v>
+        <v>1.9660200000000001</v>
       </c>
       <c r="D137" s="40">
         <f>ROUND(D122/D123,5)</f>
-        <v>1.9492700000000001</v>
+        <v>1.97288</v>
       </c>
       <c r="E137" s="40">
         <f>ROUND(E122/E123,5)</f>
-        <v>1.9702200000000001</v>
+        <v>2.0095200000000002</v>
       </c>
       <c r="F137" s="16"/>
       <c r="G137" s="16"/>
@@ -39596,21 +39695,21 @@
       <c r="AC137" s="16"/>
     </row>
     <row r="138" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A138" s="89"/>
+      <c r="A138" s="77"/>
       <c r="B138" s="15">
         <v>4</v>
       </c>
       <c r="C138" s="40">
         <f>ROUND(C122/C124,5)</f>
-        <v>3.1615700000000002</v>
+        <v>3.7708499999999998</v>
       </c>
       <c r="D138" s="40">
         <f>ROUND(D122/D124,5)</f>
-        <v>3.7886799999999998</v>
+        <v>3.7758600000000002</v>
       </c>
       <c r="E138" s="40">
         <f>ROUND(E122/E124,5)</f>
-        <v>3.87541</v>
+        <v>3.9292699999999998</v>
       </c>
       <c r="F138" s="16"/>
       <c r="G138" s="16"/>
@@ -39638,21 +39737,21 @@
       <c r="AC138" s="16"/>
     </row>
     <row r="139" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A139" s="89"/>
+      <c r="A139" s="77"/>
       <c r="B139" s="15">
         <v>6</v>
       </c>
       <c r="C139" s="40">
         <f>ROUND(C122/C125,5)</f>
-        <v>4.1524299999999998</v>
+        <v>5.16411</v>
       </c>
       <c r="D139" s="40">
         <f>ROUND(D122/D125,5)</f>
-        <v>5.4156300000000002</v>
+        <v>5.3716499999999998</v>
       </c>
       <c r="E139" s="40">
         <f>ROUND(E122/E125,5)</f>
-        <v>5.5921099999999999</v>
+        <v>5.5913500000000003</v>
       </c>
       <c r="F139" s="16"/>
       <c r="G139" s="16"/>
@@ -39680,21 +39779,21 @@
       <c r="AC139" s="16"/>
     </row>
     <row r="140" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A140" s="89"/>
+      <c r="A140" s="77"/>
       <c r="B140" s="15">
         <v>8</v>
       </c>
       <c r="C140" s="40">
         <f>ROUND(C122/C126,5)</f>
-        <v>5.1728699999999996</v>
+        <v>6.5782400000000001</v>
       </c>
       <c r="D140" s="40">
         <f>ROUND(D122/D126,5)</f>
-        <v>6.5149699999999999</v>
+        <v>6.6819499999999996</v>
       </c>
       <c r="E140" s="40">
         <f>ROUND(E122/E126,5)</f>
-        <v>7.2291800000000004</v>
+        <v>7.2440899999999999</v>
       </c>
       <c r="F140" s="16"/>
       <c r="G140" s="16"/>
@@ -39722,21 +39821,21 @@
       <c r="AC140" s="16"/>
     </row>
     <row r="141" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A141" s="89"/>
+      <c r="A141" s="77"/>
       <c r="B141" s="15">
         <v>10</v>
       </c>
       <c r="C141" s="40">
         <f>ROUND(C122/C127,5)</f>
-        <v>5.8939399999999997</v>
+        <v>7.8900300000000003</v>
       </c>
       <c r="D141" s="40">
         <f>ROUND(D122/D127,5)</f>
-        <v>7.49533</v>
+        <v>7.7864899999999997</v>
       </c>
       <c r="E141" s="40">
         <f>ROUND(E122/E127,5)</f>
-        <v>8.6001499999999993</v>
+        <v>8.63171</v>
       </c>
       <c r="F141" s="16"/>
       <c r="G141" s="16"/>
@@ -39764,21 +39863,21 @@
       <c r="AC141" s="16"/>
     </row>
     <row r="142" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A142" s="89"/>
+      <c r="A142" s="77"/>
       <c r="B142" s="15">
         <v>12</v>
       </c>
       <c r="C142" s="40">
         <f>ROUND(C122/C128,5)</f>
-        <v>6.7770000000000001</v>
+        <v>9.0895299999999999</v>
       </c>
       <c r="D142" s="40">
         <f>ROUND(D122/D128,5)</f>
-        <v>9.4797100000000007</v>
+        <v>9.1449499999999997</v>
       </c>
       <c r="E142" s="40">
         <f>ROUND(E122/E128,5)</f>
-        <v>10.197190000000001</v>
+        <v>10.00113</v>
       </c>
       <c r="F142" s="16"/>
       <c r="G142" s="16"/>
@@ -39806,21 +39905,21 @@
       <c r="AC142" s="16"/>
     </row>
     <row r="143" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A143" s="89"/>
+      <c r="A143" s="77"/>
       <c r="B143" s="15">
         <v>14</v>
       </c>
       <c r="C143" s="40">
-        <f t="shared" ref="C143:E147" si="7">ROUND(C$122/C129,5)</f>
-        <v>7.3785999999999996</v>
+        <f>ROUND(C$122/C129,5)</f>
+        <v>9.7836400000000001</v>
       </c>
       <c r="D143" s="40">
-        <f t="shared" si="7"/>
-        <v>10.43145</v>
+        <f t="shared" ref="C143:E147" si="7">ROUND(D$122/D129,5)</f>
+        <v>9.7390000000000008</v>
       </c>
       <c r="E143" s="40">
         <f t="shared" si="7"/>
-        <v>10.873419999999999</v>
+        <v>10.73166</v>
       </c>
       <c r="F143" s="16"/>
       <c r="G143" s="16"/>
@@ -39848,21 +39947,21 @@
       <c r="AC143" s="16"/>
     </row>
     <row r="144" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A144" s="89"/>
+      <c r="A144" s="77"/>
       <c r="B144" s="15">
         <v>16</v>
       </c>
       <c r="C144" s="40">
         <f t="shared" si="7"/>
-        <v>7.9517600000000002</v>
+        <v>10.21063</v>
       </c>
       <c r="D144" s="40">
         <f t="shared" si="7"/>
-        <v>11.165520000000001</v>
+        <v>10.538930000000001</v>
       </c>
       <c r="E144" s="40">
         <f t="shared" si="7"/>
-        <v>12.214650000000001</v>
+        <v>11.84442</v>
       </c>
       <c r="F144" s="31"/>
       <c r="G144" s="31"/>
@@ -39890,21 +39989,21 @@
       <c r="AC144" s="31"/>
     </row>
     <row r="145" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A145" s="89"/>
+      <c r="A145" s="77"/>
       <c r="B145" s="15">
         <v>18</v>
       </c>
       <c r="C145" s="40">
         <f t="shared" si="7"/>
-        <v>8.2695600000000002</v>
+        <v>10.82696</v>
       </c>
       <c r="D145" s="40">
         <f t="shared" si="7"/>
-        <v>12.281890000000001</v>
+        <v>11.277699999999999</v>
       </c>
       <c r="E145" s="40">
         <f t="shared" si="7"/>
-        <v>12.466200000000001</v>
+        <v>12.52894</v>
       </c>
       <c r="F145" s="16"/>
       <c r="G145" s="16"/>
@@ -39932,21 +40031,21 @@
       <c r="AC145" s="16"/>
     </row>
     <row r="146" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A146" s="89"/>
+      <c r="A146" s="77"/>
       <c r="B146" s="15">
         <v>20</v>
       </c>
       <c r="C146" s="40">
         <f t="shared" si="7"/>
-        <v>9.1143400000000003</v>
+        <v>11.23382</v>
       </c>
       <c r="D146" s="40">
         <f t="shared" si="7"/>
-        <v>12.57596</v>
+        <v>11.76956</v>
       </c>
       <c r="E146" s="40">
         <f t="shared" si="7"/>
-        <v>14.04975</v>
+        <v>13.066520000000001</v>
       </c>
       <c r="F146" s="16"/>
       <c r="G146" s="16"/>
@@ -39974,21 +40073,21 @@
       <c r="AC146" s="16"/>
     </row>
     <row r="147" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A147" s="89"/>
+      <c r="A147" s="77"/>
       <c r="B147" s="49">
         <v>40</v>
       </c>
       <c r="C147" s="50">
         <f t="shared" si="7"/>
-        <v>8.0974199999999996</v>
+        <v>10.388030000000001</v>
       </c>
       <c r="D147" s="50">
         <f t="shared" si="7"/>
-        <v>11.124739999999999</v>
+        <v>11.314310000000001</v>
       </c>
       <c r="E147" s="50">
         <f t="shared" si="7"/>
-        <v>12.47104</v>
+        <v>12.739940000000001</v>
       </c>
       <c r="F147" s="16"/>
       <c r="G147" s="16"/>
@@ -40016,13 +40115,13 @@
       <c r="AC147" s="16"/>
     </row>
     <row r="148" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A148" s="89"/>
-      <c r="B148" s="77" t="s">
+      <c r="A148" s="77"/>
+      <c r="B148" s="73" t="s">
         <v>97</v>
       </c>
-      <c r="C148" s="78"/>
-      <c r="D148" s="78"/>
-      <c r="E148" s="79"/>
+      <c r="C148" s="74"/>
+      <c r="D148" s="74"/>
+      <c r="E148" s="75"/>
       <c r="F148" s="16"/>
       <c r="G148" s="16"/>
       <c r="H148" s="16"/>
@@ -40049,7 +40148,7 @@
       <c r="AC148" s="16"/>
     </row>
     <row r="149" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A149" s="89"/>
+      <c r="A149" s="77"/>
       <c r="B149" s="42" t="s">
         <v>77</v>
       </c>
@@ -40088,16 +40187,16 @@
       <c r="AC149" s="16"/>
     </row>
     <row r="150" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A150" s="89"/>
+      <c r="A150" s="77"/>
       <c r="B150" s="15">
         <v>1</v>
       </c>
       <c r="C150" s="40">
-        <f t="shared" ref="C150:C161" si="8">ROUND(C136/$B136,5)</f>
+        <f t="shared" ref="C150:E161" si="8">ROUND(C136/$B136,5)</f>
         <v>1</v>
       </c>
       <c r="D150" s="40">
-        <f t="shared" ref="D150:E154" si="9">D136/$B136</f>
+        <f t="shared" ref="D150:E150" si="9">D136/$B136</f>
         <v>1</v>
       </c>
       <c r="E150" s="40">
@@ -40130,21 +40229,21 @@
       <c r="AC150" s="16"/>
     </row>
     <row r="151" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A151" s="89"/>
+      <c r="A151" s="77"/>
       <c r="B151" s="15">
         <v>2</v>
       </c>
       <c r="C151" s="40">
         <f t="shared" si="8"/>
-        <v>0.88441999999999998</v>
+        <v>0.98301000000000005</v>
       </c>
       <c r="D151" s="40">
-        <f t="shared" si="9"/>
-        <v>0.97463500000000003</v>
+        <f t="shared" si="8"/>
+        <v>0.98643999999999998</v>
       </c>
       <c r="E151" s="40">
-        <f t="shared" si="9"/>
-        <v>0.98511000000000004</v>
+        <f t="shared" si="8"/>
+        <v>1.0047600000000001</v>
       </c>
       <c r="F151" s="16"/>
       <c r="G151" s="16"/>
@@ -40172,21 +40271,21 @@
       <c r="AC151" s="16"/>
     </row>
     <row r="152" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A152" s="89"/>
+      <c r="A152" s="77"/>
       <c r="B152" s="15">
         <v>4</v>
       </c>
       <c r="C152" s="40">
         <f t="shared" si="8"/>
-        <v>0.79039000000000004</v>
+        <v>0.94271000000000005</v>
       </c>
       <c r="D152" s="40">
-        <f t="shared" si="9"/>
-        <v>0.94716999999999996</v>
+        <f>ROUND(D138/$B138,5)</f>
+        <v>0.94396999999999998</v>
       </c>
       <c r="E152" s="40">
-        <f t="shared" si="9"/>
-        <v>0.96885250000000001</v>
+        <f t="shared" si="8"/>
+        <v>0.98231999999999997</v>
       </c>
       <c r="F152" s="16"/>
       <c r="G152" s="16"/>
@@ -40214,21 +40313,21 @@
       <c r="AC152" s="16"/>
     </row>
     <row r="153" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A153" s="89"/>
+      <c r="A153" s="77"/>
       <c r="B153" s="15">
         <v>6</v>
       </c>
       <c r="C153" s="40">
         <f t="shared" si="8"/>
-        <v>0.69206999999999996</v>
+        <v>0.86068999999999996</v>
       </c>
       <c r="D153" s="40">
-        <f t="shared" si="9"/>
-        <v>0.90260499999999999</v>
+        <f t="shared" si="8"/>
+        <v>0.89527999999999996</v>
       </c>
       <c r="E153" s="40">
-        <f t="shared" si="9"/>
-        <v>0.93201833333333328</v>
+        <f t="shared" si="8"/>
+        <v>0.93189</v>
       </c>
       <c r="F153" s="16"/>
       <c r="G153" s="16"/>
@@ -40256,21 +40355,21 @@
       <c r="AC153" s="16"/>
     </row>
     <row r="154" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A154" s="89"/>
+      <c r="A154" s="77"/>
       <c r="B154" s="15">
         <v>8</v>
       </c>
       <c r="C154" s="40">
         <f t="shared" si="8"/>
-        <v>0.64661000000000002</v>
+        <v>0.82228000000000001</v>
       </c>
       <c r="D154" s="40">
-        <f t="shared" si="9"/>
-        <v>0.81437124999999999</v>
+        <f t="shared" si="8"/>
+        <v>0.83523999999999998</v>
       </c>
       <c r="E154" s="40">
-        <f t="shared" si="9"/>
-        <v>0.90364750000000005</v>
+        <f t="shared" si="8"/>
+        <v>0.90551000000000004</v>
       </c>
       <c r="F154" s="16"/>
       <c r="G154" s="16"/>
@@ -40298,21 +40397,21 @@
       <c r="AC154" s="16"/>
     </row>
     <row r="155" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A155" s="89"/>
+      <c r="A155" s="77"/>
       <c r="B155" s="15">
         <v>10</v>
       </c>
       <c r="C155" s="40">
         <f t="shared" si="8"/>
-        <v>0.58938999999999997</v>
+        <v>0.78900000000000003</v>
       </c>
       <c r="D155" s="40">
-        <f t="shared" ref="D155:E161" si="10">D141/$B141</f>
-        <v>0.749533</v>
+        <f t="shared" si="8"/>
+        <v>0.77864999999999995</v>
       </c>
       <c r="E155" s="40">
-        <f t="shared" si="10"/>
-        <v>0.86001499999999997</v>
+        <f t="shared" si="8"/>
+        <v>0.86316999999999999</v>
       </c>
       <c r="F155" s="16"/>
       <c r="G155" s="16"/>
@@ -40340,21 +40439,21 @@
       <c r="AC155" s="16"/>
     </row>
     <row r="156" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A156" s="89"/>
+      <c r="A156" s="77"/>
       <c r="B156" s="15">
         <v>12</v>
       </c>
       <c r="C156" s="40">
         <f t="shared" si="8"/>
-        <v>0.56474999999999997</v>
+        <v>0.75746000000000002</v>
       </c>
       <c r="D156" s="40">
-        <f t="shared" si="10"/>
-        <v>0.78997583333333343</v>
+        <f t="shared" si="8"/>
+        <v>0.76207999999999998</v>
       </c>
       <c r="E156" s="40">
-        <f t="shared" si="10"/>
-        <v>0.84976583333333344</v>
+        <f t="shared" si="8"/>
+        <v>0.83343</v>
       </c>
       <c r="F156" s="31"/>
       <c r="G156" s="31"/>
@@ -40382,21 +40481,21 @@
       <c r="AC156" s="31"/>
     </row>
     <row r="157" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A157" s="89"/>
+      <c r="A157" s="77"/>
       <c r="B157" s="15">
         <v>14</v>
       </c>
       <c r="C157" s="40">
         <f t="shared" si="8"/>
-        <v>0.52703999999999995</v>
+        <v>0.69882999999999995</v>
       </c>
       <c r="D157" s="40">
-        <f t="shared" si="10"/>
-        <v>0.74510357142857142</v>
+        <f t="shared" si="8"/>
+        <v>0.69564000000000004</v>
       </c>
       <c r="E157" s="40">
-        <f t="shared" si="10"/>
-        <v>0.77667285714285705</v>
+        <f t="shared" si="8"/>
+        <v>0.76654999999999995</v>
       </c>
       <c r="F157" s="31"/>
       <c r="G157" s="31"/>
@@ -40424,21 +40523,21 @@
       <c r="AC157" s="31"/>
     </row>
     <row r="158" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A158" s="89"/>
+      <c r="A158" s="77"/>
       <c r="B158" s="15">
         <v>16</v>
       </c>
       <c r="C158" s="40">
         <f t="shared" si="8"/>
-        <v>0.49698999999999999</v>
+        <v>0.63815999999999995</v>
       </c>
       <c r="D158" s="40">
-        <f t="shared" si="10"/>
-        <v>0.69784500000000005</v>
+        <f t="shared" si="8"/>
+        <v>0.65868000000000004</v>
       </c>
       <c r="E158" s="40">
-        <f t="shared" si="10"/>
-        <v>0.76341562500000004</v>
+        <f t="shared" si="8"/>
+        <v>0.74028000000000005</v>
       </c>
       <c r="F158" s="16"/>
       <c r="G158" s="16"/>
@@ -40466,21 +40565,21 @@
       <c r="AC158" s="16"/>
     </row>
     <row r="159" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A159" s="89"/>
+      <c r="A159" s="77"/>
       <c r="B159" s="15">
         <v>18</v>
       </c>
       <c r="C159" s="40">
         <f t="shared" si="8"/>
-        <v>0.45942</v>
+        <v>0.60150000000000003</v>
       </c>
       <c r="D159" s="40">
-        <f t="shared" si="10"/>
-        <v>0.68232722222222231</v>
+        <f t="shared" si="8"/>
+        <v>0.62653999999999999</v>
       </c>
       <c r="E159" s="40">
-        <f t="shared" si="10"/>
-        <v>0.69256666666666666</v>
+        <f t="shared" si="8"/>
+        <v>0.69604999999999995</v>
       </c>
       <c r="F159" s="16"/>
       <c r="G159" s="16"/>
@@ -40508,21 +40607,21 @@
       <c r="AC159" s="16"/>
     </row>
     <row r="160" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A160" s="89"/>
+      <c r="A160" s="77"/>
       <c r="B160" s="15">
         <v>20</v>
       </c>
       <c r="C160" s="40">
         <f t="shared" si="8"/>
-        <v>0.45572000000000001</v>
+        <v>0.56169000000000002</v>
       </c>
       <c r="D160" s="40">
-        <f t="shared" si="10"/>
-        <v>0.62879799999999997</v>
+        <f t="shared" si="8"/>
+        <v>0.58848</v>
       </c>
       <c r="E160" s="40">
-        <f t="shared" si="10"/>
-        <v>0.70248749999999993</v>
+        <f t="shared" si="8"/>
+        <v>0.65332999999999997</v>
       </c>
       <c r="F160" s="16"/>
       <c r="G160" s="16"/>
@@ -40550,21 +40649,21 @@
       <c r="AC160" s="16"/>
     </row>
     <row r="161" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A161" s="89"/>
+      <c r="A161" s="77"/>
       <c r="B161" s="49">
         <v>40</v>
       </c>
       <c r="C161" s="50">
         <f t="shared" si="8"/>
-        <v>0.20244000000000001</v>
+        <v>0.25969999999999999</v>
       </c>
       <c r="D161" s="50">
-        <f t="shared" si="10"/>
-        <v>0.27811849999999999</v>
+        <f t="shared" si="8"/>
+        <v>0.28286</v>
       </c>
       <c r="E161" s="50">
-        <f t="shared" si="10"/>
-        <v>0.311776</v>
+        <f t="shared" si="8"/>
+        <v>0.31850000000000001</v>
       </c>
       <c r="F161" s="16"/>
       <c r="G161" s="16"/>
@@ -40592,73 +40691,153 @@
       <c r="AC161" s="16"/>
     </row>
     <row r="162" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A162" s="89"/>
+      <c r="A162" s="77"/>
       <c r="B162" s="33" t="s">
         <v>86</v>
       </c>
-      <c r="C162" s="81" t="s">
-        <v>115</v>
-      </c>
-      <c r="D162" s="86"/>
-      <c r="E162" s="86"/>
-      <c r="F162" s="86"/>
-      <c r="G162" s="86"/>
-      <c r="H162" s="86"/>
-      <c r="I162" s="86"/>
-      <c r="J162" s="86"/>
-      <c r="K162" s="86"/>
-      <c r="L162" s="86"/>
-      <c r="M162" s="86"/>
-      <c r="N162" s="86"/>
-      <c r="O162" s="86"/>
-      <c r="P162" s="86"/>
-      <c r="Q162" s="86"/>
-      <c r="R162" s="86"/>
-      <c r="S162" s="86"/>
-      <c r="T162" s="86"/>
-      <c r="U162" s="86"/>
-      <c r="V162" s="86"/>
-      <c r="W162" s="86"/>
-      <c r="X162" s="86"/>
-      <c r="Y162" s="86"/>
-      <c r="Z162" s="86"/>
-      <c r="AA162" s="86"/>
-      <c r="AB162" s="86"/>
-      <c r="AC162" s="87"/>
+      <c r="C162" s="78" t="s">
+        <v>124</v>
+      </c>
+      <c r="D162" s="79"/>
+      <c r="E162" s="79"/>
+      <c r="F162" s="79"/>
+      <c r="G162" s="79"/>
+      <c r="H162" s="79"/>
+      <c r="I162" s="79"/>
+      <c r="J162" s="79"/>
+      <c r="K162" s="79"/>
+      <c r="L162" s="79"/>
+      <c r="M162" s="79"/>
+      <c r="N162" s="79"/>
+      <c r="O162" s="79"/>
+      <c r="P162" s="79"/>
+      <c r="Q162" s="79"/>
+      <c r="R162" s="79"/>
+      <c r="S162" s="79"/>
+      <c r="T162" s="79"/>
+      <c r="U162" s="79"/>
+      <c r="V162" s="79"/>
+      <c r="W162" s="79"/>
+      <c r="X162" s="79"/>
+      <c r="Y162" s="79"/>
+      <c r="Z162" s="79"/>
+      <c r="AA162" s="79"/>
+      <c r="AB162" s="79"/>
+      <c r="AC162" s="80"/>
+    </row>
+    <row r="164" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="E164" s="54" t="s">
+        <v>118</v>
+      </c>
+      <c r="F164" s="54" t="s">
+        <v>121</v>
+      </c>
+      <c r="G164" s="54" t="s">
+        <v>122</v>
+      </c>
+      <c r="H164" s="55" t="s">
+        <v>123</v>
+      </c>
     </row>
     <row r="165" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B165" s="26" t="s">
-        <v>117</v>
-      </c>
+        <v>116</v>
+      </c>
+      <c r="E165" s="54" t="s">
+        <v>119</v>
+      </c>
+      <c r="F165" s="54">
+        <v>331549</v>
+      </c>
+      <c r="G165" s="72">
+        <f>ROUND(F165/F166,5)</f>
+        <v>13.740690000000001</v>
+      </c>
+      <c r="H165" s="72">
+        <f>ROUND(G165/20,5)</f>
+        <v>0.68703000000000003</v>
+      </c>
+    </row>
+    <row r="166" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="E166" s="52" t="s">
+        <v>120</v>
+      </c>
+      <c r="F166" s="54">
+        <v>24129</v>
+      </c>
+      <c r="G166" s="72"/>
+      <c r="H166" s="72"/>
     </row>
     <row r="167" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B167" s="26" t="s">
-        <v>118</v>
-      </c>
+        <v>117</v>
+      </c>
+    </row>
+    <row r="169" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B169" s="56"/>
+      <c r="C169" s="56"/>
+      <c r="D169" s="56"/>
+      <c r="E169" s="56"/>
+      <c r="F169" s="57"/>
+      <c r="G169" s="57"/>
+      <c r="H169" s="57"/>
+    </row>
+    <row r="170" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B170" s="56"/>
+      <c r="C170" s="56"/>
+      <c r="D170" s="56"/>
+      <c r="E170" s="56"/>
+      <c r="F170" s="57"/>
+      <c r="G170" s="57"/>
+      <c r="H170" s="57"/>
+    </row>
+    <row r="171" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B171" s="53"/>
+      <c r="C171" s="53"/>
+      <c r="D171" s="53"/>
+      <c r="E171" s="53"/>
+      <c r="F171" s="58"/>
+      <c r="G171" s="58"/>
+      <c r="H171" s="58"/>
+    </row>
+    <row r="172" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B172" s="53"/>
+      <c r="C172" s="53"/>
+      <c r="D172" s="53"/>
+      <c r="E172" s="53"/>
+      <c r="F172" s="53"/>
+      <c r="G172" s="53"/>
+      <c r="H172" s="53"/>
+    </row>
+    <row r="173" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B173" s="53"/>
+      <c r="C173" s="53"/>
+      <c r="D173" s="53"/>
+      <c r="E173" s="53"/>
+      <c r="F173" s="53"/>
+      <c r="G173" s="53"/>
+      <c r="H173" s="53"/>
+    </row>
+    <row r="174" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B174" s="53"/>
+      <c r="C174" s="53"/>
+      <c r="D174" s="53"/>
+      <c r="E174" s="53"/>
+      <c r="F174" s="53"/>
+      <c r="G174" s="53"/>
+      <c r="H174" s="53"/>
+    </row>
+    <row r="175" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B175" s="53"/>
+      <c r="C175" s="53"/>
+      <c r="D175" s="53"/>
+      <c r="E175" s="53"/>
+      <c r="F175" s="53"/>
+      <c r="G175" s="53"/>
+      <c r="H175" s="53"/>
     </row>
   </sheetData>
-  <mergeCells count="35">
-    <mergeCell ref="B148:E148"/>
-    <mergeCell ref="B134:E134"/>
-    <mergeCell ref="B120:E120"/>
-    <mergeCell ref="A120:A162"/>
-    <mergeCell ref="C162:AC162"/>
-    <mergeCell ref="A89:A119"/>
-    <mergeCell ref="C119:T119"/>
-    <mergeCell ref="B89:E89"/>
-    <mergeCell ref="B99:E99"/>
-    <mergeCell ref="B109:E109"/>
-    <mergeCell ref="A24:L24"/>
-    <mergeCell ref="M24:N24"/>
-    <mergeCell ref="M1:N1"/>
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="C12:N12"/>
-    <mergeCell ref="A2:A12"/>
-    <mergeCell ref="A13:A23"/>
-    <mergeCell ref="B22:B23"/>
-    <mergeCell ref="C22:N23"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="B2:D2"/>
+  <mergeCells count="37">
     <mergeCell ref="O88:T88"/>
     <mergeCell ref="A88:N88"/>
     <mergeCell ref="A57:A87"/>
@@ -40673,6 +40852,29 @@
     <mergeCell ref="B45:D45"/>
     <mergeCell ref="B35:D35"/>
     <mergeCell ref="B25:D25"/>
+    <mergeCell ref="A24:L24"/>
+    <mergeCell ref="M24:N24"/>
+    <mergeCell ref="M1:N1"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="C12:N12"/>
+    <mergeCell ref="A2:A12"/>
+    <mergeCell ref="A13:A23"/>
+    <mergeCell ref="B22:B23"/>
+    <mergeCell ref="C22:N23"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="A120:A162"/>
+    <mergeCell ref="C162:AC162"/>
+    <mergeCell ref="A89:A119"/>
+    <mergeCell ref="C119:T119"/>
+    <mergeCell ref="B89:E89"/>
+    <mergeCell ref="B99:E99"/>
+    <mergeCell ref="B109:E109"/>
+    <mergeCell ref="G165:G166"/>
+    <mergeCell ref="H165:H166"/>
+    <mergeCell ref="B148:E148"/>
+    <mergeCell ref="B134:E134"/>
+    <mergeCell ref="B120:E120"/>
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <hyperlinks>
@@ -40731,4 +40933,24 @@
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{971D527A-984B-4A9B-8624-22FA2B3C082C}">
+  <dimension ref="M10:M17"/>
+  <sheetFormatPr defaultRowHeight="22.1" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="16384" width="9.140625" style="41"/>
+  </cols>
+  <sheetData>
+    <row r="10" spans="13:13" x14ac:dyDescent="0.3">
+      <c r="M10" s="44"/>
+    </row>
+    <row r="17" spans="13:13" x14ac:dyDescent="0.3">
+      <c r="M17" s="44"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>